<commit_message>
Update MVP workbook with partial fundamentals
</commit_message>
<xml_diff>
--- a/stock_decision_mvp_calculated.xlsx
+++ b/stock_decision_mvp_calculated.xlsx
@@ -69,7 +69,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026/05/14 19:35:38</t>
+          <t>2026/05/14 20:07:26</t>
         </is>
       </c>
     </row>
@@ -247,7 +247,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026/05/14 19:35:38</t>
+          <t>2026/05/14 20:07:26</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -719,7 +719,7 @@
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>2026/05/14 19:35:38</t>
+          <t>2026/05/14 20:07:26</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
@@ -761,7 +761,7 @@
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>2026/05/14 19:35:38</t>
+          <t>2026/05/14 20:07:26</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
@@ -803,7 +803,7 @@
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>2026/05/14 19:35:38</t>
+          <t>2026/05/14 20:07:26</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
@@ -845,7 +845,7 @@
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>2026/05/14 19:35:38</t>
+          <t>2026/05/14 20:07:26</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
@@ -887,7 +887,7 @@
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>2026/05/14 19:35:38</t>
+          <t>2026/05/14 20:07:26</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
@@ -929,7 +929,7 @@
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>2026/05/14 19:35:38</t>
+          <t>2026/05/14 20:07:26</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
@@ -971,7 +971,7 @@
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>2026/05/14 19:35:38</t>
+          <t>2026/05/14 20:07:26</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
@@ -1013,7 +1013,7 @@
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>2026/05/14 19:35:38</t>
+          <t>2026/05/14 20:07:26</t>
         </is>
       </c>
       <c r="J9" t="inlineStr">
@@ -1113,7 +1113,7 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>2026/05/14 19:35:38</t>
+          <t>2026/05/14 20:07:26</t>
         </is>
       </c>
     </row>
@@ -1149,7 +1149,7 @@
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>2026/05/14 19:35:38</t>
+          <t>2026/05/14 20:07:26</t>
         </is>
       </c>
     </row>
@@ -1185,7 +1185,7 @@
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>2026/05/14 19:35:38</t>
+          <t>2026/05/14 20:07:26</t>
         </is>
       </c>
     </row>
@@ -1221,7 +1221,7 @@
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>2026/05/14 19:35:38</t>
+          <t>2026/05/14 20:07:26</t>
         </is>
       </c>
     </row>
@@ -1242,13 +1242,13 @@
         </is>
       </c>
       <c r="D6">
-        <v>157.87</v>
+        <v>157.94</v>
       </c>
       <c r="E6">
-        <v>0.87</v>
+        <v>0.91</v>
       </c>
       <c r="F6">
-        <v>-0.59</v>
+        <v>-0.55</v>
       </c>
       <c r="G6" t="inlineStr">
         <is>
@@ -1257,7 +1257,7 @@
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>2026/05/14 19:35:38</t>
+          <t>2026/05/14 20:07:26</t>
         </is>
       </c>
     </row>
@@ -1293,7 +1293,7 @@
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>2026/05/14 19:35:38</t>
+          <t>2026/05/14 20:07:26</t>
         </is>
       </c>
     </row>
@@ -1314,13 +1314,13 @@
         </is>
       </c>
       <c r="D8">
-        <v>17.8</v>
+        <v>17.87</v>
       </c>
       <c r="E8">
-        <v>4.22</v>
+        <v>4.63</v>
       </c>
       <c r="F8">
-        <v>-0.78</v>
+        <v>-0.39</v>
       </c>
       <c r="G8" t="inlineStr">
         <is>
@@ -1329,7 +1329,7 @@
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>2026/05/14 19:35:38</t>
+          <t>2026/05/14 20:07:26</t>
         </is>
       </c>
     </row>
@@ -1350,13 +1350,13 @@
         </is>
       </c>
       <c r="D9">
-        <v>98.51</v>
+        <v>98.52</v>
       </c>
       <c r="E9">
-        <v>0.27</v>
+        <v>0.28</v>
       </c>
       <c r="F9">
-        <v>0.3</v>
+        <v>0.31</v>
       </c>
       <c r="G9" t="inlineStr">
         <is>
@@ -1365,7 +1365,7 @@
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>2026/05/14 19:35:38</t>
+          <t>2026/05/14 20:07:26</t>
         </is>
       </c>
     </row>
@@ -1449,7 +1449,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026/05/14 19:35:38</t>
+          <t>2026/05/14 20:07:26</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -1462,10 +1462,8 @@
           <t/>
         </is>
       </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t/>
-        </is>
+      <c r="D2">
+        <v>11.38</v>
       </c>
       <c r="E2" t="inlineStr">
         <is>
@@ -1494,19 +1492,19 @@
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>四季報/IR等で別途確認</t>
+          <t>Yahoo!ファイナンス日本版 https://finance.yahoo.co.jp/quote/8035.T</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>未入力</t>
+          <t>一部取得</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026/05/14 19:35:38</t>
+          <t>2026/05/14 20:07:26</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -1514,15 +1512,11 @@
           <t>6857.T</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t/>
-        </is>
+      <c r="C3">
+        <v>44.6</v>
+      </c>
+      <c r="D3">
+        <v>26.07</v>
       </c>
       <c r="E3" t="inlineStr">
         <is>
@@ -1551,19 +1545,19 @@
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>四季報/IR等で別途確認</t>
+          <t>Yahoo!ファイナンス日本版 https://finance.yahoo.co.jp/quote/6857.T</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>未入力</t>
+          <t>一部取得</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2026/05/14 19:35:38</t>
+          <t>2026/05/14 20:07:26</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -1576,10 +1570,8 @@
           <t/>
         </is>
       </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t/>
-        </is>
+      <c r="D4">
+        <v>6.98</v>
       </c>
       <c r="E4" t="inlineStr">
         <is>
@@ -1608,19 +1600,19 @@
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>四季報/IR等で別途確認</t>
+          <t>Yahoo!ファイナンス日本版 https://finance.yahoo.co.jp/quote/4519.T</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>未入力</t>
+          <t>一部取得</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026/05/14 19:35:38</t>
+          <t>2026/05/14 20:07:26</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -1633,10 +1625,8 @@
           <t/>
         </is>
       </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t/>
-        </is>
+      <c r="D5">
+        <v>1.53</v>
       </c>
       <c r="E5" t="inlineStr">
         <is>
@@ -1665,19 +1655,19 @@
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>四季報/IR等で別途確認</t>
+          <t>Yahoo!ファイナンス日本版 https://finance.yahoo.co.jp/quote/8306.T</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>未入力</t>
+          <t>一部取得</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2026/05/14 19:35:38</t>
+          <t>2026/05/14 20:07:26</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -1685,15 +1675,11 @@
           <t>8058.T</t>
         </is>
       </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t/>
-        </is>
+      <c r="C6">
+        <v>19.58</v>
+      </c>
+      <c r="D6">
+        <v>2.28</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
@@ -1722,19 +1708,19 @@
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>四季報/IR等で別途確認</t>
+          <t>Yahoo!ファイナンス日本版 https://finance.yahoo.co.jp/quote/8058.T</t>
         </is>
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>未入力</t>
+          <t>一部取得</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026/05/14 19:35:38</t>
+          <t>2026/05/14 20:07:26</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -1742,15 +1728,11 @@
           <t>7974.T</t>
         </is>
       </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="D7" t="inlineStr">
-        <is>
-          <t/>
-        </is>
+      <c r="C7">
+        <v>25.53</v>
+      </c>
+      <c r="D7">
+        <v>2.68</v>
       </c>
       <c r="E7" t="inlineStr">
         <is>
@@ -1779,19 +1761,19 @@
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>四季報/IR等で別途確認</t>
+          <t>Yahoo!ファイナンス日本版 https://finance.yahoo.co.jp/quote/7974.T</t>
         </is>
       </c>
       <c r="K7" t="inlineStr">
         <is>
-          <t>未入力</t>
+          <t>一部取得</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>2026/05/14 19:35:38</t>
+          <t>2026/05/14 20:07:26</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -1804,10 +1786,8 @@
           <t/>
         </is>
       </c>
-      <c r="D8" t="inlineStr">
-        <is>
-          <t/>
-        </is>
+      <c r="D8">
+        <v>1.98</v>
       </c>
       <c r="E8" t="inlineStr">
         <is>
@@ -1836,19 +1816,19 @@
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>四季報/IR等で別途確認</t>
+          <t>Yahoo!ファイナンス日本版 https://finance.yahoo.co.jp/quote/9433.T</t>
         </is>
       </c>
       <c r="K8" t="inlineStr">
         <is>
-          <t>未入力</t>
+          <t>一部取得</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2026/05/14 19:35:38</t>
+          <t>2026/05/14 20:07:26</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -1856,15 +1836,11 @@
           <t>2802.T</t>
         </is>
       </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="D9" t="inlineStr">
-        <is>
-          <t/>
-        </is>
+      <c r="C9">
+        <v>44.27</v>
+      </c>
+      <c r="D9">
+        <v>6.89</v>
       </c>
       <c r="E9" t="inlineStr">
         <is>
@@ -1893,12 +1869,12 @@
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>四季報/IR等で別途確認</t>
+          <t>Yahoo!ファイナンス日本版 https://finance.yahoo.co.jp/quote/2802.T</t>
         </is>
       </c>
       <c r="K9" t="inlineStr">
         <is>
-          <t>未入力</t>
+          <t>一部取得</t>
         </is>
       </c>
     </row>
@@ -2705,7 +2681,7 @@
       </c>
       <c r="J1" t="inlineStr">
         <is>
-          <t>partial_score_max70</t>
+          <t>total_score_max100</t>
         </is>
       </c>
       <c r="K1" t="inlineStr">
@@ -2727,7 +2703,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026/05/14 19:35:38</t>
+          <t>2026/05/14 20:07:26</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -2744,24 +2720,20 @@
       <c r="E2">
         <v>3</v>
       </c>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t/>
-        </is>
+      <c r="F2">
+        <v>1</v>
       </c>
       <c r="G2">
         <v>15</v>
       </c>
-      <c r="H2" t="inlineStr">
-        <is>
-          <t/>
-        </is>
+      <c r="H2">
+        <v>3</v>
       </c>
       <c r="I2">
         <v>10</v>
       </c>
       <c r="J2">
-        <v>56</v>
+        <v>60</v>
       </c>
       <c r="K2" t="inlineStr">
         <is>
@@ -2770,19 +2742,19 @@
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>終値51200 / 20日騰落16.26% / 出来高倍率0.61 / 財務・PER未入力</t>
+          <t>終値51200 / 20日騰落16.26% / 出来高倍率0.61 / PER未取得 / PBR11.38 / EPS未取得</t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>価格・市場のみ計算</t>
+          <t>価格・市場・一部財務で計算</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026/05/14 19:35:38</t>
+          <t>2026/05/14 20:07:26</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -2799,24 +2771,20 @@
       <c r="E3">
         <v>6</v>
       </c>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t/>
-        </is>
+      <c r="F3">
+        <v>2</v>
       </c>
       <c r="G3">
         <v>15</v>
       </c>
-      <c r="H3" t="inlineStr">
-        <is>
-          <t/>
-        </is>
+      <c r="H3">
+        <v>12</v>
       </c>
       <c r="I3">
         <v>3</v>
       </c>
       <c r="J3">
-        <v>55</v>
+        <v>69</v>
       </c>
       <c r="K3" t="inlineStr">
         <is>
@@ -2825,19 +2793,19 @@
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>終値28615 / 20日騰落14.51% / 出来高倍率0.9 / 財務・PER未入力</t>
+          <t>終値28615 / 20日騰落14.51% / 出来高倍率0.9 / PER44.6 / PBR26.07 / EPS641.61</t>
         </is>
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>価格・市場のみ計算</t>
+          <t>価格・市場・一部財務で計算</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2026/05/14 19:35:38</t>
+          <t>2026/05/14 20:07:26</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -2854,24 +2822,20 @@
       <c r="E4">
         <v>3</v>
       </c>
-      <c r="F4" t="inlineStr">
-        <is>
-          <t/>
-        </is>
+      <c r="F4">
+        <v>1</v>
       </c>
       <c r="G4">
         <v>15</v>
       </c>
-      <c r="H4" t="inlineStr">
-        <is>
-          <t/>
-        </is>
+      <c r="H4">
+        <v>3</v>
       </c>
       <c r="I4">
         <v>0</v>
       </c>
       <c r="J4">
-        <v>29</v>
+        <v>33</v>
       </c>
       <c r="K4" t="inlineStr">
         <is>
@@ -2880,19 +2844,19 @@
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>終値8096 / 20日騰落-6.67% / 出来高倍率0.75 / 財務・PER未入力</t>
+          <t>終値8096 / 20日騰落-6.67% / 出来高倍率0.75 / PER未取得 / PBR6.98 / EPS未取得</t>
         </is>
       </c>
       <c r="M4" t="inlineStr">
         <is>
-          <t>価格・市場のみ計算</t>
+          <t>価格・市場・一部財務で計算</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026/05/14 19:35:38</t>
+          <t>2026/05/14 20:07:26</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -2909,45 +2873,41 @@
       <c r="E5">
         <v>6</v>
       </c>
-      <c r="F5" t="inlineStr">
-        <is>
-          <t/>
-        </is>
+      <c r="F5">
+        <v>5</v>
       </c>
       <c r="G5">
         <v>15</v>
       </c>
-      <c r="H5" t="inlineStr">
-        <is>
-          <t/>
-        </is>
+      <c r="H5">
+        <v>3</v>
       </c>
       <c r="I5">
         <v>10</v>
       </c>
       <c r="J5">
-        <v>60</v>
+        <v>68</v>
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>少額候補（財務未確認）</t>
+          <t>様子見</t>
         </is>
       </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t>終値2877 / 20日騰落1.23% / 出来高倍率0.96 / 財務・PER未入力</t>
+          <t>終値2877 / 20日騰落1.23% / 出来高倍率0.96 / PER未取得 / PBR1.53 / EPS未取得</t>
         </is>
       </c>
       <c r="M5" t="inlineStr">
         <is>
-          <t>価格・市場のみ計算</t>
+          <t>価格・市場・一部財務で計算</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2026/05/14 19:35:38</t>
+          <t>2026/05/14 20:07:26</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -2964,45 +2924,41 @@
       <c r="E6">
         <v>3</v>
       </c>
-      <c r="F6" t="inlineStr">
-        <is>
-          <t/>
-        </is>
+      <c r="F6">
+        <v>9</v>
       </c>
       <c r="G6">
         <v>15</v>
       </c>
-      <c r="H6" t="inlineStr">
-        <is>
-          <t/>
-        </is>
+      <c r="H6">
+        <v>12</v>
       </c>
       <c r="I6">
         <v>6</v>
       </c>
       <c r="J6">
-        <v>59</v>
+        <v>80</v>
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>様子見</t>
+          <t>買い候補（決算要確認）</t>
         </is>
       </c>
       <c r="L6" t="inlineStr">
         <is>
-          <t>終値5882 / 20日騰落10.83% / 出来高倍率0.71 / 財務・PER未入力</t>
+          <t>終値5882 / 20日騰落10.83% / 出来高倍率0.71 / PER19.58 / PBR2.28 / EPS300.42</t>
         </is>
       </c>
       <c r="M6" t="inlineStr">
         <is>
-          <t>価格・市場のみ計算</t>
+          <t>価格・市場・一部財務で計算</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026/05/14 19:35:38</t>
+          <t>2026/05/14 20:07:26</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -3019,24 +2975,20 @@
       <c r="E7">
         <v>8</v>
       </c>
-      <c r="F7" t="inlineStr">
-        <is>
-          <t/>
-        </is>
+      <c r="F7">
+        <v>6</v>
       </c>
       <c r="G7">
         <v>15</v>
       </c>
-      <c r="H7" t="inlineStr">
-        <is>
-          <t/>
-        </is>
+      <c r="H7">
+        <v>12</v>
       </c>
       <c r="I7">
         <v>3</v>
       </c>
       <c r="J7">
-        <v>26</v>
+        <v>44</v>
       </c>
       <c r="K7" t="inlineStr">
         <is>
@@ -3045,19 +2997,19 @@
       </c>
       <c r="L7" t="inlineStr">
         <is>
-          <t>終値6864 / 20日騰落-17.3% / 出来高倍率1.36 / 財務・PER未入力</t>
+          <t>終値6864 / 20日騰落-17.3% / 出来高倍率1.36 / PER25.53 / PBR2.68 / EPS268.9</t>
         </is>
       </c>
       <c r="M7" t="inlineStr">
         <is>
-          <t>価格・市場のみ計算</t>
+          <t>価格・市場・一部財務で計算</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>2026/05/14 19:35:38</t>
+          <t>2026/05/14 20:07:26</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -3074,24 +3026,20 @@
       <c r="E8">
         <v>6</v>
       </c>
-      <c r="F8" t="inlineStr">
-        <is>
-          <t/>
-        </is>
+      <c r="F8">
+        <v>5</v>
       </c>
       <c r="G8">
         <v>15</v>
       </c>
-      <c r="H8" t="inlineStr">
-        <is>
-          <t/>
-        </is>
+      <c r="H8">
+        <v>3</v>
       </c>
       <c r="I8">
         <v>10</v>
       </c>
       <c r="J8">
-        <v>59</v>
+        <v>67</v>
       </c>
       <c r="K8" t="inlineStr">
         <is>
@@ -3100,19 +3048,19 @@
       </c>
       <c r="L8" t="inlineStr">
         <is>
-          <t>終値2645.5 / 20日騰落2.46% / 出来高倍率1.2 / 財務・PER未入力</t>
+          <t>終値2645.5 / 20日騰落2.46% / 出来高倍率1.2 / PER未取得 / PBR1.98 / EPS未取得</t>
         </is>
       </c>
       <c r="M8" t="inlineStr">
         <is>
-          <t>価格・市場のみ計算</t>
+          <t>価格・市場・一部財務で計算</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2026/05/14 19:35:38</t>
+          <t>2026/05/14 20:07:26</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -3129,38 +3077,34 @@
       <c r="E9">
         <v>8</v>
       </c>
-      <c r="F9" t="inlineStr">
-        <is>
-          <t/>
-        </is>
+      <c r="F9">
+        <v>2</v>
       </c>
       <c r="G9">
         <v>15</v>
       </c>
-      <c r="H9" t="inlineStr">
-        <is>
-          <t/>
-        </is>
+      <c r="H9">
+        <v>12</v>
       </c>
       <c r="I9">
         <v>10</v>
       </c>
       <c r="J9">
-        <v>65</v>
+        <v>79</v>
       </c>
       <c r="K9" t="inlineStr">
         <is>
-          <t>少額候補（財務未確認）</t>
+          <t>少額候補（決算要確認）</t>
         </is>
       </c>
       <c r="L9" t="inlineStr">
         <is>
-          <t>終値5542 / 20日騰落19.13% / 出来高倍率1.21 / 財務・PER未入力</t>
+          <t>終値5542 / 20日騰落19.13% / 出来高倍率1.21 / PER44.27 / PBR6.89 / EPS125.2</t>
         </is>
       </c>
       <c r="M9" t="inlineStr">
         <is>
-          <t>価格・市場のみ計算</t>
+          <t>価格・市場・一部財務で計算</t>
         </is>
       </c>
     </row>
@@ -3238,7 +3182,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026/05/14 19:35:38</t>
+          <t>2026/05/14 20:07:26</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">

</xml_diff>

<commit_message>
Add top candidate review to MVP workbook
</commit_message>
<xml_diff>
--- a/stock_decision_mvp_calculated.xlsx
+++ b/stock_decision_mvp_calculated.xlsx
@@ -38,6 +38,7 @@
     <sheet name="08_predictions" sheetId="9" r:id="rId9"/>
     <sheet name="09_errors" sheetId="10" r:id="rId10"/>
     <sheet name="10_model_versions" sheetId="11" r:id="rId11"/>
+    <sheet name="11_top_review" sheetId="12" r:id="rId12"/>
   </sheets>
 </workbook>
 </file>
@@ -69,7 +70,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026/05/14 20:07:26</t>
+          <t>2026/05/14 20:13:50</t>
         </is>
       </c>
     </row>
@@ -247,7 +248,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026/05/14 20:07:26</t>
+          <t>2026/05/14 20:13:50</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -263,6 +264,177 @@
       <c r="E2" t="inlineStr">
         <is>
           <t>Codex</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+</worksheet>
+</file>
+
+<file path=xl\worksheets\sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <cols>
+    <col min="1" max="1" width="16" customWidth="1"/>
+    <col min="2" max="2" width="22" customWidth="1"/>
+    <col min="3" max="3" width="22" customWidth="1"/>
+    <col min="4" max="4" width="22" customWidth="1"/>
+    <col min="5" max="5" width="22" customWidth="1"/>
+    <col min="6" max="6" width="22" customWidth="1"/>
+    <col min="7" max="7" width="22" customWidth="1"/>
+    <col min="8" max="8" width="22" customWidth="1"/>
+    <col min="9" max="9" width="22" customWidth="1"/>
+    <col min="10" max="10" width="22" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>review_date</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>ticker</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>company</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>score_before_review</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>official_data_checked</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>positive_points</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>risk_points</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>next_action</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>source_url</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>review_status</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>2026/05/14 20:13:50</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>8058.T</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>三菱商事</t>
+        </is>
+      </c>
+      <c r="D2">
+        <v>80</v>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>2026年3月期決算短信を確認。税引前利益は前期比減、親会社所有者帰属利益も減益。一方、営業収益キャッシュフローは増加。</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>株主還元・キャッシュフローは確認対象。PBRは低めで割安性点が入りやすい。</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>減益決算。資源・事業売却益反動・ネット有利子負債増加などを確認する必要あり。</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>買い候補のまま即購入せず、2027年3月期会社予想、配当、自社株買い、資源価格感応度を確認してから判定。</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>https://www.mitsubishicorp.com/jp/ja/ir/library/earnings/pdf/202605j.pdf</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>決算要確認</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>2026/05/14 20:13:50</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>2802.T</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>味の素</t>
+        </is>
+      </c>
+      <c r="D3">
+        <v>79</v>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>2026年3月期決算短信と2027年3月期業績予想資料を確認。2026年3月期は売上高・事業利益・営業利益・親会社帰属利益が増加。</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>2027年3月期は売上高と事業利益の増収増益予想。ヘルスケア等の成長が確認対象。</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>PERが高め。2027年3月期は営業利益・親会社帰属利益が前年から減少予想のため、事業利益だけで判断しない。</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>少額候補。ただし5,300円以上を追わず、次回決算で事業利益進捗、ABF/ヘルスケア、営業利益予想を確認。</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>https://www.ajinomoto.co.jp/company/jp/ir/event/presentation/main/011111114/teaserItems1/00/linkList/03/link/FY25Q4_Presentation_J.pdf</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>少額候補・決算要確認</t>
         </is>
       </c>
     </row>
@@ -719,7 +891,7 @@
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>2026/05/14 20:07:26</t>
+          <t>2026/05/14 20:13:50</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
@@ -761,7 +933,7 @@
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>2026/05/14 20:07:26</t>
+          <t>2026/05/14 20:13:50</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
@@ -803,7 +975,7 @@
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>2026/05/14 20:07:26</t>
+          <t>2026/05/14 20:13:50</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
@@ -845,7 +1017,7 @@
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>2026/05/14 20:07:26</t>
+          <t>2026/05/14 20:13:50</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
@@ -887,7 +1059,7 @@
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>2026/05/14 20:07:26</t>
+          <t>2026/05/14 20:13:50</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
@@ -929,7 +1101,7 @@
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>2026/05/14 20:07:26</t>
+          <t>2026/05/14 20:13:50</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
@@ -971,7 +1143,7 @@
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>2026/05/14 20:07:26</t>
+          <t>2026/05/14 20:13:50</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
@@ -1013,7 +1185,7 @@
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>2026/05/14 20:07:26</t>
+          <t>2026/05/14 20:13:50</t>
         </is>
       </c>
       <c r="J9" t="inlineStr">
@@ -1113,7 +1285,7 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>2026/05/14 20:07:26</t>
+          <t>2026/05/14 20:13:50</t>
         </is>
       </c>
     </row>
@@ -1149,7 +1321,7 @@
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>2026/05/14 20:07:26</t>
+          <t>2026/05/14 20:13:50</t>
         </is>
       </c>
     </row>
@@ -1185,7 +1357,7 @@
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>2026/05/14 20:07:26</t>
+          <t>2026/05/14 20:13:50</t>
         </is>
       </c>
     </row>
@@ -1221,7 +1393,7 @@
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>2026/05/14 20:07:26</t>
+          <t>2026/05/14 20:13:50</t>
         </is>
       </c>
     </row>
@@ -1242,13 +1414,13 @@
         </is>
       </c>
       <c r="D6">
-        <v>157.94</v>
+        <v>157.89</v>
       </c>
       <c r="E6">
-        <v>0.91</v>
+        <v>0.88</v>
       </c>
       <c r="F6">
-        <v>-0.55</v>
+        <v>-0.58</v>
       </c>
       <c r="G6" t="inlineStr">
         <is>
@@ -1257,7 +1429,7 @@
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>2026/05/14 20:07:26</t>
+          <t>2026/05/14 20:13:50</t>
         </is>
       </c>
     </row>
@@ -1293,7 +1465,7 @@
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>2026/05/14 20:07:26</t>
+          <t>2026/05/14 20:13:50</t>
         </is>
       </c>
     </row>
@@ -1314,13 +1486,13 @@
         </is>
       </c>
       <c r="D8">
-        <v>17.87</v>
+        <v>17.86</v>
       </c>
       <c r="E8">
-        <v>4.63</v>
+        <v>4.57</v>
       </c>
       <c r="F8">
-        <v>-0.39</v>
+        <v>-0.45</v>
       </c>
       <c r="G8" t="inlineStr">
         <is>
@@ -1329,7 +1501,7 @@
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>2026/05/14 20:07:26</t>
+          <t>2026/05/14 20:13:50</t>
         </is>
       </c>
     </row>
@@ -1350,13 +1522,13 @@
         </is>
       </c>
       <c r="D9">
-        <v>98.52</v>
+        <v>98.55</v>
       </c>
       <c r="E9">
-        <v>0.28</v>
+        <v>0.31</v>
       </c>
       <c r="F9">
-        <v>0.31</v>
+        <v>0.34</v>
       </c>
       <c r="G9" t="inlineStr">
         <is>
@@ -1365,7 +1537,7 @@
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>2026/05/14 20:07:26</t>
+          <t>2026/05/14 20:13:50</t>
         </is>
       </c>
     </row>
@@ -1449,7 +1621,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026/05/14 20:07:26</t>
+          <t>2026/05/14 20:13:50</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -1504,7 +1676,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026/05/14 20:07:26</t>
+          <t>2026/05/14 20:13:50</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -1557,7 +1729,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2026/05/14 20:07:26</t>
+          <t>2026/05/14 20:13:50</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -1612,7 +1784,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026/05/14 20:07:26</t>
+          <t>2026/05/14 20:13:50</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -1667,7 +1839,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2026/05/14 20:07:26</t>
+          <t>2026/05/14 20:13:50</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -1720,7 +1892,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026/05/14 20:07:26</t>
+          <t>2026/05/14 20:13:50</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -1773,7 +1945,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>2026/05/14 20:07:26</t>
+          <t>2026/05/14 20:13:50</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -1828,7 +2000,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2026/05/14 20:07:26</t>
+          <t>2026/05/14 20:13:50</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -2703,7 +2875,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026/05/14 20:07:26</t>
+          <t>2026/05/14 20:13:50</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -2754,7 +2926,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026/05/14 20:07:26</t>
+          <t>2026/05/14 20:13:50</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -2805,7 +2977,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2026/05/14 20:07:26</t>
+          <t>2026/05/14 20:13:50</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -2856,7 +3028,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026/05/14 20:07:26</t>
+          <t>2026/05/14 20:13:50</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -2907,7 +3079,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2026/05/14 20:07:26</t>
+          <t>2026/05/14 20:13:50</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -2958,7 +3130,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026/05/14 20:07:26</t>
+          <t>2026/05/14 20:13:50</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -3009,7 +3181,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>2026/05/14 20:07:26</t>
+          <t>2026/05/14 20:13:50</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -3060,7 +3232,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2026/05/14 20:07:26</t>
+          <t>2026/05/14 20:13:50</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -3182,7 +3354,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026/05/14 20:07:26</t>
+          <t>2026/05/14 20:13:50</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">

</xml_diff>

<commit_message>
Add pre-buy checklist to MVP workbook
</commit_message>
<xml_diff>
--- a/stock_decision_mvp_calculated.xlsx
+++ b/stock_decision_mvp_calculated.xlsx
@@ -39,6 +39,8 @@
     <sheet name="09_errors" sheetId="10" r:id="rId10"/>
     <sheet name="10_model_versions" sheetId="11" r:id="rId11"/>
     <sheet name="11_top_review" sheetId="12" r:id="rId12"/>
+    <sheet name="12_pre_buy_checklist" sheetId="13" r:id="rId13"/>
+    <sheet name="13_buy_plan" sheetId="14" r:id="rId14"/>
   </sheets>
 </workbook>
 </file>
@@ -70,7 +72,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026/05/14 20:13:50</t>
+          <t>2026/05/14 20:43:20</t>
         </is>
       </c>
     </row>
@@ -248,7 +250,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026/05/14 20:13:50</t>
+          <t>2026/05/14 20:43:20</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -341,7 +343,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026/05/14 20:13:50</t>
+          <t>2026/05/14 20:43:20</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -391,7 +393,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026/05/14 20:13:50</t>
+          <t>2026/05/14 20:43:20</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -435,6 +437,721 @@
       <c r="J3" t="inlineStr">
         <is>
           <t>少額候補・決算要確認</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+</worksheet>
+</file>
+
+<file path=xl\worksheets\sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <cols>
+    <col min="1" max="1" width="16" customWidth="1"/>
+    <col min="2" max="2" width="22" customWidth="1"/>
+    <col min="3" max="3" width="22" customWidth="1"/>
+    <col min="4" max="4" width="22" customWidth="1"/>
+    <col min="5" max="5" width="22" customWidth="1"/>
+    <col min="6" max="6" width="22" customWidth="1"/>
+    <col min="7" max="7" width="22" customWidth="1"/>
+    <col min="8" max="8" width="22" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>check_id</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>category</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>check_item</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>pass_condition</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>current_value</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>result</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>action_if_fail</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>note</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>MKT-01</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>市場</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>日経平均の地合い</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>日経平均20日騰落率が-5%より悪くない</t>
+        </is>
+      </c>
+      <c r="E2">
+        <v>10.07</v>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>新規購入停止</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>初期MVPでは75日線判定の代替として20日騰落率を使用</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>MKT-02</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>市場</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>NASDAQの地合い</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>NASDAQ20日騰落率が-5%より悪くない</t>
+        </is>
+      </c>
+      <c r="E3">
+        <v>9.94</v>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>高PER/半導体銘柄を延期</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>AI/半導体テーマのリスク確認</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>MKT-03</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>市場</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>VIX</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>VIXが30未満。25以上なら投入半分</t>
+        </is>
+      </c>
+      <c r="E4">
+        <v>17.92</v>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>新規購入停止</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>25以上は警戒</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>MKT-04</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>市場</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>米10年金利</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>米10年金利が4.70%未満</t>
+        </is>
+      </c>
+      <c r="E5">
+        <v>4.481</v>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>高PER銘柄の購入停止</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>金利上昇は高PERに逆風</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>EVT-01</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>イベント</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>米CPI</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>2026/6/10通過後に悪化していない</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>未通過</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>未判定</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>6/10まで購入しない</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>6月上旬は仮想売買のみ</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>EVT-02</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>イベント</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>FOMC</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>2026/6/16-17通過後に金利急騰していない</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>未通過</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>未判定</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>6/18まで購入しない</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>FOMC通過後の米市場反応を見る</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>EVT-03</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>イベント</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>日銀会合</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>2026/6/19通過後に急な円高ショックがない</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>未通過</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>未判定</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>6/22まで購入しない</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>日本株全体への影響を見る</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>DATA-01</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>データ</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>価格データ取得</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>対象銘柄すべて取得成功</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>取得成功</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>購入判断に使わない</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>取得失敗時はスコア無効</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>DATA-02</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>データ</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>財務データ</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>PER/PBR/EPS等が主要候補で確認済み</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>一部取得</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>要確認</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>決算確認まで購入しない</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>Yahoo取得値は公式IR/四季報で照合</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>BUY-01</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>購入</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>初回投入額</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>総資金の5〜10%以内</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>100万円なら5万〜10万円</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>上限超過なら購入しない</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>本格購入ではなく実地テスト</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>BUY-02</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>購入</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>対象銘柄</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>スコア70点以上かつ決算レビュー済み</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>8058/2802が候補</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>要確認</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>未レビュー銘柄は買わない</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>スコア上位は買いではなくレビュー対象</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+</worksheet>
+</file>
+
+<file path=xl\worksheets\sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <cols>
+    <col min="1" max="1" width="16" customWidth="1"/>
+    <col min="2" max="2" width="22" customWidth="1"/>
+    <col min="3" max="3" width="22" customWidth="1"/>
+    <col min="4" max="4" width="22" customWidth="1"/>
+    <col min="5" max="5" width="22" customWidth="1"/>
+    <col min="6" max="6" width="22" customWidth="1"/>
+    <col min="7" max="7" width="22" customWidth="1"/>
+    <col min="8" max="8" width="22" customWidth="1"/>
+    <col min="9" max="9" width="22" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>plan_date</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>capital_case</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>max_test_amount</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>candidate_ticker</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>candidate_name</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>machine_score</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>status</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>planned_action</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>reason</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>2026-06-22以降</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>100万円</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>5万〜10万円</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>8058.T</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>三菱商事</t>
+        </is>
+      </c>
+      <c r="F2">
+        <v>80</v>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>決算要確認</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>条件が揃えば少額候補</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>PBR/還元は候補。ただし減益・資源価格・会社予想を確認</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>2026-06-22以降</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>100万円</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>5万〜10万円</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>2802.T</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>味の素</t>
+        </is>
+      </c>
+      <c r="F3">
+        <v>79</v>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>決算要確認</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>条件が揃えば少額候補</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>事業利益成長は候補。ただしPER高め、営業利益/純利益予想を確認</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>2026-06-22以降</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>200万円</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>10万〜20万円</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>8058.T / 2802.T</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>三菱商事 / 味の素</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>分散検討</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>1銘柄集中せず分割</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>初回はモデル検証目的のため上限を超えない</t>
         </is>
       </c>
     </row>
@@ -891,7 +1608,7 @@
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>2026/05/14 20:13:50</t>
+          <t>2026/05/14 20:43:20</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
@@ -933,7 +1650,7 @@
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>2026/05/14 20:13:50</t>
+          <t>2026/05/14 20:43:20</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
@@ -975,7 +1692,7 @@
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>2026/05/14 20:13:50</t>
+          <t>2026/05/14 20:43:20</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
@@ -1017,7 +1734,7 @@
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>2026/05/14 20:13:50</t>
+          <t>2026/05/14 20:43:20</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
@@ -1059,7 +1776,7 @@
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>2026/05/14 20:13:50</t>
+          <t>2026/05/14 20:43:20</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
@@ -1101,7 +1818,7 @@
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>2026/05/14 20:13:50</t>
+          <t>2026/05/14 20:43:20</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
@@ -1143,7 +1860,7 @@
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>2026/05/14 20:13:50</t>
+          <t>2026/05/14 20:43:20</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
@@ -1185,7 +1902,7 @@
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>2026/05/14 20:13:50</t>
+          <t>2026/05/14 20:43:20</t>
         </is>
       </c>
       <c r="J9" t="inlineStr">
@@ -1285,7 +2002,7 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>2026/05/14 20:13:50</t>
+          <t>2026/05/14 20:43:20</t>
         </is>
       </c>
     </row>
@@ -1321,7 +2038,7 @@
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>2026/05/14 20:13:50</t>
+          <t>2026/05/14 20:43:20</t>
         </is>
       </c>
     </row>
@@ -1357,7 +2074,7 @@
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>2026/05/14 20:13:50</t>
+          <t>2026/05/14 20:43:20</t>
         </is>
       </c>
     </row>
@@ -1393,7 +2110,7 @@
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>2026/05/14 20:13:50</t>
+          <t>2026/05/14 20:43:20</t>
         </is>
       </c>
     </row>
@@ -1414,13 +2131,13 @@
         </is>
       </c>
       <c r="D6">
-        <v>157.89</v>
+        <v>157.94</v>
       </c>
       <c r="E6">
-        <v>0.88</v>
+        <v>0.92</v>
       </c>
       <c r="F6">
-        <v>-0.58</v>
+        <v>-0.54</v>
       </c>
       <c r="G6" t="inlineStr">
         <is>
@@ -1429,7 +2146,7 @@
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>2026/05/14 20:13:50</t>
+          <t>2026/05/14 20:43:20</t>
         </is>
       </c>
     </row>
@@ -1465,7 +2182,7 @@
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>2026/05/14 20:13:50</t>
+          <t>2026/05/14 20:43:20</t>
         </is>
       </c>
     </row>
@@ -1486,13 +2203,13 @@
         </is>
       </c>
       <c r="D8">
-        <v>17.86</v>
+        <v>17.92</v>
       </c>
       <c r="E8">
-        <v>4.57</v>
+        <v>4.92</v>
       </c>
       <c r="F8">
-        <v>-0.45</v>
+        <v>-0.11</v>
       </c>
       <c r="G8" t="inlineStr">
         <is>
@@ -1501,7 +2218,7 @@
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>2026/05/14 20:13:50</t>
+          <t>2026/05/14 20:43:20</t>
         </is>
       </c>
     </row>
@@ -1522,7 +2239,7 @@
         </is>
       </c>
       <c r="D9">
-        <v>98.55</v>
+        <v>98.56</v>
       </c>
       <c r="E9">
         <v>0.31</v>
@@ -1537,7 +2254,7 @@
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>2026/05/14 20:13:50</t>
+          <t>2026/05/14 20:43:20</t>
         </is>
       </c>
     </row>
@@ -1621,7 +2338,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026/05/14 20:13:50</t>
+          <t>2026/05/14 20:43:20</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -1676,7 +2393,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026/05/14 20:13:50</t>
+          <t>2026/05/14 20:43:20</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -1729,7 +2446,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2026/05/14 20:13:50</t>
+          <t>2026/05/14 20:43:20</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -1784,7 +2501,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026/05/14 20:13:50</t>
+          <t>2026/05/14 20:43:20</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -1839,7 +2556,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2026/05/14 20:13:50</t>
+          <t>2026/05/14 20:43:20</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -1892,7 +2609,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026/05/14 20:13:50</t>
+          <t>2026/05/14 20:43:20</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -1945,7 +2662,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>2026/05/14 20:13:50</t>
+          <t>2026/05/14 20:43:20</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -2000,7 +2717,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2026/05/14 20:13:50</t>
+          <t>2026/05/14 20:43:20</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -2875,7 +3592,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026/05/14 20:13:50</t>
+          <t>2026/05/14 20:43:20</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -2926,7 +3643,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026/05/14 20:13:50</t>
+          <t>2026/05/14 20:43:20</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -2977,7 +3694,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2026/05/14 20:13:50</t>
+          <t>2026/05/14 20:43:20</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -3028,7 +3745,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026/05/14 20:13:50</t>
+          <t>2026/05/14 20:43:20</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -3079,7 +3796,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2026/05/14 20:13:50</t>
+          <t>2026/05/14 20:43:20</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -3130,7 +3847,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026/05/14 20:13:50</t>
+          <t>2026/05/14 20:43:20</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -3181,7 +3898,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>2026/05/14 20:13:50</t>
+          <t>2026/05/14 20:43:20</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -3232,7 +3949,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2026/05/14 20:13:50</t>
+          <t>2026/05/14 20:43:20</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -3354,7 +4071,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026/05/14 20:13:50</t>
+          <t>2026/05/14 20:43:20</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">

</xml_diff>

<commit_message>
Add MVP daily score history
</commit_message>
<xml_diff>
--- a/stock_decision_mvp_calculated.xlsx
+++ b/stock_decision_mvp_calculated.xlsx
@@ -41,6 +41,7 @@
     <sheet name="11_top_review" sheetId="12" r:id="rId12"/>
     <sheet name="12_pre_buy_checklist" sheetId="13" r:id="rId13"/>
     <sheet name="13_buy_plan" sheetId="14" r:id="rId14"/>
+    <sheet name="14_score_history" sheetId="15" r:id="rId15"/>
   </sheets>
 </workbook>
 </file>
@@ -72,7 +73,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026/05/14 20:43:20</t>
+          <t>2026/05/14 20:46:40</t>
         </is>
       </c>
     </row>
@@ -250,7 +251,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026/05/14 20:43:20</t>
+          <t>2026/05/14 20:46:40</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -343,7 +344,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026/05/14 20:43:20</t>
+          <t>2026/05/14 20:46:40</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -393,7 +394,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026/05/14 20:43:20</t>
+          <t>2026/05/14 20:46:40</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -601,7 +602,7 @@
         </is>
       </c>
       <c r="E4">
-        <v>17.92</v>
+        <v>17.88</v>
       </c>
       <c r="F4" t="inlineStr">
         <is>
@@ -1152,6 +1153,565 @@
       <c r="I4" t="inlineStr">
         <is>
           <t>初回はモデル検証目的のため上限を超えない</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+</worksheet>
+</file>
+
+<file path=xl\worksheets\sheet15.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <cols>
+    <col min="1" max="1" width="16" customWidth="1"/>
+    <col min="2" max="2" width="22" customWidth="1"/>
+    <col min="3" max="3" width="22" customWidth="1"/>
+    <col min="4" max="4" width="22" customWidth="1"/>
+    <col min="5" max="5" width="22" customWidth="1"/>
+    <col min="6" max="6" width="22" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>updated_at</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>ticker</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>score</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>decision</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>status</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>reason</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>2026/05/14 20:45:31</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>8035.T</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>60</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>様子見</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>価格・市場・一部財務で計算</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>終値51200 / 20日騰落16.26% / 出来高倍率0.61 / PER未取得 / PBR11.38 / EPS未取得</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>2026/05/14 20:45:31</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>6857.T</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>69</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>様子見</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>価格・市場・一部財務で計算</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>終値28615 / 20日騰落14.51% / 出来高倍率0.9 / PER44.6 / PBR26.07 / EPS641.61</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>2026/05/14 20:45:31</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>4519.T</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>33</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>除外/待機</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>価格・市場・一部財務で計算</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>終値8096 / 20日騰落-6.67% / 出来高倍率0.75 / PER未取得 / PBR6.98 / EPS未取得</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>2026/05/14 20:45:31</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>8306.T</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>68</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>様子見</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>価格・市場・一部財務で計算</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>終値2877 / 20日騰落1.23% / 出来高倍率0.96 / PER未取得 / PBR1.53 / EPS未取得</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>2026/05/14 20:45:31</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>8058.T</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>80</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>買い候補（決算要確認）</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>価格・市場・一部財務で計算</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>終値5882 / 20日騰落10.83% / 出来高倍率0.71 / PER19.58 / PBR2.28 / EPS300.42</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>2026/05/14 20:45:31</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>7974.T</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>44</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>除外/待機</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>価格・市場・一部財務で計算</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>終値6864 / 20日騰落-17.3% / 出来高倍率1.36 / PER25.53 / PBR2.68 / EPS268.9</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>2026/05/14 20:45:31</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>9433.T</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>67</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>様子見</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>価格・市場・一部財務で計算</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>終値2645.5 / 20日騰落2.46% / 出来高倍率1.2 / PER未取得 / PBR1.98 / EPS未取得</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>2026/05/14 20:45:31</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>2802.T</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>79</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>少額候補（決算要確認）</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>価格・市場・一部財務で計算</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>終値5542 / 20日騰落19.13% / 出来高倍率1.21 / PER44.27 / PBR6.89 / EPS125.2</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>2026/05/14 20:46:40</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>8035.T</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>60</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>様子見</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>価格・市場・一部財務で計算</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>終値51200 / 20日騰落16.26% / 出来高倍率0.61 / PER未取得 / PBR11.38 / EPS未取得</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>2026/05/14 20:46:40</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>6857.T</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>69</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>様子見</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>価格・市場・一部財務で計算</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>終値28615 / 20日騰落14.51% / 出来高倍率0.9 / PER44.6 / PBR26.07 / EPS641.61</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>2026/05/14 20:46:40</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>4519.T</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>33</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>除外/待機</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>価格・市場・一部財務で計算</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>終値8096 / 20日騰落-6.67% / 出来高倍率0.75 / PER未取得 / PBR6.98 / EPS未取得</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>2026/05/14 20:46:40</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>8306.T</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>68</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>様子見</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>価格・市場・一部財務で計算</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>終値2877 / 20日騰落1.23% / 出来高倍率0.96 / PER未取得 / PBR1.53 / EPS未取得</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>2026/05/14 20:46:40</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>8058.T</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>80</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>買い候補（決算要確認）</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>価格・市場・一部財務で計算</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>終値5882 / 20日騰落10.83% / 出来高倍率0.71 / PER19.58 / PBR2.28 / EPS300.42</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>2026/05/14 20:46:40</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>7974.T</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>44</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>除外/待機</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>価格・市場・一部財務で計算</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>終値6864 / 20日騰落-17.3% / 出来高倍率1.36 / PER25.53 / PBR2.68 / EPS268.9</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>2026/05/14 20:46:40</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>9433.T</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>67</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>様子見</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>価格・市場・一部財務で計算</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>終値2645.5 / 20日騰落2.46% / 出来高倍率1.2 / PER未取得 / PBR1.98 / EPS未取得</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>2026/05/14 20:46:40</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>2802.T</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>79</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>少額候補（決算要確認）</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>価格・市場・一部財務で計算</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>終値5542 / 20日騰落19.13% / 出来高倍率1.21 / PER44.27 / PBR6.89 / EPS125.2</t>
         </is>
       </c>
     </row>
@@ -1608,7 +2168,7 @@
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>2026/05/14 20:43:20</t>
+          <t>2026/05/14 20:46:40</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
@@ -1650,7 +2210,7 @@
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>2026/05/14 20:43:20</t>
+          <t>2026/05/14 20:46:40</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
@@ -1692,7 +2252,7 @@
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>2026/05/14 20:43:20</t>
+          <t>2026/05/14 20:46:40</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
@@ -1734,7 +2294,7 @@
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>2026/05/14 20:43:20</t>
+          <t>2026/05/14 20:46:40</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
@@ -1776,7 +2336,7 @@
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>2026/05/14 20:43:20</t>
+          <t>2026/05/14 20:46:40</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
@@ -1818,7 +2378,7 @@
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>2026/05/14 20:43:20</t>
+          <t>2026/05/14 20:46:40</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
@@ -1860,7 +2420,7 @@
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>2026/05/14 20:43:20</t>
+          <t>2026/05/14 20:46:40</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
@@ -1902,7 +2462,7 @@
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>2026/05/14 20:43:20</t>
+          <t>2026/05/14 20:46:40</t>
         </is>
       </c>
       <c r="J9" t="inlineStr">
@@ -2002,7 +2562,7 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>2026/05/14 20:43:20</t>
+          <t>2026/05/14 20:46:40</t>
         </is>
       </c>
     </row>
@@ -2038,7 +2598,7 @@
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>2026/05/14 20:43:20</t>
+          <t>2026/05/14 20:46:40</t>
         </is>
       </c>
     </row>
@@ -2074,7 +2634,7 @@
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>2026/05/14 20:43:20</t>
+          <t>2026/05/14 20:46:40</t>
         </is>
       </c>
     </row>
@@ -2110,7 +2670,7 @@
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>2026/05/14 20:43:20</t>
+          <t>2026/05/14 20:46:40</t>
         </is>
       </c>
     </row>
@@ -2134,10 +2694,10 @@
         <v>157.94</v>
       </c>
       <c r="E6">
-        <v>0.92</v>
+        <v>0.91</v>
       </c>
       <c r="F6">
-        <v>-0.54</v>
+        <v>-0.55</v>
       </c>
       <c r="G6" t="inlineStr">
         <is>
@@ -2146,7 +2706,7 @@
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>2026/05/14 20:43:20</t>
+          <t>2026/05/14 20:46:40</t>
         </is>
       </c>
     </row>
@@ -2182,7 +2742,7 @@
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>2026/05/14 20:43:20</t>
+          <t>2026/05/14 20:46:40</t>
         </is>
       </c>
     </row>
@@ -2203,13 +2763,13 @@
         </is>
       </c>
       <c r="D8">
-        <v>17.92</v>
+        <v>17.88</v>
       </c>
       <c r="E8">
-        <v>4.92</v>
+        <v>4.68</v>
       </c>
       <c r="F8">
-        <v>-0.11</v>
+        <v>-0.33</v>
       </c>
       <c r="G8" t="inlineStr">
         <is>
@@ -2218,7 +2778,7 @@
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>2026/05/14 20:43:20</t>
+          <t>2026/05/14 20:46:40</t>
         </is>
       </c>
     </row>
@@ -2239,13 +2799,13 @@
         </is>
       </c>
       <c r="D9">
-        <v>98.56</v>
+        <v>98.57</v>
       </c>
       <c r="E9">
-        <v>0.31</v>
+        <v>0.32</v>
       </c>
       <c r="F9">
-        <v>0.34</v>
+        <v>0.36</v>
       </c>
       <c r="G9" t="inlineStr">
         <is>
@@ -2254,7 +2814,7 @@
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>2026/05/14 20:43:20</t>
+          <t>2026/05/14 20:46:40</t>
         </is>
       </c>
     </row>
@@ -2338,7 +2898,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026/05/14 20:43:20</t>
+          <t>2026/05/14 20:46:40</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -2393,7 +2953,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026/05/14 20:43:20</t>
+          <t>2026/05/14 20:46:40</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -2446,7 +3006,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2026/05/14 20:43:20</t>
+          <t>2026/05/14 20:46:40</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -2501,7 +3061,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026/05/14 20:43:20</t>
+          <t>2026/05/14 20:46:40</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -2556,7 +3116,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2026/05/14 20:43:20</t>
+          <t>2026/05/14 20:46:40</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -2609,7 +3169,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026/05/14 20:43:20</t>
+          <t>2026/05/14 20:46:40</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -2662,7 +3222,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>2026/05/14 20:43:20</t>
+          <t>2026/05/14 20:46:40</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -2717,7 +3277,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2026/05/14 20:43:20</t>
+          <t>2026/05/14 20:46:40</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -3592,7 +4152,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026/05/14 20:43:20</t>
+          <t>2026/05/14 20:46:40</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -3643,7 +4203,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026/05/14 20:43:20</t>
+          <t>2026/05/14 20:46:40</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -3694,7 +4254,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2026/05/14 20:43:20</t>
+          <t>2026/05/14 20:46:40</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -3745,7 +4305,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026/05/14 20:43:20</t>
+          <t>2026/05/14 20:46:40</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -3796,7 +4356,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2026/05/14 20:43:20</t>
+          <t>2026/05/14 20:46:40</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -3847,7 +4407,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026/05/14 20:43:20</t>
+          <t>2026/05/14 20:46:40</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -3898,7 +4458,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>2026/05/14 20:43:20</t>
+          <t>2026/05/14 20:46:40</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -3949,7 +4509,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2026/05/14 20:43:20</t>
+          <t>2026/05/14 20:46:40</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -4071,7 +4631,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026/05/14 20:43:20</t>
+          <t>2026/05/14 20:46:40</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">

</xml_diff>

<commit_message>
Add review adjusted scoring
</commit_message>
<xml_diff>
--- a/stock_decision_mvp_calculated.xlsx
+++ b/stock_decision_mvp_calculated.xlsx
@@ -42,6 +42,7 @@
     <sheet name="12_pre_buy_checklist" sheetId="13" r:id="rId13"/>
     <sheet name="13_buy_plan" sheetId="14" r:id="rId14"/>
     <sheet name="14_score_history" sheetId="15" r:id="rId15"/>
+    <sheet name="15_review_adjusted" sheetId="16" r:id="rId16"/>
   </sheets>
 </workbook>
 </file>
@@ -73,7 +74,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026/05/14 20:46:40</t>
+          <t>2026/05/14 20:52:36</t>
         </is>
       </c>
     </row>
@@ -251,7 +252,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026/05/14 20:46:40</t>
+          <t>2026/05/14 20:52:36</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -344,7 +345,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026/05/14 20:46:40</t>
+          <t>2026/05/14 20:52:36</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -394,7 +395,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026/05/14 20:46:40</t>
+          <t>2026/05/14 20:52:36</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -1712,6 +1713,437 @@
       <c r="F17" t="inlineStr">
         <is>
           <t>終値5542 / 20日騰落19.13% / 出来高倍率1.21 / PER44.27 / PBR6.89 / EPS125.2</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>2026/05/14 20:52:36</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>8035.T</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>60</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>様子見</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>価格・市場・一部財務で計算</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>終値51200 / 20日騰落16.26% / 出来高倍率0.61 / PER未取得 / PBR11.38 / EPS未取得</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>2026/05/14 20:52:36</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>6857.T</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>69</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>様子見</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>価格・市場・一部財務で計算</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>終値28615 / 20日騰落14.51% / 出来高倍率0.9 / PER44.6 / PBR26.07 / EPS641.61</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>2026/05/14 20:52:36</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>4519.T</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>33</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>除外/待機</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>価格・市場・一部財務で計算</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>終値8096 / 20日騰落-6.67% / 出来高倍率0.75 / PER未取得 / PBR6.98 / EPS未取得</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>2026/05/14 20:52:36</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>8306.T</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>68</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>様子見</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>価格・市場・一部財務で計算</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>終値2877 / 20日騰落1.23% / 出来高倍率0.96 / PER未取得 / PBR1.53 / EPS未取得</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>2026/05/14 20:52:36</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>8058.T</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>80</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>買い候補（決算要確認）</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>価格・市場・一部財務で計算</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>終値5882 / 20日騰落10.83% / 出来高倍率0.71 / PER19.58 / PBR2.28 / EPS300.42</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>2026/05/14 20:52:36</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>7974.T</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>44</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>除外/待機</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>価格・市場・一部財務で計算</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>終値6864 / 20日騰落-17.3% / 出来高倍率1.36 / PER25.53 / PBR2.68 / EPS268.9</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>2026/05/14 20:52:36</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>9433.T</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>67</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>様子見</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>価格・市場・一部財務で計算</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>終値2645.5 / 20日騰落2.46% / 出来高倍率1.2 / PER未取得 / PBR1.98 / EPS未取得</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>2026/05/14 20:52:36</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>2802.T</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>79</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>少額候補（決算要確認）</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>価格・市場・一部財務で計算</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>終値5542 / 20日騰落19.13% / 出来高倍率1.21 / PER44.27 / PBR6.89 / EPS125.2</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+</worksheet>
+</file>
+
+<file path=xl\worksheets\sheet16.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <cols>
+    <col min="1" max="1" width="16" customWidth="1"/>
+    <col min="2" max="2" width="22" customWidth="1"/>
+    <col min="3" max="3" width="22" customWidth="1"/>
+    <col min="4" max="4" width="22" customWidth="1"/>
+    <col min="5" max="5" width="22" customWidth="1"/>
+    <col min="6" max="6" width="22" customWidth="1"/>
+    <col min="7" max="7" width="22" customWidth="1"/>
+    <col min="8" max="8" width="22" customWidth="1"/>
+    <col min="9" max="9" width="22" customWidth="1"/>
+    <col min="10" max="10" width="22" customWidth="1"/>
+    <col min="11" max="11" width="22" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>review_date</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>ticker</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>company</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>machine_score</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>positive_adjustment</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>negative_adjustment</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>review_score</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>review_result</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>official_numbers</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>reason</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>source_url</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>2026/05/14 20:52:36</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>8058.T</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>三菱商事</t>
+        </is>
+      </c>
+      <c r="D2">
+        <v>80</v>
+      </c>
+      <c r="E2">
+        <v>7</v>
+      </c>
+      <c r="F2">
+        <v>-11</v>
+      </c>
+      <c r="G2">
+        <v>76</v>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>条件付き少額候補。即購入ではなく6月イベント通過後に再判定</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>2026年3月期: 収益189,160億円、親会社所有者帰属利益8,005億円。2027年3月期見通し: 当期純利益11,000億円。FCF10,414億円。</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>翌期利益見通しと還元方針はプラス。一方、2026年3月期は親会社帰属利益が9,507億円から8,005億円へ減少、FCFも13,844億円から10,414億円へ減少。資源価格と一過性要因の確認が必要。</t>
+        </is>
+      </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>https://www.mitsubishicorp.com/jp/ja/ir/library/earnings/pdf/202605j.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>2026/05/14 20:52:36</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>2802.T</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>味の素</t>
+        </is>
+      </c>
+      <c r="D3">
+        <v>79</v>
+      </c>
+      <c r="E3">
+        <v>8</v>
+      </c>
+      <c r="F3">
+        <v>-15</v>
+      </c>
+      <c r="G3">
+        <v>72</v>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>条件付き少額候補。高値追い禁止、次決算確認優先</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>2026年3月期: 売上高1,583,719百万円、事業利益181,163百万円、営業利益199,412百万円、親会社帰属利益134,675百万円。2027年3月期予想: 売上高17,230億円、事業利益1,970億円、営業利益1,792億円、親会社帰属利益1,200億円。</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>売上高と事業利益の増収増益予想はプラス。一方、PER44倍台で割高、2027年3月期は営業利益・親会社帰属利益が減益予想。中東情勢で事業利益に300億円規模の影響可能性が示されており、追い買いは不可。</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>https://www.ajinomoto.co.jp/company/jp/ir/event/presentation/main/011111114/teaserItems1/00/linkList/03/link/FY25Q4_Presentation_J.pdf</t>
         </is>
       </c>
     </row>
@@ -2168,7 +2600,7 @@
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>2026/05/14 20:46:40</t>
+          <t>2026/05/14 20:52:36</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
@@ -2210,7 +2642,7 @@
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>2026/05/14 20:46:40</t>
+          <t>2026/05/14 20:52:36</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
@@ -2252,7 +2684,7 @@
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>2026/05/14 20:46:40</t>
+          <t>2026/05/14 20:52:36</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
@@ -2294,7 +2726,7 @@
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>2026/05/14 20:46:40</t>
+          <t>2026/05/14 20:52:36</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
@@ -2336,7 +2768,7 @@
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>2026/05/14 20:46:40</t>
+          <t>2026/05/14 20:52:36</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
@@ -2378,7 +2810,7 @@
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>2026/05/14 20:46:40</t>
+          <t>2026/05/14 20:52:36</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
@@ -2420,7 +2852,7 @@
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>2026/05/14 20:46:40</t>
+          <t>2026/05/14 20:52:36</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
@@ -2462,7 +2894,7 @@
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>2026/05/14 20:46:40</t>
+          <t>2026/05/14 20:52:36</t>
         </is>
       </c>
       <c r="J9" t="inlineStr">
@@ -2562,7 +2994,7 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>2026/05/14 20:46:40</t>
+          <t>2026/05/14 20:52:36</t>
         </is>
       </c>
     </row>
@@ -2598,7 +3030,7 @@
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>2026/05/14 20:46:40</t>
+          <t>2026/05/14 20:52:36</t>
         </is>
       </c>
     </row>
@@ -2634,7 +3066,7 @@
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>2026/05/14 20:46:40</t>
+          <t>2026/05/14 20:52:36</t>
         </is>
       </c>
     </row>
@@ -2670,7 +3102,7 @@
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>2026/05/14 20:46:40</t>
+          <t>2026/05/14 20:52:36</t>
         </is>
       </c>
     </row>
@@ -2691,13 +3123,13 @@
         </is>
       </c>
       <c r="D6">
-        <v>157.94</v>
+        <v>157.9</v>
       </c>
       <c r="E6">
-        <v>0.91</v>
+        <v>0.89</v>
       </c>
       <c r="F6">
-        <v>-0.55</v>
+        <v>-0.57</v>
       </c>
       <c r="G6" t="inlineStr">
         <is>
@@ -2706,7 +3138,7 @@
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>2026/05/14 20:46:40</t>
+          <t>2026/05/14 20:52:36</t>
         </is>
       </c>
     </row>
@@ -2742,7 +3174,7 @@
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>2026/05/14 20:46:40</t>
+          <t>2026/05/14 20:52:36</t>
         </is>
       </c>
     </row>
@@ -2778,7 +3210,7 @@
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>2026/05/14 20:46:40</t>
+          <t>2026/05/14 20:52:36</t>
         </is>
       </c>
     </row>
@@ -2802,7 +3234,7 @@
         <v>98.57</v>
       </c>
       <c r="E9">
-        <v>0.32</v>
+        <v>0.33</v>
       </c>
       <c r="F9">
         <v>0.36</v>
@@ -2814,7 +3246,7 @@
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>2026/05/14 20:46:40</t>
+          <t>2026/05/14 20:52:36</t>
         </is>
       </c>
     </row>
@@ -2898,7 +3330,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026/05/14 20:46:40</t>
+          <t>2026/05/14 20:52:36</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -2953,7 +3385,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026/05/14 20:46:40</t>
+          <t>2026/05/14 20:52:36</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -3006,7 +3438,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2026/05/14 20:46:40</t>
+          <t>2026/05/14 20:52:36</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -3061,7 +3493,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026/05/14 20:46:40</t>
+          <t>2026/05/14 20:52:36</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -3116,7 +3548,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2026/05/14 20:46:40</t>
+          <t>2026/05/14 20:52:36</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -3169,7 +3601,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026/05/14 20:46:40</t>
+          <t>2026/05/14 20:52:36</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -3222,7 +3654,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>2026/05/14 20:46:40</t>
+          <t>2026/05/14 20:52:36</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -3277,7 +3709,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2026/05/14 20:46:40</t>
+          <t>2026/05/14 20:52:36</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -4152,7 +4584,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026/05/14 20:46:40</t>
+          <t>2026/05/14 20:52:36</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -4203,7 +4635,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026/05/14 20:46:40</t>
+          <t>2026/05/14 20:52:36</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -4254,7 +4686,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2026/05/14 20:46:40</t>
+          <t>2026/05/14 20:52:36</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -4305,7 +4737,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026/05/14 20:46:40</t>
+          <t>2026/05/14 20:52:36</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -4356,7 +4788,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2026/05/14 20:46:40</t>
+          <t>2026/05/14 20:52:36</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -4407,7 +4839,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026/05/14 20:46:40</t>
+          <t>2026/05/14 20:52:36</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -4458,7 +4890,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>2026/05/14 20:46:40</t>
+          <t>2026/05/14 20:52:36</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -4509,7 +4941,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2026/05/14 20:46:40</t>
+          <t>2026/05/14 20:52:36</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -4631,7 +5063,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026/05/14 20:46:40</t>
+          <t>2026/05/14 20:52:36</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">

</xml_diff>

<commit_message>
Add formula audit sheets to MVP workbook
</commit_message>
<xml_diff>
--- a/stock_decision_mvp_calculated.xlsx
+++ b/stock_decision_mvp_calculated.xlsx
@@ -43,6 +43,8 @@
     <sheet name="13_buy_plan" sheetId="14" r:id="rId14"/>
     <sheet name="14_score_history" sheetId="15" r:id="rId15"/>
     <sheet name="15_review_adjusted" sheetId="16" r:id="rId16"/>
+    <sheet name="16_formula_spec" sheetId="17" r:id="rId17"/>
+    <sheet name="17_excel_audit" sheetId="18" r:id="rId18"/>
   </sheets>
 </workbook>
 </file>
@@ -74,7 +76,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026/05/14 20:52:36</t>
+          <t>2026/05/14 20:55:23</t>
         </is>
       </c>
     </row>
@@ -252,7 +254,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026/05/14 20:52:36</t>
+          <t>2026/05/14 20:55:23</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -345,7 +347,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026/05/14 20:52:36</t>
+          <t>2026/05/14 20:55:23</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -395,7 +397,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026/05/14 20:52:36</t>
+          <t>2026/05/14 20:55:23</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -603,7 +605,7 @@
         </is>
       </c>
       <c r="E4">
-        <v>17.88</v>
+        <v>17.87</v>
       </c>
       <c r="F4" t="inlineStr">
         <is>
@@ -1967,6 +1969,262 @@
         </is>
       </c>
       <c r="F25" t="inlineStr">
+        <is>
+          <t>終値5542 / 20日騰落19.13% / 出来高倍率1.21 / PER44.27 / PBR6.89 / EPS125.2</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>2026/05/14 20:55:23</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>8035.T</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>60</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>様子見</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>価格・市場・一部財務で計算</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>終値51200 / 20日騰落16.26% / 出来高倍率0.61 / PER未取得 / PBR11.38 / EPS未取得</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>2026/05/14 20:55:23</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>6857.T</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>69</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>様子見</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>価格・市場・一部財務で計算</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>終値28615 / 20日騰落14.51% / 出来高倍率0.9 / PER44.6 / PBR26.07 / EPS641.61</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>2026/05/14 20:55:23</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>4519.T</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>33</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>除外/待機</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>価格・市場・一部財務で計算</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>終値8096 / 20日騰落-6.67% / 出来高倍率0.75 / PER未取得 / PBR6.98 / EPS未取得</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>2026/05/14 20:55:23</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>8306.T</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>68</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>様子見</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>価格・市場・一部財務で計算</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>終値2877 / 20日騰落1.23% / 出来高倍率0.96 / PER未取得 / PBR1.53 / EPS未取得</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>2026/05/14 20:55:23</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>8058.T</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>80</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>買い候補（決算要確認）</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>価格・市場・一部財務で計算</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>終値5882 / 20日騰落10.83% / 出来高倍率0.71 / PER19.58 / PBR2.28 / EPS300.42</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>2026/05/14 20:55:23</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>7974.T</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>44</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>除外/待機</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>価格・市場・一部財務で計算</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>終値6864 / 20日騰落-17.3% / 出来高倍率1.36 / PER25.53 / PBR2.68 / EPS268.9</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>2026/05/14 20:55:23</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>9433.T</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>67</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>様子見</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>価格・市場・一部財務で計算</t>
+        </is>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>終値2645.5 / 20日騰落2.46% / 出来高倍率1.2 / PER未取得 / PBR1.98 / EPS未取得</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>2026/05/14 20:55:23</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>2802.T</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>79</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>少額候補（決算要確認）</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>価格・市場・一部財務で計算</t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr">
         <is>
           <t>終値5542 / 20日騰落19.13% / 出来高倍率1.21 / PER44.27 / PBR6.89 / EPS125.2</t>
         </is>
@@ -2052,7 +2310,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026/05/14 20:52:36</t>
+          <t>2026/05/14 20:55:23</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -2101,7 +2359,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026/05/14 20:52:36</t>
+          <t>2026/05/14 20:55:23</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -2145,6 +2403,938 @@
         <is>
           <t>https://www.ajinomoto.co.jp/company/jp/ir/event/presentation/main/011111114/teaserItems1/00/linkList/03/link/FY25Q4_Presentation_J.pdf</t>
         </is>
+      </c>
+    </row>
+  </sheetData>
+</worksheet>
+</file>
+
+<file path=xl\worksheets\sheet17.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <cols>
+    <col min="1" max="1" width="16" customWidth="1"/>
+    <col min="2" max="2" width="22" customWidth="1"/>
+    <col min="3" max="3" width="22" customWidth="1"/>
+    <col min="4" max="4" width="22" customWidth="1"/>
+    <col min="5" max="5" width="22" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>score_part</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>max_point</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>input_data</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>formula_rule</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>current_status</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>trend_20</t>
+        </is>
+      </c>
+      <c r="B2">
+        <v>20</v>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>close, ma25, ma75, ma200</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>close&gt;=ma25で+6、close&gt;=ma75で+7、close&gt;=ma200で+7</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>実データ計算済</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>momentum_15</t>
+        </is>
+      </c>
+      <c r="B3">
+        <v>15</v>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>ret5_pct, ret20_pct, ret60_pct</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>ret5&gt;0で+4、ret20&gt;0で+5、ret60&gt;0で+6、ret20&gt;15なら-3</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>実データ計算済</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>volume_10</t>
+        </is>
+      </c>
+      <c r="B4">
+        <v>10</v>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>volume_ratio20</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>1.5以上=10、1.2以上=8、0.8以上=6、それ未満=3</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>実データ計算済</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>valuation_15</t>
+        </is>
+      </c>
+      <c r="B5">
+        <v>15</v>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>PER, PBR</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>PER&lt;=15で+8、&lt;=25で+6、&lt;=40で+3、それ以上+1。PBR&lt;=1.2で+7、&lt;=2で+5、&lt;=4で+3、それ以上+1</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>一部財務で計算</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>macro_15</t>
+        </is>
+      </c>
+      <c r="B6">
+        <v>15</v>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>VIX, US10Y, Nikkei20d, Nasdaq20d</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>初期15点から、VIX&gt;=25で-5、VIX&gt;=30で-5、US10Y&gt;=4.7で-3、日経20日&lt;-5で-3、NASDAQ20日&lt;-5で-3</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>実データ計算済</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>fundamental_15</t>
+        </is>
+      </c>
+      <c r="B7">
+        <v>15</v>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>EPS, PER, PBR</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>EPS&gt;0で+6、PER取得で+3、PBR取得で+3。売上/営業利益成長は未実装</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>一部財務で計算</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>risk_10</t>
+        </is>
+      </c>
+      <c r="B8">
+        <v>10</v>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>max_drawdown20, volatility20</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>初期10点から、20日最大下落&lt;-10で-4、&lt;-15で-3、ボラ&gt;3.5で-3、&gt;5で-2</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>実データ計算済</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>review_adjusted</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>公式決算資料</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>機械スコアに対して決算・会社予想・リスクで加点/減点</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>一部手動</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+</worksheet>
+</file>
+
+<file path=xl\worksheets\sheet18.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <cols>
+    <col min="1" max="1" width="16" customWidth="1"/>
+    <col min="2" max="2" width="22" customWidth="1"/>
+    <col min="3" max="3" width="22" customWidth="1"/>
+    <col min="4" max="4" width="22" customWidth="1"/>
+    <col min="5" max="5" width="22" customWidth="1"/>
+    <col min="6" max="6" width="22" customWidth="1"/>
+    <col min="7" max="7" width="22" customWidth="1"/>
+    <col min="8" max="8" width="22" customWidth="1"/>
+    <col min="9" max="9" width="22" customWidth="1"/>
+    <col min="10" max="10" width="22" customWidth="1"/>
+    <col min="11" max="11" width="22" customWidth="1"/>
+    <col min="12" max="12" width="22" customWidth="1"/>
+    <col min="13" max="13" width="22" customWidth="1"/>
+    <col min="14" max="14" width="22" customWidth="1"/>
+    <col min="15" max="15" width="22" customWidth="1"/>
+    <col min="16" max="16" width="22" customWidth="1"/>
+    <col min="17" max="17" width="22" customWidth="1"/>
+    <col min="18" max="18" width="22" customWidth="1"/>
+    <col min="19" max="19" width="22" customWidth="1"/>
+    <col min="20" max="20" width="22" customWidth="1"/>
+    <col min="21" max="21" width="22" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>ticker</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>close</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>ma25</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>ma75</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>ma200</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>ret5_pct</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>ret20_pct</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>ret60_pct</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>volume_ratio20</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>per</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>pbr</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>eps</t>
+        </is>
+      </c>
+      <c r="M1" t="inlineStr">
+        <is>
+          <t>max_drawdown20_pct</t>
+        </is>
+      </c>
+      <c r="N1" t="inlineStr">
+        <is>
+          <t>volatility20_pct</t>
+        </is>
+      </c>
+      <c r="O1" t="inlineStr">
+        <is>
+          <t>trend_calc</t>
+        </is>
+      </c>
+      <c r="P1" t="inlineStr">
+        <is>
+          <t>momentum_calc</t>
+        </is>
+      </c>
+      <c r="Q1" t="inlineStr">
+        <is>
+          <t>volume_calc</t>
+        </is>
+      </c>
+      <c r="R1" t="inlineStr">
+        <is>
+          <t>valuation_calc</t>
+        </is>
+      </c>
+      <c r="S1" t="inlineStr">
+        <is>
+          <t>fundamental_calc</t>
+        </is>
+      </c>
+      <c r="T1" t="inlineStr">
+        <is>
+          <t>risk_calc</t>
+        </is>
+      </c>
+      <c r="U1" t="inlineStr">
+        <is>
+          <t>total_check</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>8035.T</t>
+        </is>
+      </c>
+      <c r="B2">
+        <v>51200</v>
+      </c>
+      <c r="C2">
+        <v>45873.6</v>
+      </c>
+      <c r="D2">
+        <v>42674</v>
+      </c>
+      <c r="E2">
+        <v>34139.57</v>
+      </c>
+      <c r="F2">
+        <v>-1.01</v>
+      </c>
+      <c r="G2">
+        <v>16.26</v>
+      </c>
+      <c r="H2">
+        <v>23.37</v>
+      </c>
+      <c r="I2">
+        <v>0.61</v>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="K2">
+        <v>11.38</v>
+      </c>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="M2">
+        <v>-5.75</v>
+      </c>
+      <c r="N2">
+        <v>3.3</v>
+      </c>
+      <c r="O2">
+        <f>IF(B2&gt;=C2,6,0)+IF(B2&gt;=D2,7,0)+IF(B2&gt;=E2,7,0)</f>
+      </c>
+      <c r="P2">
+        <f>MAX(0,MIN(15,IF(F2&gt;0,4,0)+IF(G2&gt;0,5,0)+IF(H2&gt;0,6,0)-IF(G2&gt;15,3,0)))</f>
+      </c>
+      <c r="Q2">
+        <f>IF(I2&gt;=1.5,10,IF(I2&gt;=1.2,8,IF(I2&gt;=0.8,6,3)))</f>
+      </c>
+      <c r="R2">
+        <f>MIN(15,IF(J2="",0,IF(J2&lt;=15,8,IF(J2&lt;=25,6,IF(J2&lt;=40,3,1))))+IF(K2="",0,IF(K2&lt;=1.2,7,IF(K2&lt;=2,5,IF(K2&lt;=4,3,1)))))</f>
+      </c>
+      <c r="S2">
+        <f>IF(L2&gt;0,6,0)+IF(J2&lt;&gt;"",3,0)+IF(K2&lt;&gt;"",3,0)</f>
+      </c>
+      <c r="T2">
+        <f>MAX(0,10-IF(M2&lt;-10,4,0)-IF(M2&lt;-15,3,0)-IF(N2&gt;3.5,3,0)-IF(N2&gt;5,2,0))</f>
+      </c>
+      <c r="U2">
+        <f>O2+P2+Q2+R2+15+S2+T2</f>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>6857.T</t>
+        </is>
+      </c>
+      <c r="B3">
+        <v>28615</v>
+      </c>
+      <c r="C3">
+        <v>27438.2</v>
+      </c>
+      <c r="D3">
+        <v>25608.73</v>
+      </c>
+      <c r="E3">
+        <v>19856.25</v>
+      </c>
+      <c r="F3">
+        <v>-3.7</v>
+      </c>
+      <c r="G3">
+        <v>14.51</v>
+      </c>
+      <c r="H3">
+        <v>3.4</v>
+      </c>
+      <c r="I3">
+        <v>0.9</v>
+      </c>
+      <c r="J3">
+        <v>44.6</v>
+      </c>
+      <c r="K3">
+        <v>26.07</v>
+      </c>
+      <c r="L3">
+        <v>641.61</v>
+      </c>
+      <c r="M3">
+        <v>-11.7</v>
+      </c>
+      <c r="N3">
+        <v>3.99</v>
+      </c>
+      <c r="O3">
+        <f>IF(B3&gt;=C3,6,0)+IF(B3&gt;=D3,7,0)+IF(B3&gt;=E3,7,0)</f>
+      </c>
+      <c r="P3">
+        <f>MAX(0,MIN(15,IF(F3&gt;0,4,0)+IF(G3&gt;0,5,0)+IF(H3&gt;0,6,0)-IF(G3&gt;15,3,0)))</f>
+      </c>
+      <c r="Q3">
+        <f>IF(I3&gt;=1.5,10,IF(I3&gt;=1.2,8,IF(I3&gt;=0.8,6,3)))</f>
+      </c>
+      <c r="R3">
+        <f>MIN(15,IF(J3="",0,IF(J3&lt;=15,8,IF(J3&lt;=25,6,IF(J3&lt;=40,3,1))))+IF(K3="",0,IF(K3&lt;=1.2,7,IF(K3&lt;=2,5,IF(K3&lt;=4,3,1)))))</f>
+      </c>
+      <c r="S3">
+        <f>IF(L3&gt;0,6,0)+IF(J3&lt;&gt;"",3,0)+IF(K3&lt;&gt;"",3,0)</f>
+      </c>
+      <c r="T3">
+        <f>MAX(0,10-IF(M3&lt;-10,4,0)-IF(M3&lt;-15,3,0)-IF(N3&gt;3.5,3,0)-IF(N3&gt;5,2,0))</f>
+      </c>
+      <c r="U3">
+        <f>O3+P3+Q3+R3+15+S3+T3</f>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>4519.T</t>
+        </is>
+      </c>
+      <c r="B4">
+        <v>8096</v>
+      </c>
+      <c r="C4">
+        <v>8403.88</v>
+      </c>
+      <c r="D4">
+        <v>8880.21</v>
+      </c>
+      <c r="E4">
+        <v>7934.89</v>
+      </c>
+      <c r="F4">
+        <v>0.01</v>
+      </c>
+      <c r="G4">
+        <v>-6.67</v>
+      </c>
+      <c r="H4">
+        <v>-10.26</v>
+      </c>
+      <c r="I4">
+        <v>0.75</v>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="K4">
+        <v>6.98</v>
+      </c>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="M4">
+        <v>-16.59</v>
+      </c>
+      <c r="N4">
+        <v>4.49</v>
+      </c>
+      <c r="O4">
+        <f>IF(B4&gt;=C4,6,0)+IF(B4&gt;=D4,7,0)+IF(B4&gt;=E4,7,0)</f>
+      </c>
+      <c r="P4">
+        <f>MAX(0,MIN(15,IF(F4&gt;0,4,0)+IF(G4&gt;0,5,0)+IF(H4&gt;0,6,0)-IF(G4&gt;15,3,0)))</f>
+      </c>
+      <c r="Q4">
+        <f>IF(I4&gt;=1.5,10,IF(I4&gt;=1.2,8,IF(I4&gt;=0.8,6,3)))</f>
+      </c>
+      <c r="R4">
+        <f>MIN(15,IF(J4="",0,IF(J4&lt;=15,8,IF(J4&lt;=25,6,IF(J4&lt;=40,3,1))))+IF(K4="",0,IF(K4&lt;=1.2,7,IF(K4&lt;=2,5,IF(K4&lt;=4,3,1)))))</f>
+      </c>
+      <c r="S4">
+        <f>IF(L4&gt;0,6,0)+IF(J4&lt;&gt;"",3,0)+IF(K4&lt;&gt;"",3,0)</f>
+      </c>
+      <c r="T4">
+        <f>MAX(0,10-IF(M4&lt;-10,4,0)-IF(M4&lt;-15,3,0)-IF(N4&gt;3.5,3,0)-IF(N4&gt;5,2,0))</f>
+      </c>
+      <c r="U4">
+        <f>O4+P4+Q4+R4+15+S4+T4</f>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>8306.T</t>
+        </is>
+      </c>
+      <c r="B5">
+        <v>2877</v>
+      </c>
+      <c r="C5">
+        <v>2844.34</v>
+      </c>
+      <c r="D5">
+        <v>2812.37</v>
+      </c>
+      <c r="E5">
+        <v>2522.66</v>
+      </c>
+      <c r="F5">
+        <v>0.49</v>
+      </c>
+      <c r="G5">
+        <v>1.23</v>
+      </c>
+      <c r="H5">
+        <v>-5.17</v>
+      </c>
+      <c r="I5">
+        <v>0.96</v>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="K5">
+        <v>1.53</v>
+      </c>
+      <c r="L5" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="M5">
+        <v>-6.6</v>
+      </c>
+      <c r="N5">
+        <v>1.67</v>
+      </c>
+      <c r="O5">
+        <f>IF(B5&gt;=C5,6,0)+IF(B5&gt;=D5,7,0)+IF(B5&gt;=E5,7,0)</f>
+      </c>
+      <c r="P5">
+        <f>MAX(0,MIN(15,IF(F5&gt;0,4,0)+IF(G5&gt;0,5,0)+IF(H5&gt;0,6,0)-IF(G5&gt;15,3,0)))</f>
+      </c>
+      <c r="Q5">
+        <f>IF(I5&gt;=1.5,10,IF(I5&gt;=1.2,8,IF(I5&gt;=0.8,6,3)))</f>
+      </c>
+      <c r="R5">
+        <f>MIN(15,IF(J5="",0,IF(J5&lt;=15,8,IF(J5&lt;=25,6,IF(J5&lt;=40,3,1))))+IF(K5="",0,IF(K5&lt;=1.2,7,IF(K5&lt;=2,5,IF(K5&lt;=4,3,1)))))</f>
+      </c>
+      <c r="S5">
+        <f>IF(L5&gt;0,6,0)+IF(J5&lt;&gt;"",3,0)+IF(K5&lt;&gt;"",3,0)</f>
+      </c>
+      <c r="T5">
+        <f>MAX(0,10-IF(M5&lt;-10,4,0)-IF(M5&lt;-15,3,0)-IF(N5&gt;3.5,3,0)-IF(N5&gt;5,2,0))</f>
+      </c>
+      <c r="U5">
+        <f>O5+P5+Q5+R5+15+S5+T5</f>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>8058.T</t>
+        </is>
+      </c>
+      <c r="B6">
+        <v>5882</v>
+      </c>
+      <c r="C6">
+        <v>5192</v>
+      </c>
+      <c r="D6">
+        <v>5037.77</v>
+      </c>
+      <c r="E6">
+        <v>4075.95</v>
+      </c>
+      <c r="F6">
+        <v>8.97</v>
+      </c>
+      <c r="G6">
+        <v>10.83</v>
+      </c>
+      <c r="H6">
+        <v>14.5</v>
+      </c>
+      <c r="I6">
+        <v>0.71</v>
+      </c>
+      <c r="J6">
+        <v>19.58</v>
+      </c>
+      <c r="K6">
+        <v>2.28</v>
+      </c>
+      <c r="L6">
+        <v>300.42</v>
+      </c>
+      <c r="M6">
+        <v>-10.03</v>
+      </c>
+      <c r="N6">
+        <v>2.92</v>
+      </c>
+      <c r="O6">
+        <f>IF(B6&gt;=C6,6,0)+IF(B6&gt;=D6,7,0)+IF(B6&gt;=E6,7,0)</f>
+      </c>
+      <c r="P6">
+        <f>MAX(0,MIN(15,IF(F6&gt;0,4,0)+IF(G6&gt;0,5,0)+IF(H6&gt;0,6,0)-IF(G6&gt;15,3,0)))</f>
+      </c>
+      <c r="Q6">
+        <f>IF(I6&gt;=1.5,10,IF(I6&gt;=1.2,8,IF(I6&gt;=0.8,6,3)))</f>
+      </c>
+      <c r="R6">
+        <f>MIN(15,IF(J6="",0,IF(J6&lt;=15,8,IF(J6&lt;=25,6,IF(J6&lt;=40,3,1))))+IF(K6="",0,IF(K6&lt;=1.2,7,IF(K6&lt;=2,5,IF(K6&lt;=4,3,1)))))</f>
+      </c>
+      <c r="S6">
+        <f>IF(L6&gt;0,6,0)+IF(J6&lt;&gt;"",3,0)+IF(K6&lt;&gt;"",3,0)</f>
+      </c>
+      <c r="T6">
+        <f>MAX(0,10-IF(M6&lt;-10,4,0)-IF(M6&lt;-15,3,0)-IF(N6&gt;3.5,3,0)-IF(N6&gt;5,2,0))</f>
+      </c>
+      <c r="U6">
+        <f>O6+P6+Q6+R6+15+S6+T6</f>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>7974.T</t>
+        </is>
+      </c>
+      <c r="B7">
+        <v>6864</v>
+      </c>
+      <c r="C7">
+        <v>8030.04</v>
+      </c>
+      <c r="D7">
+        <v>8814.31</v>
+      </c>
+      <c r="E7">
+        <v>11235.42</v>
+      </c>
+      <c r="F7">
+        <v>-7.29</v>
+      </c>
+      <c r="G7">
+        <v>-17.3</v>
+      </c>
+      <c r="H7">
+        <v>-23.14</v>
+      </c>
+      <c r="I7">
+        <v>1.36</v>
+      </c>
+      <c r="J7">
+        <v>25.53</v>
+      </c>
+      <c r="K7">
+        <v>2.68</v>
+      </c>
+      <c r="L7">
+        <v>268.9</v>
+      </c>
+      <c r="M7">
+        <v>-20.33</v>
+      </c>
+      <c r="N7">
+        <v>2.7</v>
+      </c>
+      <c r="O7">
+        <f>IF(B7&gt;=C7,6,0)+IF(B7&gt;=D7,7,0)+IF(B7&gt;=E7,7,0)</f>
+      </c>
+      <c r="P7">
+        <f>MAX(0,MIN(15,IF(F7&gt;0,4,0)+IF(G7&gt;0,5,0)+IF(H7&gt;0,6,0)-IF(G7&gt;15,3,0)))</f>
+      </c>
+      <c r="Q7">
+        <f>IF(I7&gt;=1.5,10,IF(I7&gt;=1.2,8,IF(I7&gt;=0.8,6,3)))</f>
+      </c>
+      <c r="R7">
+        <f>MIN(15,IF(J7="",0,IF(J7&lt;=15,8,IF(J7&lt;=25,6,IF(J7&lt;=40,3,1))))+IF(K7="",0,IF(K7&lt;=1.2,7,IF(K7&lt;=2,5,IF(K7&lt;=4,3,1)))))</f>
+      </c>
+      <c r="S7">
+        <f>IF(L7&gt;0,6,0)+IF(J7&lt;&gt;"",3,0)+IF(K7&lt;&gt;"",3,0)</f>
+      </c>
+      <c r="T7">
+        <f>MAX(0,10-IF(M7&lt;-10,4,0)-IF(M7&lt;-15,3,0)-IF(N7&gt;3.5,3,0)-IF(N7&gt;5,2,0))</f>
+      </c>
+      <c r="U7">
+        <f>O7+P7+Q7+R7+15+S7+T7</f>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>9433.T</t>
+        </is>
+      </c>
+      <c r="B8">
+        <v>2645.5</v>
+      </c>
+      <c r="C8">
+        <v>2604.04</v>
+      </c>
+      <c r="D8">
+        <v>2647.67</v>
+      </c>
+      <c r="E8">
+        <v>2593.13</v>
+      </c>
+      <c r="F8">
+        <v>4.77</v>
+      </c>
+      <c r="G8">
+        <v>2.46</v>
+      </c>
+      <c r="H8">
+        <v>2.54</v>
+      </c>
+      <c r="I8">
+        <v>1.2</v>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="K8">
+        <v>1.98</v>
+      </c>
+      <c r="L8" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="M8">
+        <v>-4.4</v>
+      </c>
+      <c r="N8">
+        <v>1.4</v>
+      </c>
+      <c r="O8">
+        <f>IF(B8&gt;=C8,6,0)+IF(B8&gt;=D8,7,0)+IF(B8&gt;=E8,7,0)</f>
+      </c>
+      <c r="P8">
+        <f>MAX(0,MIN(15,IF(F8&gt;0,4,0)+IF(G8&gt;0,5,0)+IF(H8&gt;0,6,0)-IF(G8&gt;15,3,0)))</f>
+      </c>
+      <c r="Q8">
+        <f>IF(I8&gt;=1.5,10,IF(I8&gt;=1.2,8,IF(I8&gt;=0.8,6,3)))</f>
+      </c>
+      <c r="R8">
+        <f>MIN(15,IF(J8="",0,IF(J8&lt;=15,8,IF(J8&lt;=25,6,IF(J8&lt;=40,3,1))))+IF(K8="",0,IF(K8&lt;=1.2,7,IF(K8&lt;=2,5,IF(K8&lt;=4,3,1)))))</f>
+      </c>
+      <c r="S8">
+        <f>IF(L8&gt;0,6,0)+IF(J8&lt;&gt;"",3,0)+IF(K8&lt;&gt;"",3,0)</f>
+      </c>
+      <c r="T8">
+        <f>MAX(0,10-IF(M8&lt;-10,4,0)-IF(M8&lt;-15,3,0)-IF(N8&gt;3.5,3,0)-IF(N8&gt;5,2,0))</f>
+      </c>
+      <c r="U8">
+        <f>O8+P8+Q8+R8+15+S8+T8</f>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>2802.T</t>
+        </is>
+      </c>
+      <c r="B9">
+        <v>5542</v>
+      </c>
+      <c r="C9">
+        <v>4854.44</v>
+      </c>
+      <c r="D9">
+        <v>4477.05</v>
+      </c>
+      <c r="E9">
+        <v>4107.9</v>
+      </c>
+      <c r="F9">
+        <v>11.78</v>
+      </c>
+      <c r="G9">
+        <v>19.13</v>
+      </c>
+      <c r="H9">
+        <v>28.73</v>
+      </c>
+      <c r="I9">
+        <v>1.21</v>
+      </c>
+      <c r="J9">
+        <v>44.27</v>
+      </c>
+      <c r="K9">
+        <v>6.89</v>
+      </c>
+      <c r="L9">
+        <v>125.2</v>
+      </c>
+      <c r="M9">
+        <v>-4.09</v>
+      </c>
+      <c r="N9">
+        <v>2.99</v>
+      </c>
+      <c r="O9">
+        <f>IF(B9&gt;=C9,6,0)+IF(B9&gt;=D9,7,0)+IF(B9&gt;=E9,7,0)</f>
+      </c>
+      <c r="P9">
+        <f>MAX(0,MIN(15,IF(F9&gt;0,4,0)+IF(G9&gt;0,5,0)+IF(H9&gt;0,6,0)-IF(G9&gt;15,3,0)))</f>
+      </c>
+      <c r="Q9">
+        <f>IF(I9&gt;=1.5,10,IF(I9&gt;=1.2,8,IF(I9&gt;=0.8,6,3)))</f>
+      </c>
+      <c r="R9">
+        <f>MIN(15,IF(J9="",0,IF(J9&lt;=15,8,IF(J9&lt;=25,6,IF(J9&lt;=40,3,1))))+IF(K9="",0,IF(K9&lt;=1.2,7,IF(K9&lt;=2,5,IF(K9&lt;=4,3,1)))))</f>
+      </c>
+      <c r="S9">
+        <f>IF(L9&gt;0,6,0)+IF(J9&lt;&gt;"",3,0)+IF(K9&lt;&gt;"",3,0)</f>
+      </c>
+      <c r="T9">
+        <f>MAX(0,10-IF(M9&lt;-10,4,0)-IF(M9&lt;-15,3,0)-IF(N9&gt;3.5,3,0)-IF(N9&gt;5,2,0))</f>
+      </c>
+      <c r="U9">
+        <f>O9+P9+Q9+R9+15+S9+T9</f>
       </c>
     </row>
   </sheetData>
@@ -2600,7 +3790,7 @@
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>2026/05/14 20:52:36</t>
+          <t>2026/05/14 20:55:23</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
@@ -2642,7 +3832,7 @@
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>2026/05/14 20:52:36</t>
+          <t>2026/05/14 20:55:23</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
@@ -2684,7 +3874,7 @@
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>2026/05/14 20:52:36</t>
+          <t>2026/05/14 20:55:23</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
@@ -2726,7 +3916,7 @@
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>2026/05/14 20:52:36</t>
+          <t>2026/05/14 20:55:23</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
@@ -2768,7 +3958,7 @@
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>2026/05/14 20:52:36</t>
+          <t>2026/05/14 20:55:23</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
@@ -2810,7 +4000,7 @@
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>2026/05/14 20:52:36</t>
+          <t>2026/05/14 20:55:23</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
@@ -2852,7 +4042,7 @@
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>2026/05/14 20:52:36</t>
+          <t>2026/05/14 20:55:23</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
@@ -2894,7 +4084,7 @@
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>2026/05/14 20:52:36</t>
+          <t>2026/05/14 20:55:23</t>
         </is>
       </c>
       <c r="J9" t="inlineStr">
@@ -2994,7 +4184,7 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>2026/05/14 20:52:36</t>
+          <t>2026/05/14 20:55:23</t>
         </is>
       </c>
     </row>
@@ -3030,7 +4220,7 @@
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>2026/05/14 20:52:36</t>
+          <t>2026/05/14 20:55:23</t>
         </is>
       </c>
     </row>
@@ -3066,7 +4256,7 @@
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>2026/05/14 20:52:36</t>
+          <t>2026/05/14 20:55:23</t>
         </is>
       </c>
     </row>
@@ -3102,7 +4292,7 @@
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>2026/05/14 20:52:36</t>
+          <t>2026/05/14 20:55:23</t>
         </is>
       </c>
     </row>
@@ -3123,13 +4313,13 @@
         </is>
       </c>
       <c r="D6">
-        <v>157.9</v>
+        <v>157.92</v>
       </c>
       <c r="E6">
-        <v>0.89</v>
+        <v>0.9</v>
       </c>
       <c r="F6">
-        <v>-0.57</v>
+        <v>-0.56</v>
       </c>
       <c r="G6" t="inlineStr">
         <is>
@@ -3138,7 +4328,7 @@
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>2026/05/14 20:52:36</t>
+          <t>2026/05/14 20:55:23</t>
         </is>
       </c>
     </row>
@@ -3174,7 +4364,7 @@
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>2026/05/14 20:52:36</t>
+          <t>2026/05/14 20:55:23</t>
         </is>
       </c>
     </row>
@@ -3195,13 +4385,13 @@
         </is>
       </c>
       <c r="D8">
-        <v>17.88</v>
+        <v>17.87</v>
       </c>
       <c r="E8">
-        <v>4.68</v>
+        <v>4.63</v>
       </c>
       <c r="F8">
-        <v>-0.33</v>
+        <v>-0.39</v>
       </c>
       <c r="G8" t="inlineStr">
         <is>
@@ -3210,7 +4400,7 @@
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>2026/05/14 20:52:36</t>
+          <t>2026/05/14 20:55:23</t>
         </is>
       </c>
     </row>
@@ -3246,7 +4436,7 @@
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>2026/05/14 20:52:36</t>
+          <t>2026/05/14 20:55:23</t>
         </is>
       </c>
     </row>
@@ -3330,7 +4520,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026/05/14 20:52:36</t>
+          <t>2026/05/14 20:55:23</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -3385,7 +4575,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026/05/14 20:52:36</t>
+          <t>2026/05/14 20:55:23</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -3438,7 +4628,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2026/05/14 20:52:36</t>
+          <t>2026/05/14 20:55:23</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -3493,7 +4683,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026/05/14 20:52:36</t>
+          <t>2026/05/14 20:55:23</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -3548,7 +4738,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2026/05/14 20:52:36</t>
+          <t>2026/05/14 20:55:23</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -3601,7 +4791,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026/05/14 20:52:36</t>
+          <t>2026/05/14 20:55:23</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -3654,7 +4844,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>2026/05/14 20:52:36</t>
+          <t>2026/05/14 20:55:23</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -3709,7 +4899,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2026/05/14 20:52:36</t>
+          <t>2026/05/14 20:55:23</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -4584,7 +5774,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026/05/14 20:52:36</t>
+          <t>2026/05/14 20:55:23</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -4635,7 +5825,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026/05/14 20:52:36</t>
+          <t>2026/05/14 20:55:23</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -4686,7 +5876,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2026/05/14 20:52:36</t>
+          <t>2026/05/14 20:55:23</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -4737,7 +5927,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026/05/14 20:52:36</t>
+          <t>2026/05/14 20:55:23</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -4788,7 +5978,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2026/05/14 20:52:36</t>
+          <t>2026/05/14 20:55:23</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -4839,7 +6029,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026/05/14 20:52:36</t>
+          <t>2026/05/14 20:55:23</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -4890,7 +6080,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>2026/05/14 20:52:36</t>
+          <t>2026/05/14 20:55:23</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -4941,7 +6131,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2026/05/14 20:52:36</t>
+          <t>2026/05/14 20:55:23</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -5063,7 +6253,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026/05/14 20:52:36</t>
+          <t>2026/05/14 20:55:23</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">

</xml_diff>

<commit_message>
Add MVP score consistency check
</commit_message>
<xml_diff>
--- a/stock_decision_mvp_calculated.xlsx
+++ b/stock_decision_mvp_calculated.xlsx
@@ -45,6 +45,7 @@
     <sheet name="15_review_adjusted" sheetId="16" r:id="rId16"/>
     <sheet name="16_formula_spec" sheetId="17" r:id="rId17"/>
     <sheet name="17_excel_audit" sheetId="18" r:id="rId18"/>
+    <sheet name="18_consistency_check" sheetId="19" r:id="rId19"/>
   </sheets>
 </workbook>
 </file>
@@ -76,7 +77,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026/05/14 20:55:23</t>
+          <t>2026/05/14 20:57:14</t>
         </is>
       </c>
     </row>
@@ -254,7 +255,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026/05/14 20:55:23</t>
+          <t>2026/05/14 20:57:14</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -347,7 +348,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026/05/14 20:55:23</t>
+          <t>2026/05/14 20:57:14</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -397,7 +398,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026/05/14 20:55:23</t>
+          <t>2026/05/14 20:57:14</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -2225,6 +2226,262 @@
         </is>
       </c>
       <c r="F33" t="inlineStr">
+        <is>
+          <t>終値5542 / 20日騰落19.13% / 出来高倍率1.21 / PER44.27 / PBR6.89 / EPS125.2</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>2026/05/14 20:57:14</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>8035.T</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>60</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>様子見</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>価格・市場・一部財務で計算</t>
+        </is>
+      </c>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>終値51200 / 20日騰落16.26% / 出来高倍率0.61 / PER未取得 / PBR11.38 / EPS未取得</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>2026/05/14 20:57:14</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>6857.T</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>69</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>様子見</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>価格・市場・一部財務で計算</t>
+        </is>
+      </c>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>終値28615 / 20日騰落14.51% / 出来高倍率0.9 / PER44.6 / PBR26.07 / EPS641.61</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>2026/05/14 20:57:14</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>4519.T</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>33</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>除外/待機</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>価格・市場・一部財務で計算</t>
+        </is>
+      </c>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>終値8096 / 20日騰落-6.67% / 出来高倍率0.75 / PER未取得 / PBR6.98 / EPS未取得</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>2026/05/14 20:57:14</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>8306.T</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>68</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>様子見</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>価格・市場・一部財務で計算</t>
+        </is>
+      </c>
+      <c r="F37" t="inlineStr">
+        <is>
+          <t>終値2877 / 20日騰落1.23% / 出来高倍率0.96 / PER未取得 / PBR1.53 / EPS未取得</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>2026/05/14 20:57:14</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>8058.T</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>80</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>買い候補（決算要確認）</t>
+        </is>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>価格・市場・一部財務で計算</t>
+        </is>
+      </c>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>終値5882 / 20日騰落10.83% / 出来高倍率0.71 / PER19.58 / PBR2.28 / EPS300.42</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>2026/05/14 20:57:14</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>7974.T</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>44</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>除外/待機</t>
+        </is>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>価格・市場・一部財務で計算</t>
+        </is>
+      </c>
+      <c r="F39" t="inlineStr">
+        <is>
+          <t>終値6864 / 20日騰落-17.3% / 出来高倍率1.36 / PER25.53 / PBR2.68 / EPS268.9</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>2026/05/14 20:57:14</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>9433.T</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>67</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>様子見</t>
+        </is>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>価格・市場・一部財務で計算</t>
+        </is>
+      </c>
+      <c r="F40" t="inlineStr">
+        <is>
+          <t>終値2645.5 / 20日騰落2.46% / 出来高倍率1.2 / PER未取得 / PBR1.98 / EPS未取得</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>2026/05/14 20:57:14</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>2802.T</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>79</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>少額候補（決算要確認）</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>価格・市場・一部財務で計算</t>
+        </is>
+      </c>
+      <c r="F41" t="inlineStr">
         <is>
           <t>終値5542 / 20日騰落19.13% / 出来高倍率1.21 / PER44.27 / PBR6.89 / EPS125.2</t>
         </is>
@@ -2310,7 +2567,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026/05/14 20:55:23</t>
+          <t>2026/05/14 20:57:14</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -2359,7 +2616,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026/05/14 20:55:23</t>
+          <t>2026/05/14 20:57:14</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -3341,6 +3598,261 @@
 </worksheet>
 </file>
 
+<file path=xl\worksheets\sheet19.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <cols>
+    <col min="1" max="1" width="16" customWidth="1"/>
+    <col min="2" max="2" width="22" customWidth="1"/>
+    <col min="3" max="3" width="22" customWidth="1"/>
+    <col min="4" max="4" width="22" customWidth="1"/>
+    <col min="5" max="5" width="22" customWidth="1"/>
+    <col min="6" max="6" width="22" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>ticker</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>script_total_score</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>audit_total_score</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>difference</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>result</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>detail</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>8035.T</t>
+        </is>
+      </c>
+      <c r="B2">
+        <v>60</v>
+      </c>
+      <c r="C2">
+        <v>60</v>
+      </c>
+      <c r="D2">
+        <v>0</v>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>trend:20/20, momentum:8/8, volume:3/3, valuation:1/1, macro:15/15, fundamental:3/3, risk:10/10</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>6857.T</t>
+        </is>
+      </c>
+      <c r="B3">
+        <v>69</v>
+      </c>
+      <c r="C3">
+        <v>69</v>
+      </c>
+      <c r="D3">
+        <v>0</v>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>trend:20/20, momentum:11/11, volume:6/6, valuation:2/2, macro:15/15, fundamental:12/12, risk:3/3</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>4519.T</t>
+        </is>
+      </c>
+      <c r="B4">
+        <v>33</v>
+      </c>
+      <c r="C4">
+        <v>33</v>
+      </c>
+      <c r="D4">
+        <v>0</v>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>trend:7/7, momentum:4/4, volume:3/3, valuation:1/1, macro:15/15, fundamental:3/3, risk:0/0</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>8306.T</t>
+        </is>
+      </c>
+      <c r="B5">
+        <v>68</v>
+      </c>
+      <c r="C5">
+        <v>68</v>
+      </c>
+      <c r="D5">
+        <v>0</v>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>trend:20/20, momentum:9/9, volume:6/6, valuation:5/5, macro:15/15, fundamental:3/3, risk:10/10</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>8058.T</t>
+        </is>
+      </c>
+      <c r="B6">
+        <v>80</v>
+      </c>
+      <c r="C6">
+        <v>80</v>
+      </c>
+      <c r="D6">
+        <v>0</v>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>trend:20/20, momentum:15/15, volume:3/3, valuation:9/9, macro:15/15, fundamental:12/12, risk:6/6</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>7974.T</t>
+        </is>
+      </c>
+      <c r="B7">
+        <v>44</v>
+      </c>
+      <c r="C7">
+        <v>44</v>
+      </c>
+      <c r="D7">
+        <v>0</v>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>trend:0/0, momentum:0/0, volume:8/8, valuation:6/6, macro:15/15, fundamental:12/12, risk:3/3</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>9433.T</t>
+        </is>
+      </c>
+      <c r="B8">
+        <v>67</v>
+      </c>
+      <c r="C8">
+        <v>67</v>
+      </c>
+      <c r="D8">
+        <v>0</v>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>trend:13/13, momentum:15/15, volume:6/6, valuation:5/5, macro:15/15, fundamental:3/3, risk:10/10</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>2802.T</t>
+        </is>
+      </c>
+      <c r="B9">
+        <v>79</v>
+      </c>
+      <c r="C9">
+        <v>79</v>
+      </c>
+      <c r="D9">
+        <v>0</v>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>trend:20/20, momentum:12/12, volume:8/8, valuation:2/2, macro:15/15, fundamental:12/12, risk:10/10</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+</worksheet>
+</file>
+
 <file path=xl\worksheets\sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <cols>
@@ -3790,7 +4302,7 @@
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>2026/05/14 20:55:23</t>
+          <t>2026/05/14 20:57:14</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
@@ -3832,7 +4344,7 @@
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>2026/05/14 20:55:23</t>
+          <t>2026/05/14 20:57:14</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
@@ -3874,7 +4386,7 @@
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>2026/05/14 20:55:23</t>
+          <t>2026/05/14 20:57:14</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
@@ -3916,7 +4428,7 @@
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>2026/05/14 20:55:23</t>
+          <t>2026/05/14 20:57:14</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
@@ -3958,7 +4470,7 @@
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>2026/05/14 20:55:23</t>
+          <t>2026/05/14 20:57:14</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
@@ -4000,7 +4512,7 @@
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>2026/05/14 20:55:23</t>
+          <t>2026/05/14 20:57:14</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
@@ -4042,7 +4554,7 @@
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>2026/05/14 20:55:23</t>
+          <t>2026/05/14 20:57:14</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
@@ -4084,7 +4596,7 @@
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>2026/05/14 20:55:23</t>
+          <t>2026/05/14 20:57:14</t>
         </is>
       </c>
       <c r="J9" t="inlineStr">
@@ -4184,7 +4696,7 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>2026/05/14 20:55:23</t>
+          <t>2026/05/14 20:57:14</t>
         </is>
       </c>
     </row>
@@ -4220,7 +4732,7 @@
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>2026/05/14 20:55:23</t>
+          <t>2026/05/14 20:57:14</t>
         </is>
       </c>
     </row>
@@ -4256,7 +4768,7 @@
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>2026/05/14 20:55:23</t>
+          <t>2026/05/14 20:57:14</t>
         </is>
       </c>
     </row>
@@ -4292,7 +4804,7 @@
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>2026/05/14 20:55:23</t>
+          <t>2026/05/14 20:57:14</t>
         </is>
       </c>
     </row>
@@ -4313,13 +4825,13 @@
         </is>
       </c>
       <c r="D6">
-        <v>157.92</v>
+        <v>157.95</v>
       </c>
       <c r="E6">
-        <v>0.9</v>
+        <v>0.92</v>
       </c>
       <c r="F6">
-        <v>-0.56</v>
+        <v>-0.54</v>
       </c>
       <c r="G6" t="inlineStr">
         <is>
@@ -4328,7 +4840,7 @@
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>2026/05/14 20:55:23</t>
+          <t>2026/05/14 20:57:14</t>
         </is>
       </c>
     </row>
@@ -4364,7 +4876,7 @@
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>2026/05/14 20:55:23</t>
+          <t>2026/05/14 20:57:14</t>
         </is>
       </c>
     </row>
@@ -4400,7 +4912,7 @@
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>2026/05/14 20:55:23</t>
+          <t>2026/05/14 20:57:14</t>
         </is>
       </c>
     </row>
@@ -4436,7 +4948,7 @@
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>2026/05/14 20:55:23</t>
+          <t>2026/05/14 20:57:14</t>
         </is>
       </c>
     </row>
@@ -4520,7 +5032,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026/05/14 20:55:23</t>
+          <t>2026/05/14 20:57:14</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -4575,7 +5087,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026/05/14 20:55:23</t>
+          <t>2026/05/14 20:57:14</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -4628,7 +5140,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2026/05/14 20:55:23</t>
+          <t>2026/05/14 20:57:14</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -4683,7 +5195,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026/05/14 20:55:23</t>
+          <t>2026/05/14 20:57:14</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -4738,7 +5250,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2026/05/14 20:55:23</t>
+          <t>2026/05/14 20:57:14</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -4791,7 +5303,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026/05/14 20:55:23</t>
+          <t>2026/05/14 20:57:14</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -4844,7 +5356,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>2026/05/14 20:55:23</t>
+          <t>2026/05/14 20:57:14</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -4899,7 +5411,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2026/05/14 20:55:23</t>
+          <t>2026/05/14 20:57:14</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -5774,7 +6286,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026/05/14 20:55:23</t>
+          <t>2026/05/14 20:57:14</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -5825,7 +6337,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026/05/14 20:55:23</t>
+          <t>2026/05/14 20:57:14</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -5876,7 +6388,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2026/05/14 20:55:23</t>
+          <t>2026/05/14 20:57:14</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -5927,7 +6439,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026/05/14 20:55:23</t>
+          <t>2026/05/14 20:57:14</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -5978,7 +6490,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2026/05/14 20:55:23</t>
+          <t>2026/05/14 20:57:14</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -6029,7 +6541,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026/05/14 20:55:23</t>
+          <t>2026/05/14 20:57:14</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -6080,7 +6592,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>2026/05/14 20:55:23</t>
+          <t>2026/05/14 20:57:14</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -6131,7 +6643,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2026/05/14 20:55:23</t>
+          <t>2026/05/14 20:57:14</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -6253,7 +6765,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026/05/14 20:55:23</t>
+          <t>2026/05/14 20:57:14</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">

</xml_diff>

<commit_message>
Add MVP prediction actuals tracking
</commit_message>
<xml_diff>
--- a/stock_decision_mvp_calculated.xlsx
+++ b/stock_decision_mvp_calculated.xlsx
@@ -78,7 +78,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026/05/14 21:07:01</t>
+          <t>2026/05/14 21:24:24</t>
         </is>
       </c>
     </row>
@@ -158,52 +158,1148 @@
     <col min="7" max="7" width="22" customWidth="1"/>
     <col min="8" max="8" width="22" customWidth="1"/>
     <col min="9" max="9" width="22" customWidth="1"/>
+    <col min="10" max="10" width="22" customWidth="1"/>
+    <col min="11" max="11" width="22" customWidth="1"/>
+    <col min="12" max="12" width="22" customWidth="1"/>
+    <col min="13" max="13" width="22" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
+          <t>prediction_id</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
           <t>prediction_date</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>ticker</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>predicted_direction</t>
-        </is>
-      </c>
       <c r="D1" t="inlineStr">
         <is>
-          <t>actual_return_1d_pct</t>
+          <t>score</t>
         </is>
       </c>
       <c r="E1" t="inlineStr">
         <is>
-          <t>actual_return_5d_pct</t>
+          <t>decision</t>
         </is>
       </c>
       <c r="F1" t="inlineStr">
         <is>
-          <t>error_type</t>
+          <t>entry_close</t>
         </is>
       </c>
       <c r="G1" t="inlineStr">
         <is>
-          <t>reason_category</t>
+          <t>latest_close</t>
         </is>
       </c>
       <c r="H1" t="inlineStr">
         <is>
-          <t>lesson</t>
+          <t>return_pct</t>
         </is>
       </c>
       <c r="I1" t="inlineStr">
         <is>
-          <t>model_change_needed</t>
+          <t>check_type</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>check_date</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>status</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>result</t>
+        </is>
+      </c>
+      <c r="M1" t="inlineStr">
+        <is>
+          <t>note</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>2026-05-14_8035.T</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>2026/05/14 21:07:01</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>8035.T</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>60</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>様子見</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>51200</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>1d</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>2026-05-15</t>
+        </is>
+      </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>未到来</t>
+        </is>
+      </c>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>未検証</t>
+        </is>
+      </c>
+      <c r="M2" t="inlineStr">
+        <is>
+          <t>2026-05-15以降に評価</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>2026-05-14_8035.T</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>2026/05/14 21:07:01</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>8035.T</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>60</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>様子見</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>51200</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>5d</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>2026-05-19</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>未到来</t>
+        </is>
+      </c>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>未検証</t>
+        </is>
+      </c>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>2026-05-19以降に評価</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>2026-05-14_6857.T</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>2026/05/14 21:07:01</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>6857.T</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>69</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>様子見</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>28615</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>1d</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>2026-05-15</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>未到来</t>
+        </is>
+      </c>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>未検証</t>
+        </is>
+      </c>
+      <c r="M4" t="inlineStr">
+        <is>
+          <t>2026-05-15以降に評価</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>2026-05-14_6857.T</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>2026/05/14 21:07:01</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>6857.T</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>69</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>様子見</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>28615</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>5d</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>2026-05-19</t>
+        </is>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>未到来</t>
+        </is>
+      </c>
+      <c r="L5" t="inlineStr">
+        <is>
+          <t>未検証</t>
+        </is>
+      </c>
+      <c r="M5" t="inlineStr">
+        <is>
+          <t>2026-05-19以降に評価</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>2026-05-14_4519.T</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>2026/05/14 21:07:01</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>4519.T</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>33</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>除外/待機</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>8096</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>1d</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>2026-05-15</t>
+        </is>
+      </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>未到来</t>
+        </is>
+      </c>
+      <c r="L6" t="inlineStr">
+        <is>
+          <t>未検証</t>
+        </is>
+      </c>
+      <c r="M6" t="inlineStr">
+        <is>
+          <t>2026-05-15以降に評価</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>2026-05-14_4519.T</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>2026/05/14 21:07:01</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>4519.T</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>33</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>除外/待機</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>8096</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>5d</t>
+        </is>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>2026-05-19</t>
+        </is>
+      </c>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>未到来</t>
+        </is>
+      </c>
+      <c r="L7" t="inlineStr">
+        <is>
+          <t>未検証</t>
+        </is>
+      </c>
+      <c r="M7" t="inlineStr">
+        <is>
+          <t>2026-05-19以降に評価</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>2026-05-14_8306.T</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>2026/05/14 21:07:01</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>8306.T</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>68</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>様子見</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>2877</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>1d</t>
+        </is>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>2026-05-15</t>
+        </is>
+      </c>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>未到来</t>
+        </is>
+      </c>
+      <c r="L8" t="inlineStr">
+        <is>
+          <t>未検証</t>
+        </is>
+      </c>
+      <c r="M8" t="inlineStr">
+        <is>
+          <t>2026-05-15以降に評価</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>2026-05-14_8306.T</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>2026/05/14 21:07:01</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>8306.T</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>68</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>様子見</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>2877</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>5d</t>
+        </is>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>2026-05-19</t>
+        </is>
+      </c>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>未到来</t>
+        </is>
+      </c>
+      <c r="L9" t="inlineStr">
+        <is>
+          <t>未検証</t>
+        </is>
+      </c>
+      <c r="M9" t="inlineStr">
+        <is>
+          <t>2026-05-19以降に評価</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>2026-05-14_8058.T</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>2026/05/14 21:07:01</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>8058.T</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>80</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>買い候補（決算要確認）</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>5882</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>1d</t>
+        </is>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>2026-05-15</t>
+        </is>
+      </c>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t>未到来</t>
+        </is>
+      </c>
+      <c r="L10" t="inlineStr">
+        <is>
+          <t>未検証</t>
+        </is>
+      </c>
+      <c r="M10" t="inlineStr">
+        <is>
+          <t>2026-05-15以降に評価</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>2026-05-14_8058.T</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>2026/05/14 21:07:01</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>8058.T</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>80</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>買い候補（決算要確認）</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>5882</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>5d</t>
+        </is>
+      </c>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>2026-05-19</t>
+        </is>
+      </c>
+      <c r="K11" t="inlineStr">
+        <is>
+          <t>未到来</t>
+        </is>
+      </c>
+      <c r="L11" t="inlineStr">
+        <is>
+          <t>未検証</t>
+        </is>
+      </c>
+      <c r="M11" t="inlineStr">
+        <is>
+          <t>2026-05-19以降に評価</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>2026-05-14_7974.T</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>2026/05/14 21:07:01</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>7974.T</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>44</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>除外/待機</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>6864</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>1d</t>
+        </is>
+      </c>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>2026-05-15</t>
+        </is>
+      </c>
+      <c r="K12" t="inlineStr">
+        <is>
+          <t>未到来</t>
+        </is>
+      </c>
+      <c r="L12" t="inlineStr">
+        <is>
+          <t>未検証</t>
+        </is>
+      </c>
+      <c r="M12" t="inlineStr">
+        <is>
+          <t>2026-05-15以降に評価</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>2026-05-14_7974.T</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>2026/05/14 21:07:01</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>7974.T</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>44</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>除外/待機</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>6864</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>5d</t>
+        </is>
+      </c>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>2026-05-19</t>
+        </is>
+      </c>
+      <c r="K13" t="inlineStr">
+        <is>
+          <t>未到来</t>
+        </is>
+      </c>
+      <c r="L13" t="inlineStr">
+        <is>
+          <t>未検証</t>
+        </is>
+      </c>
+      <c r="M13" t="inlineStr">
+        <is>
+          <t>2026-05-19以降に評価</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>2026-05-14_9433.T</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>2026/05/14 21:07:01</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>9433.T</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>67</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>様子見</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>2645.5</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>1d</t>
+        </is>
+      </c>
+      <c r="J14" t="inlineStr">
+        <is>
+          <t>2026-05-15</t>
+        </is>
+      </c>
+      <c r="K14" t="inlineStr">
+        <is>
+          <t>未到来</t>
+        </is>
+      </c>
+      <c r="L14" t="inlineStr">
+        <is>
+          <t>未検証</t>
+        </is>
+      </c>
+      <c r="M14" t="inlineStr">
+        <is>
+          <t>2026-05-15以降に評価</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>2026-05-14_9433.T</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>2026/05/14 21:07:01</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>9433.T</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>67</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>様子見</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>2645.5</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>5d</t>
+        </is>
+      </c>
+      <c r="J15" t="inlineStr">
+        <is>
+          <t>2026-05-19</t>
+        </is>
+      </c>
+      <c r="K15" t="inlineStr">
+        <is>
+          <t>未到来</t>
+        </is>
+      </c>
+      <c r="L15" t="inlineStr">
+        <is>
+          <t>未検証</t>
+        </is>
+      </c>
+      <c r="M15" t="inlineStr">
+        <is>
+          <t>2026-05-19以降に評価</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>2026-05-14_2802.T</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>2026/05/14 21:07:01</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>2802.T</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>79</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>少額候補（決算要確認）</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>5542</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>1d</t>
+        </is>
+      </c>
+      <c r="J16" t="inlineStr">
+        <is>
+          <t>2026-05-15</t>
+        </is>
+      </c>
+      <c r="K16" t="inlineStr">
+        <is>
+          <t>未到来</t>
+        </is>
+      </c>
+      <c r="L16" t="inlineStr">
+        <is>
+          <t>未検証</t>
+        </is>
+      </c>
+      <c r="M16" t="inlineStr">
+        <is>
+          <t>2026-05-15以降に評価</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>2026-05-14_2802.T</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>2026/05/14 21:07:01</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>2802.T</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>79</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>少額候補（決算要確認）</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>5542</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>5d</t>
+        </is>
+      </c>
+      <c r="J17" t="inlineStr">
+        <is>
+          <t>2026-05-19</t>
+        </is>
+      </c>
+      <c r="K17" t="inlineStr">
+        <is>
+          <t>未到来</t>
+        </is>
+      </c>
+      <c r="L17" t="inlineStr">
+        <is>
+          <t>未検証</t>
+        </is>
+      </c>
+      <c r="M17" t="inlineStr">
+        <is>
+          <t>2026-05-19以降に評価</t>
         </is>
       </c>
     </row>
@@ -740,6 +1836,462 @@
         </is>
       </c>
     </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>2026-05-14_8035.T</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>2026/05/14 21:24:24</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>8035.T</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>60</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>様子見</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>51200</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>横ばい/様子見</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>2026-05-15</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>2026-05-19</t>
+        </is>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>未検証</t>
+        </is>
+      </c>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t>終値51200 / 20日騰落16.26% / 出来高倍率0.61 / PER未取得 / PBR11.38 / EPS未取得</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>2026-05-14_6857.T</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>2026/05/14 21:24:24</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>6857.T</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>69</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>様子見</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>28615</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>横ばい/様子見</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>2026-05-15</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>2026-05-19</t>
+        </is>
+      </c>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>未検証</t>
+        </is>
+      </c>
+      <c r="K11" t="inlineStr">
+        <is>
+          <t>終値28615 / 20日騰落14.51% / 出来高倍率0.9 / PER44.6 / PBR26.07 / EPS641.61</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>2026-05-14_4519.T</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>2026/05/14 21:24:24</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>4519.T</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>33</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>除外/待機</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>8096</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>弱含み/待機</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>2026-05-15</t>
+        </is>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>2026-05-19</t>
+        </is>
+      </c>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>未検証</t>
+        </is>
+      </c>
+      <c r="K12" t="inlineStr">
+        <is>
+          <t>終値8096 / 20日騰落-6.67% / 出来高倍率0.75 / PER未取得 / PBR6.98 / EPS未取得</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>2026-05-14_8306.T</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>2026/05/14 21:24:24</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>8306.T</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>68</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>様子見</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>2877</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>横ばい/様子見</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>2026-05-15</t>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>2026-05-19</t>
+        </is>
+      </c>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>未検証</t>
+        </is>
+      </c>
+      <c r="K13" t="inlineStr">
+        <is>
+          <t>終値2877 / 20日騰落1.23% / 出来高倍率0.96 / PER未取得 / PBR1.53 / EPS未取得</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>2026-05-14_8058.T</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>2026/05/14 21:24:24</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>8058.T</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>80</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>買い候補（決算要確認）</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>5882</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>上昇/相対優位を期待</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>2026-05-15</t>
+        </is>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>2026-05-19</t>
+        </is>
+      </c>
+      <c r="J14" t="inlineStr">
+        <is>
+          <t>未検証</t>
+        </is>
+      </c>
+      <c r="K14" t="inlineStr">
+        <is>
+          <t>終値5882 / 20日騰落10.83% / 出来高倍率0.71 / PER19.58 / PBR2.28 / EPS300.42</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>2026-05-14_7974.T</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>2026/05/14 21:24:24</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>7974.T</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>44</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>除外/待機</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>6864</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>弱含み/待機</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>2026-05-15</t>
+        </is>
+      </c>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>2026-05-19</t>
+        </is>
+      </c>
+      <c r="J15" t="inlineStr">
+        <is>
+          <t>未検証</t>
+        </is>
+      </c>
+      <c r="K15" t="inlineStr">
+        <is>
+          <t>終値6864 / 20日騰落-17.3% / 出来高倍率1.36 / PER25.53 / PBR2.68 / EPS268.9</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>2026-05-14_9433.T</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>2026/05/14 21:24:24</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>9433.T</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>67</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>様子見</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>2645.5</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>横ばい/様子見</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>2026-05-15</t>
+        </is>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>2026-05-19</t>
+        </is>
+      </c>
+      <c r="J16" t="inlineStr">
+        <is>
+          <t>未検証</t>
+        </is>
+      </c>
+      <c r="K16" t="inlineStr">
+        <is>
+          <t>終値2645.5 / 20日騰落2.46% / 出来高倍率1.2 / PER未取得 / PBR1.98 / EPS未取得</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>2026-05-14_2802.T</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>2026/05/14 21:24:24</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>2802.T</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>79</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>少額候補（決算要確認）</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>5542</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>上昇/相対優位を期待</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>2026-05-15</t>
+        </is>
+      </c>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>2026-05-19</t>
+        </is>
+      </c>
+      <c r="J17" t="inlineStr">
+        <is>
+          <t>未検証</t>
+        </is>
+      </c>
+      <c r="K17" t="inlineStr">
+        <is>
+          <t>終値5542 / 20日騰落19.13% / 出来高倍率1.21 / PER44.27 / PBR6.89 / EPS125.2</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
 </worksheet>
 </file>
@@ -789,7 +2341,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026/05/14 21:07:01</t>
+          <t>2026/05/14 21:24:24</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -882,7 +2434,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026/05/14 21:07:01</t>
+          <t>2026/05/14 21:24:24</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -932,7 +2484,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026/05/14 21:07:01</t>
+          <t>2026/05/14 21:24:24</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -1140,7 +2692,7 @@
         </is>
       </c>
       <c r="E4">
-        <v>17.83</v>
+        <v>17.84</v>
       </c>
       <c r="F4" t="inlineStr">
         <is>
@@ -3272,6 +4824,262 @@
         </is>
       </c>
       <c r="F49" t="inlineStr">
+        <is>
+          <t>終値5542 / 20日騰落19.13% / 出来高倍率1.21 / PER44.27 / PBR6.89 / EPS125.2</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>2026/05/14 21:24:24</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>8035.T</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>60</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>様子見</t>
+        </is>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>価格・市場・一部財務で計算</t>
+        </is>
+      </c>
+      <c r="F50" t="inlineStr">
+        <is>
+          <t>終値51200 / 20日騰落16.26% / 出来高倍率0.61 / PER未取得 / PBR11.38 / EPS未取得</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>2026/05/14 21:24:24</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>6857.T</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>69</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>様子見</t>
+        </is>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>価格・市場・一部財務で計算</t>
+        </is>
+      </c>
+      <c r="F51" t="inlineStr">
+        <is>
+          <t>終値28615 / 20日騰落14.51% / 出来高倍率0.9 / PER44.6 / PBR26.07 / EPS641.61</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>2026/05/14 21:24:24</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>4519.T</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>33</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>除外/待機</t>
+        </is>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>価格・市場・一部財務で計算</t>
+        </is>
+      </c>
+      <c r="F52" t="inlineStr">
+        <is>
+          <t>終値8096 / 20日騰落-6.67% / 出来高倍率0.75 / PER未取得 / PBR6.98 / EPS未取得</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>2026/05/14 21:24:24</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>8306.T</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>68</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>様子見</t>
+        </is>
+      </c>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>価格・市場・一部財務で計算</t>
+        </is>
+      </c>
+      <c r="F53" t="inlineStr">
+        <is>
+          <t>終値2877 / 20日騰落1.23% / 出来高倍率0.96 / PER未取得 / PBR1.53 / EPS未取得</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>2026/05/14 21:24:24</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>8058.T</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>80</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>買い候補（決算要確認）</t>
+        </is>
+      </c>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>価格・市場・一部財務で計算</t>
+        </is>
+      </c>
+      <c r="F54" t="inlineStr">
+        <is>
+          <t>終値5882 / 20日騰落10.83% / 出来高倍率0.71 / PER19.58 / PBR2.28 / EPS300.42</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>2026/05/14 21:24:24</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>7974.T</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>44</t>
+        </is>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>除外/待機</t>
+        </is>
+      </c>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>価格・市場・一部財務で計算</t>
+        </is>
+      </c>
+      <c r="F55" t="inlineStr">
+        <is>
+          <t>終値6864 / 20日騰落-17.3% / 出来高倍率1.36 / PER25.53 / PBR2.68 / EPS268.9</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>2026/05/14 21:24:24</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>9433.T</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>67</t>
+        </is>
+      </c>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t>様子見</t>
+        </is>
+      </c>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>価格・市場・一部財務で計算</t>
+        </is>
+      </c>
+      <c r="F56" t="inlineStr">
+        <is>
+          <t>終値2645.5 / 20日騰落2.46% / 出来高倍率1.2 / PER未取得 / PBR1.98 / EPS未取得</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>2026/05/14 21:24:24</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>2802.T</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>79</t>
+        </is>
+      </c>
+      <c r="D57" t="inlineStr">
+        <is>
+          <t>少額候補（決算要確認）</t>
+        </is>
+      </c>
+      <c r="E57" t="inlineStr">
+        <is>
+          <t>価格・市場・一部財務で計算</t>
+        </is>
+      </c>
+      <c r="F57" t="inlineStr">
         <is>
           <t>終値5542 / 20日騰落19.13% / 出来高倍率1.21 / PER44.27 / PBR6.89 / EPS125.2</t>
         </is>
@@ -3357,7 +5165,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026/05/14 21:07:01</t>
+          <t>2026/05/14 21:24:24</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -3406,7 +5214,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026/05/14 21:07:01</t>
+          <t>2026/05/14 21:24:24</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -5092,7 +6900,7 @@
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>2026/05/14 21:07:01</t>
+          <t>2026/05/14 21:24:24</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
@@ -5134,7 +6942,7 @@
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>2026/05/14 21:07:01</t>
+          <t>2026/05/14 21:24:24</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
@@ -5176,7 +6984,7 @@
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>2026/05/14 21:07:01</t>
+          <t>2026/05/14 21:24:24</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
@@ -5218,7 +7026,7 @@
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>2026/05/14 21:07:01</t>
+          <t>2026/05/14 21:24:24</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
@@ -5260,7 +7068,7 @@
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>2026/05/14 21:07:01</t>
+          <t>2026/05/14 21:24:24</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
@@ -5302,7 +7110,7 @@
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>2026/05/14 21:07:01</t>
+          <t>2026/05/14 21:24:24</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
@@ -5344,7 +7152,7 @@
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>2026/05/14 21:07:01</t>
+          <t>2026/05/14 21:24:24</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
@@ -5386,7 +7194,7 @@
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>2026/05/14 21:07:01</t>
+          <t>2026/05/14 21:24:24</t>
         </is>
       </c>
       <c r="J9" t="inlineStr">
@@ -5486,7 +7294,7 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>2026/05/14 21:07:01</t>
+          <t>2026/05/14 21:24:24</t>
         </is>
       </c>
     </row>
@@ -5522,7 +7330,7 @@
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>2026/05/14 21:07:01</t>
+          <t>2026/05/14 21:24:24</t>
         </is>
       </c>
     </row>
@@ -5558,7 +7366,7 @@
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>2026/05/14 21:07:01</t>
+          <t>2026/05/14 21:24:24</t>
         </is>
       </c>
     </row>
@@ -5594,7 +7402,7 @@
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>2026/05/14 21:07:01</t>
+          <t>2026/05/14 21:24:24</t>
         </is>
       </c>
     </row>
@@ -5615,13 +7423,13 @@
         </is>
       </c>
       <c r="D6">
-        <v>157.91</v>
+        <v>157.9</v>
       </c>
       <c r="E6">
-        <v>0.9</v>
+        <v>0.89</v>
       </c>
       <c r="F6">
-        <v>-0.56</v>
+        <v>-0.57</v>
       </c>
       <c r="G6" t="inlineStr">
         <is>
@@ -5630,7 +7438,7 @@
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>2026/05/14 21:07:01</t>
+          <t>2026/05/14 21:24:24</t>
         </is>
       </c>
     </row>
@@ -5666,7 +7474,7 @@
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>2026/05/14 21:07:01</t>
+          <t>2026/05/14 21:24:24</t>
         </is>
       </c>
     </row>
@@ -5687,13 +7495,13 @@
         </is>
       </c>
       <c r="D8">
-        <v>17.83</v>
+        <v>17.84</v>
       </c>
       <c r="E8">
-        <v>4.39</v>
+        <v>4.45</v>
       </c>
       <c r="F8">
-        <v>-0.61</v>
+        <v>-0.56</v>
       </c>
       <c r="G8" t="inlineStr">
         <is>
@@ -5702,7 +7510,7 @@
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>2026/05/14 21:07:01</t>
+          <t>2026/05/14 21:24:24</t>
         </is>
       </c>
     </row>
@@ -5723,13 +7531,13 @@
         </is>
       </c>
       <c r="D9">
-        <v>98.57</v>
+        <v>98.55</v>
       </c>
       <c r="E9">
-        <v>0.32</v>
+        <v>0.3</v>
       </c>
       <c r="F9">
-        <v>0.35</v>
+        <v>0.33</v>
       </c>
       <c r="G9" t="inlineStr">
         <is>
@@ -5738,7 +7546,7 @@
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>2026/05/14 21:07:01</t>
+          <t>2026/05/14 21:24:24</t>
         </is>
       </c>
     </row>
@@ -5822,7 +7630,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026/05/14 21:07:01</t>
+          <t>2026/05/14 21:24:24</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -5877,7 +7685,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026/05/14 21:07:01</t>
+          <t>2026/05/14 21:24:24</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -5930,7 +7738,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2026/05/14 21:07:01</t>
+          <t>2026/05/14 21:24:24</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -5985,7 +7793,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026/05/14 21:07:01</t>
+          <t>2026/05/14 21:24:24</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -6040,7 +7848,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2026/05/14 21:07:01</t>
+          <t>2026/05/14 21:24:24</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -6093,7 +7901,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026/05/14 21:07:01</t>
+          <t>2026/05/14 21:24:24</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -6146,7 +7954,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>2026/05/14 21:07:01</t>
+          <t>2026/05/14 21:24:24</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -6201,7 +8009,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2026/05/14 21:07:01</t>
+          <t>2026/05/14 21:24:24</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -7076,7 +8884,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026/05/14 21:07:01</t>
+          <t>2026/05/14 21:24:24</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -7127,7 +8935,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026/05/14 21:07:01</t>
+          <t>2026/05/14 21:24:24</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -7178,7 +8986,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2026/05/14 21:07:01</t>
+          <t>2026/05/14 21:24:24</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -7229,7 +9037,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026/05/14 21:07:01</t>
+          <t>2026/05/14 21:24:24</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -7280,7 +9088,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2026/05/14 21:07:01</t>
+          <t>2026/05/14 21:24:24</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -7331,7 +9139,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026/05/14 21:07:01</t>
+          <t>2026/05/14 21:24:24</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -7382,7 +9190,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>2026/05/14 21:07:01</t>
+          <t>2026/05/14 21:24:24</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -7433,7 +9241,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2026/05/14 21:07:01</t>
+          <t>2026/05/14 21:24:24</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -7555,7 +9363,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026/05/14 21:07:01</t>
+          <t>2026/05/14 21:24:24</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">

</xml_diff>

<commit_message>
Evaluate first MVP prediction actuals
</commit_message>
<xml_diff>
--- a/stock_decision_mvp_calculated.xlsx
+++ b/stock_decision_mvp_calculated.xlsx
@@ -78,7 +78,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026/05/14 21:24:24</t>
+          <t>2026/05/15 10:55:11</t>
         </is>
       </c>
     </row>
@@ -239,7 +239,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026/05/14 21:07:01</t>
+          <t>2026/05/14 21:24:24</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -264,12 +264,12 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t/>
+          <t>51030</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t/>
+          <t>-0.33</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
@@ -284,17 +284,17 @@
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>未到来</t>
+          <t>評価済</t>
         </is>
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>未検証</t>
+          <t>方向一致</t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>2026-05-15以降に評価</t>
+          <t>横ばい/様子見</t>
         </is>
       </c>
     </row>
@@ -306,7 +306,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>2026/05/14 21:07:01</t>
+          <t>2026/05/14 21:24:24</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -373,7 +373,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>2026/05/14 21:07:01</t>
+          <t>2026/05/14 21:24:24</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -398,12 +398,12 @@
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t/>
+          <t>27535</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t/>
+          <t>-3.77</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
@@ -418,17 +418,17 @@
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>未到来</t>
+          <t>評価済</t>
         </is>
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>未検証</t>
+          <t>方向不一致</t>
         </is>
       </c>
       <c r="M4" t="inlineStr">
         <is>
-          <t>2026-05-15以降に評価</t>
+          <t>横ばい/様子見</t>
         </is>
       </c>
     </row>
@@ -440,7 +440,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>2026/05/14 21:07:01</t>
+          <t>2026/05/14 21:24:24</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -507,7 +507,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>2026/05/14 21:07:01</t>
+          <t>2026/05/14 21:24:24</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -532,12 +532,12 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t/>
+          <t>8014</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t/>
+          <t>-1.01</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
@@ -552,17 +552,17 @@
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>未到来</t>
+          <t>評価済</t>
         </is>
       </c>
       <c r="L6" t="inlineStr">
         <is>
-          <t>未検証</t>
+          <t>方向一致</t>
         </is>
       </c>
       <c r="M6" t="inlineStr">
         <is>
-          <t>2026-05-15以降に評価</t>
+          <t>弱含み/待機</t>
         </is>
       </c>
     </row>
@@ -574,7 +574,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>2026/05/14 21:07:01</t>
+          <t>2026/05/14 21:24:24</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -641,7 +641,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>2026/05/14 21:07:01</t>
+          <t>2026/05/14 21:24:24</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -666,12 +666,12 @@
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t/>
+          <t>2927.5</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t/>
+          <t>1.76</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
@@ -686,17 +686,17 @@
       </c>
       <c r="K8" t="inlineStr">
         <is>
-          <t>未到来</t>
+          <t>評価済</t>
         </is>
       </c>
       <c r="L8" t="inlineStr">
         <is>
-          <t>未検証</t>
+          <t>方向不一致</t>
         </is>
       </c>
       <c r="M8" t="inlineStr">
         <is>
-          <t>2026-05-15以降に評価</t>
+          <t>横ばい/様子見</t>
         </is>
       </c>
     </row>
@@ -708,7 +708,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>2026/05/14 21:07:01</t>
+          <t>2026/05/14 21:24:24</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -775,7 +775,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>2026/05/14 21:07:01</t>
+          <t>2026/05/14 21:24:24</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -800,12 +800,12 @@
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t/>
+          <t>5859</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t/>
+          <t>-0.39</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
@@ -820,17 +820,17 @@
       </c>
       <c r="K10" t="inlineStr">
         <is>
-          <t>未到来</t>
+          <t>評価済</t>
         </is>
       </c>
       <c r="L10" t="inlineStr">
         <is>
-          <t>未検証</t>
+          <t>方向不一致</t>
         </is>
       </c>
       <c r="M10" t="inlineStr">
         <is>
-          <t>2026-05-15以降に評価</t>
+          <t>上昇/相対優位を期待</t>
         </is>
       </c>
     </row>
@@ -842,7 +842,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>2026/05/14 21:07:01</t>
+          <t>2026/05/14 21:24:24</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -909,7 +909,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>2026/05/14 21:07:01</t>
+          <t>2026/05/14 21:24:24</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -934,12 +934,12 @@
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t/>
+          <t>6992</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t/>
+          <t>1.86</t>
         </is>
       </c>
       <c r="I12" t="inlineStr">
@@ -954,17 +954,17 @@
       </c>
       <c r="K12" t="inlineStr">
         <is>
-          <t>未到来</t>
+          <t>評価済</t>
         </is>
       </c>
       <c r="L12" t="inlineStr">
         <is>
-          <t>未検証</t>
+          <t>方向不一致</t>
         </is>
       </c>
       <c r="M12" t="inlineStr">
         <is>
-          <t>2026-05-15以降に評価</t>
+          <t>弱含み/待機</t>
         </is>
       </c>
     </row>
@@ -976,7 +976,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>2026/05/14 21:07:01</t>
+          <t>2026/05/14 21:24:24</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -1043,7 +1043,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>2026/05/14 21:07:01</t>
+          <t>2026/05/14 21:24:24</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -1068,12 +1068,12 @@
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t/>
+          <t>2653</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t/>
+          <t>0.28</t>
         </is>
       </c>
       <c r="I14" t="inlineStr">
@@ -1088,17 +1088,17 @@
       </c>
       <c r="K14" t="inlineStr">
         <is>
-          <t>未到来</t>
+          <t>評価済</t>
         </is>
       </c>
       <c r="L14" t="inlineStr">
         <is>
-          <t>未検証</t>
+          <t>方向一致</t>
         </is>
       </c>
       <c r="M14" t="inlineStr">
         <is>
-          <t>2026-05-15以降に評価</t>
+          <t>横ばい/様子見</t>
         </is>
       </c>
     </row>
@@ -1110,7 +1110,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>2026/05/14 21:07:01</t>
+          <t>2026/05/14 21:24:24</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -1177,7 +1177,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>2026/05/14 21:07:01</t>
+          <t>2026/05/14 21:24:24</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -1202,12 +1202,12 @@
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t/>
+          <t>5426</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t/>
+          <t>-2.09</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
@@ -1222,17 +1222,17 @@
       </c>
       <c r="K16" t="inlineStr">
         <is>
-          <t>未到来</t>
+          <t>評価済</t>
         </is>
       </c>
       <c r="L16" t="inlineStr">
         <is>
-          <t>未検証</t>
+          <t>方向不一致</t>
         </is>
       </c>
       <c r="M16" t="inlineStr">
         <is>
-          <t>2026-05-15以降に評価</t>
+          <t>上昇/相対優位を期待</t>
         </is>
       </c>
     </row>
@@ -1244,7 +1244,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>2026/05/14 21:07:01</t>
+          <t>2026/05/14 21:24:24</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -1300,6 +1300,1078 @@
       <c r="M17" t="inlineStr">
         <is>
           <t>2026-05-19以降に評価</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>2026-05-15_8035.T</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>2026/05/15 10:55:11</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>8035.T</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>60</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>様子見</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>51030</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>1d</t>
+        </is>
+      </c>
+      <c r="J18" t="inlineStr">
+        <is>
+          <t>2026-05-16</t>
+        </is>
+      </c>
+      <c r="K18" t="inlineStr">
+        <is>
+          <t>未到来</t>
+        </is>
+      </c>
+      <c r="L18" t="inlineStr">
+        <is>
+          <t>未検証</t>
+        </is>
+      </c>
+      <c r="M18" t="inlineStr">
+        <is>
+          <t>2026-05-16以降に評価</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>2026-05-15_8035.T</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>2026/05/15 10:55:11</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>8035.T</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>60</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>様子見</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>51030</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="I19" t="inlineStr">
+        <is>
+          <t>5d</t>
+        </is>
+      </c>
+      <c r="J19" t="inlineStr">
+        <is>
+          <t>2026-05-20</t>
+        </is>
+      </c>
+      <c r="K19" t="inlineStr">
+        <is>
+          <t>未到来</t>
+        </is>
+      </c>
+      <c r="L19" t="inlineStr">
+        <is>
+          <t>未検証</t>
+        </is>
+      </c>
+      <c r="M19" t="inlineStr">
+        <is>
+          <t>2026-05-20以降に評価</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>2026-05-15_6857.T</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>2026/05/15 10:55:11</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>6857.T</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>60</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>様子見</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>27535</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="I20" t="inlineStr">
+        <is>
+          <t>1d</t>
+        </is>
+      </c>
+      <c r="J20" t="inlineStr">
+        <is>
+          <t>2026-05-16</t>
+        </is>
+      </c>
+      <c r="K20" t="inlineStr">
+        <is>
+          <t>未到来</t>
+        </is>
+      </c>
+      <c r="L20" t="inlineStr">
+        <is>
+          <t>未検証</t>
+        </is>
+      </c>
+      <c r="M20" t="inlineStr">
+        <is>
+          <t>2026-05-16以降に評価</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>2026-05-15_6857.T</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>2026/05/15 10:55:11</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>6857.T</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>60</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>様子見</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>27535</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="I21" t="inlineStr">
+        <is>
+          <t>5d</t>
+        </is>
+      </c>
+      <c r="J21" t="inlineStr">
+        <is>
+          <t>2026-05-20</t>
+        </is>
+      </c>
+      <c r="K21" t="inlineStr">
+        <is>
+          <t>未到来</t>
+        </is>
+      </c>
+      <c r="L21" t="inlineStr">
+        <is>
+          <t>未検証</t>
+        </is>
+      </c>
+      <c r="M21" t="inlineStr">
+        <is>
+          <t>2026-05-20以降に評価</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>2026-05-15_4519.T</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>2026/05/15 10:55:11</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>4519.T</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>33</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>除外/待機</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>8014</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="I22" t="inlineStr">
+        <is>
+          <t>1d</t>
+        </is>
+      </c>
+      <c r="J22" t="inlineStr">
+        <is>
+          <t>2026-05-16</t>
+        </is>
+      </c>
+      <c r="K22" t="inlineStr">
+        <is>
+          <t>未到来</t>
+        </is>
+      </c>
+      <c r="L22" t="inlineStr">
+        <is>
+          <t>未検証</t>
+        </is>
+      </c>
+      <c r="M22" t="inlineStr">
+        <is>
+          <t>2026-05-16以降に評価</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>2026-05-15_4519.T</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>2026/05/15 10:55:11</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>4519.T</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>33</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>除外/待機</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>8014</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="I23" t="inlineStr">
+        <is>
+          <t>5d</t>
+        </is>
+      </c>
+      <c r="J23" t="inlineStr">
+        <is>
+          <t>2026-05-20</t>
+        </is>
+      </c>
+      <c r="K23" t="inlineStr">
+        <is>
+          <t>未到来</t>
+        </is>
+      </c>
+      <c r="L23" t="inlineStr">
+        <is>
+          <t>未検証</t>
+        </is>
+      </c>
+      <c r="M23" t="inlineStr">
+        <is>
+          <t>2026-05-20以降に評価</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>2026-05-15_8306.T</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>2026/05/15 10:55:11</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>8306.T</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>65</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>様子見</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>2927.5</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="I24" t="inlineStr">
+        <is>
+          <t>1d</t>
+        </is>
+      </c>
+      <c r="J24" t="inlineStr">
+        <is>
+          <t>2026-05-16</t>
+        </is>
+      </c>
+      <c r="K24" t="inlineStr">
+        <is>
+          <t>未到来</t>
+        </is>
+      </c>
+      <c r="L24" t="inlineStr">
+        <is>
+          <t>未検証</t>
+        </is>
+      </c>
+      <c r="M24" t="inlineStr">
+        <is>
+          <t>2026-05-16以降に評価</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>2026-05-15_8306.T</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>2026/05/15 10:55:11</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>8306.T</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>65</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>様子見</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>2927.5</t>
+        </is>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="I25" t="inlineStr">
+        <is>
+          <t>5d</t>
+        </is>
+      </c>
+      <c r="J25" t="inlineStr">
+        <is>
+          <t>2026-05-20</t>
+        </is>
+      </c>
+      <c r="K25" t="inlineStr">
+        <is>
+          <t>未到来</t>
+        </is>
+      </c>
+      <c r="L25" t="inlineStr">
+        <is>
+          <t>未検証</t>
+        </is>
+      </c>
+      <c r="M25" t="inlineStr">
+        <is>
+          <t>2026-05-20以降に評価</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>2026-05-15_8058.T</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>2026/05/15 10:55:11</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>8058.T</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>84</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>買い候補（決算要確認）</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>5859</t>
+        </is>
+      </c>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="H26" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="I26" t="inlineStr">
+        <is>
+          <t>1d</t>
+        </is>
+      </c>
+      <c r="J26" t="inlineStr">
+        <is>
+          <t>2026-05-16</t>
+        </is>
+      </c>
+      <c r="K26" t="inlineStr">
+        <is>
+          <t>未到来</t>
+        </is>
+      </c>
+      <c r="L26" t="inlineStr">
+        <is>
+          <t>未検証</t>
+        </is>
+      </c>
+      <c r="M26" t="inlineStr">
+        <is>
+          <t>2026-05-16以降に評価</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>2026-05-15_8058.T</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>2026/05/15 10:55:11</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>8058.T</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>84</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>買い候補（決算要確認）</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>5859</t>
+        </is>
+      </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="H27" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="I27" t="inlineStr">
+        <is>
+          <t>5d</t>
+        </is>
+      </c>
+      <c r="J27" t="inlineStr">
+        <is>
+          <t>2026-05-20</t>
+        </is>
+      </c>
+      <c r="K27" t="inlineStr">
+        <is>
+          <t>未到来</t>
+        </is>
+      </c>
+      <c r="L27" t="inlineStr">
+        <is>
+          <t>未検証</t>
+        </is>
+      </c>
+      <c r="M27" t="inlineStr">
+        <is>
+          <t>2026-05-20以降に評価</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>2026-05-15_7974.T</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>2026/05/15 10:55:11</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>7974.T</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>39</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>除外/待機</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>6992</t>
+        </is>
+      </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="H28" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="I28" t="inlineStr">
+        <is>
+          <t>1d</t>
+        </is>
+      </c>
+      <c r="J28" t="inlineStr">
+        <is>
+          <t>2026-05-16</t>
+        </is>
+      </c>
+      <c r="K28" t="inlineStr">
+        <is>
+          <t>未到来</t>
+        </is>
+      </c>
+      <c r="L28" t="inlineStr">
+        <is>
+          <t>未検証</t>
+        </is>
+      </c>
+      <c r="M28" t="inlineStr">
+        <is>
+          <t>2026-05-16以降に評価</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>2026-05-15_7974.T</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>2026/05/15 10:55:11</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>7974.T</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>39</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>除外/待機</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>6992</t>
+        </is>
+      </c>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="H29" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="I29" t="inlineStr">
+        <is>
+          <t>5d</t>
+        </is>
+      </c>
+      <c r="J29" t="inlineStr">
+        <is>
+          <t>2026-05-20</t>
+        </is>
+      </c>
+      <c r="K29" t="inlineStr">
+        <is>
+          <t>未到来</t>
+        </is>
+      </c>
+      <c r="L29" t="inlineStr">
+        <is>
+          <t>未検証</t>
+        </is>
+      </c>
+      <c r="M29" t="inlineStr">
+        <is>
+          <t>2026-05-20以降に評価</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>2026-05-15_9433.T</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>2026/05/15 10:55:11</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>9433.T</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>65</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>様子見</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>2653</t>
+        </is>
+      </c>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="H30" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="I30" t="inlineStr">
+        <is>
+          <t>1d</t>
+        </is>
+      </c>
+      <c r="J30" t="inlineStr">
+        <is>
+          <t>2026-05-16</t>
+        </is>
+      </c>
+      <c r="K30" t="inlineStr">
+        <is>
+          <t>未到来</t>
+        </is>
+      </c>
+      <c r="L30" t="inlineStr">
+        <is>
+          <t>未検証</t>
+        </is>
+      </c>
+      <c r="M30" t="inlineStr">
+        <is>
+          <t>2026-05-16以降に評価</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>2026-05-15_9433.T</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>2026/05/15 10:55:11</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>9433.T</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>65</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>様子見</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>2653</t>
+        </is>
+      </c>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="H31" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="I31" t="inlineStr">
+        <is>
+          <t>5d</t>
+        </is>
+      </c>
+      <c r="J31" t="inlineStr">
+        <is>
+          <t>2026-05-20</t>
+        </is>
+      </c>
+      <c r="K31" t="inlineStr">
+        <is>
+          <t>未到来</t>
+        </is>
+      </c>
+      <c r="L31" t="inlineStr">
+        <is>
+          <t>未検証</t>
+        </is>
+      </c>
+      <c r="M31" t="inlineStr">
+        <is>
+          <t>2026-05-20以降に評価</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>2026-05-15_2802.T</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>2026/05/15 10:55:11</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>2802.T</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>74</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>少額候補（決算要確認）</t>
+        </is>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>5426</t>
+        </is>
+      </c>
+      <c r="G32" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="H32" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="I32" t="inlineStr">
+        <is>
+          <t>1d</t>
+        </is>
+      </c>
+      <c r="J32" t="inlineStr">
+        <is>
+          <t>2026-05-16</t>
+        </is>
+      </c>
+      <c r="K32" t="inlineStr">
+        <is>
+          <t>未到来</t>
+        </is>
+      </c>
+      <c r="L32" t="inlineStr">
+        <is>
+          <t>未検証</t>
+        </is>
+      </c>
+      <c r="M32" t="inlineStr">
+        <is>
+          <t>2026-05-16以降に評価</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>2026-05-15_2802.T</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>2026/05/15 10:55:11</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>2802.T</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>74</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>少額候補（決算要確認）</t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>5426</t>
+        </is>
+      </c>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="H33" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="I33" t="inlineStr">
+        <is>
+          <t>5d</t>
+        </is>
+      </c>
+      <c r="J33" t="inlineStr">
+        <is>
+          <t>2026-05-20</t>
+        </is>
+      </c>
+      <c r="K33" t="inlineStr">
+        <is>
+          <t>未到来</t>
+        </is>
+      </c>
+      <c r="L33" t="inlineStr">
+        <is>
+          <t>未検証</t>
+        </is>
+      </c>
+      <c r="M33" t="inlineStr">
+        <is>
+          <t>2026-05-20以降に評価</t>
         </is>
       </c>
     </row>
@@ -1388,7 +2460,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026/05/14 21:07:01</t>
+          <t>2026/05/14 21:24:24</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -1445,7 +2517,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>2026/05/14 21:07:01</t>
+          <t>2026/05/14 21:24:24</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -1502,7 +2574,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>2026/05/14 21:07:01</t>
+          <t>2026/05/14 21:24:24</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -1559,7 +2631,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>2026/05/14 21:07:01</t>
+          <t>2026/05/14 21:24:24</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -1616,7 +2688,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>2026/05/14 21:07:01</t>
+          <t>2026/05/14 21:24:24</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -1673,7 +2745,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>2026/05/14 21:07:01</t>
+          <t>2026/05/14 21:24:24</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -1730,7 +2802,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>2026/05/14 21:07:01</t>
+          <t>2026/05/14 21:24:24</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -1787,7 +2859,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>2026/05/14 21:07:01</t>
+          <t>2026/05/14 21:24:24</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -1839,12 +2911,12 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>2026-05-14_8035.T</t>
+          <t>2026-05-15_8035.T</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>2026/05/14 21:24:24</t>
+          <t>2026/05/15 10:55:11</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -1864,7 +2936,7 @@
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>51200</t>
+          <t>51030</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
@@ -1874,12 +2946,12 @@
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>2026-05-15</t>
+          <t>2026-05-16</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>2026-05-19</t>
+          <t>2026-05-20</t>
         </is>
       </c>
       <c r="J10" t="inlineStr">
@@ -1889,19 +2961,19 @@
       </c>
       <c r="K10" t="inlineStr">
         <is>
-          <t>終値51200 / 20日騰落16.26% / 出来高倍率0.61 / PER未取得 / PBR11.38 / EPS未取得</t>
+          <t>終値51030 / 20日騰落20.18% / 出来高倍率0.31 / PER未取得 / PBR11.18 / EPS未取得</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2026-05-14_6857.T</t>
+          <t>2026-05-15_6857.T</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>2026/05/14 21:24:24</t>
+          <t>2026/05/15 10:55:11</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -1911,7 +2983,7 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>69</t>
+          <t>60</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
@@ -1921,7 +2993,7 @@
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>28615</t>
+          <t>27535</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
@@ -1931,12 +3003,12 @@
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>2026-05-15</t>
+          <t>2026-05-16</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>2026-05-19</t>
+          <t>2026-05-20</t>
         </is>
       </c>
       <c r="J11" t="inlineStr">
@@ -1946,19 +3018,19 @@
       </c>
       <c r="K11" t="inlineStr">
         <is>
-          <t>終値28615 / 20日騰落14.51% / 出来高倍率0.9 / PER44.6 / PBR26.07 / EPS641.61</t>
+          <t>終値27535 / 20日騰落10.67% / 出来高倍率0.31 / PER42.39 / PBR24.78 / EPS641.61</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>2026-05-14_4519.T</t>
+          <t>2026-05-15_4519.T</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>2026/05/14 21:24:24</t>
+          <t>2026/05/15 10:55:11</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -1978,7 +3050,7 @@
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>8096</t>
+          <t>8014</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
@@ -1988,12 +3060,12 @@
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>2026-05-15</t>
+          <t>2026-05-16</t>
         </is>
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>2026-05-19</t>
+          <t>2026-05-20</t>
         </is>
       </c>
       <c r="J12" t="inlineStr">
@@ -2003,19 +3075,19 @@
       </c>
       <c r="K12" t="inlineStr">
         <is>
-          <t>終値8096 / 20日騰落-6.67% / 出来高倍率0.75 / PER未取得 / PBR6.98 / EPS未取得</t>
+          <t>終値8014 / 20日騰落-6.65% / 出来高倍率0.15 / PER未取得 / PBR6.93 / EPS未取得</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>2026-05-14_8306.T</t>
+          <t>2026-05-15_8306.T</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>2026/05/14 21:24:24</t>
+          <t>2026/05/15 10:55:11</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -2025,7 +3097,7 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>68</t>
+          <t>65</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
@@ -2035,7 +3107,7 @@
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>2877</t>
+          <t>2927.5</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
@@ -2045,12 +3117,12 @@
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>2026-05-15</t>
+          <t>2026-05-16</t>
         </is>
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>2026-05-19</t>
+          <t>2026-05-20</t>
         </is>
       </c>
       <c r="J13" t="inlineStr">
@@ -2060,19 +3132,19 @@
       </c>
       <c r="K13" t="inlineStr">
         <is>
-          <t>終値2877 / 20日騰落1.23% / 出来高倍率0.96 / PER未取得 / PBR1.53 / EPS未取得</t>
+          <t>終値2927.5 / 20日騰落2.36% / 出来高倍率0.58 / PER未取得 / PBR1.55 / EPS未取得</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>2026-05-14_8058.T</t>
+          <t>2026-05-15_8058.T</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>2026/05/14 21:24:24</t>
+          <t>2026/05/15 10:55:11</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -2082,7 +3154,7 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>80</t>
+          <t>84</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
@@ -2092,7 +3164,7 @@
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>5882</t>
+          <t>5859</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
@@ -2102,12 +3174,12 @@
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>2026-05-15</t>
+          <t>2026-05-16</t>
         </is>
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>2026-05-19</t>
+          <t>2026-05-20</t>
         </is>
       </c>
       <c r="J14" t="inlineStr">
@@ -2117,19 +3189,19 @@
       </c>
       <c r="K14" t="inlineStr">
         <is>
-          <t>終値5882 / 20日騰落10.83% / 出来高倍率0.71 / PER19.58 / PBR2.28 / EPS300.42</t>
+          <t>終値5859 / 20日騰落11.07% / 出来高倍率0.29 / PER19.44 / PBR2.27 / EPS300.42</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>2026-05-14_7974.T</t>
+          <t>2026-05-15_7974.T</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>2026/05/14 21:24:24</t>
+          <t>2026/05/15 10:55:11</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -2139,7 +3211,7 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>44</t>
+          <t>39</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
@@ -2149,7 +3221,7 @@
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>6864</t>
+          <t>6992</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
@@ -2159,12 +3231,12 @@
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>2026-05-15</t>
+          <t>2026-05-16</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>2026-05-19</t>
+          <t>2026-05-20</t>
         </is>
       </c>
       <c r="J15" t="inlineStr">
@@ -2174,19 +3246,19 @@
       </c>
       <c r="K15" t="inlineStr">
         <is>
-          <t>終値6864 / 20日騰落-17.3% / 出来高倍率1.36 / PER25.53 / PBR2.68 / EPS268.9</t>
+          <t>終値6992 / 20日騰落-15.73% / 出来高倍率0.36 / PER26.11 / PBR2.74 / EPS268.9</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>2026-05-14_9433.T</t>
+          <t>2026-05-15_9433.T</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>2026/05/14 21:24:24</t>
+          <t>2026/05/15 10:55:11</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -2196,7 +3268,7 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>67</t>
+          <t>65</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
@@ -2206,7 +3278,7 @@
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>2645.5</t>
+          <t>2653</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
@@ -2216,12 +3288,12 @@
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>2026-05-15</t>
+          <t>2026-05-16</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>2026-05-19</t>
+          <t>2026-05-20</t>
         </is>
       </c>
       <c r="J16" t="inlineStr">
@@ -2231,19 +3303,19 @@
       </c>
       <c r="K16" t="inlineStr">
         <is>
-          <t>終値2645.5 / 20日騰落2.46% / 出来高倍率1.2 / PER未取得 / PBR1.98 / EPS未取得</t>
+          <t>終値2653 / 20日騰落1.26% / 出来高倍率0.31 / PER未取得 / PBR1.99 / EPS未取得</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>2026-05-14_2802.T</t>
+          <t>2026-05-15_2802.T</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>2026/05/14 21:24:24</t>
+          <t>2026/05/15 10:55:11</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -2253,7 +3325,7 @@
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>79</t>
+          <t>74</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
@@ -2263,7 +3335,7 @@
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>5542</t>
+          <t>5426</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
@@ -2273,12 +3345,12 @@
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>2026-05-15</t>
+          <t>2026-05-16</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>2026-05-19</t>
+          <t>2026-05-20</t>
         </is>
       </c>
       <c r="J17" t="inlineStr">
@@ -2288,7 +3360,7 @@
       </c>
       <c r="K17" t="inlineStr">
         <is>
-          <t>終値5542 / 20日騰落19.13% / 出来高倍率1.21 / PER44.27 / PBR6.89 / EPS125.2</t>
+          <t>終値5426 / 20日騰落17.78% / 出来高倍率0.24 / PER43.07 / PBR6.7 / EPS125.2</t>
         </is>
       </c>
     </row>
@@ -2341,7 +3413,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026/05/14 21:24:24</t>
+          <t>2026/05/15 10:55:11</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -2434,7 +3506,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026/05/14 21:24:24</t>
+          <t>2026/05/15 10:55:11</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -2448,7 +3520,7 @@
         </is>
       </c>
       <c r="D2">
-        <v>80</v>
+        <v>84</v>
       </c>
       <c r="E2" t="inlineStr">
         <is>
@@ -2484,7 +3556,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026/05/14 21:24:24</t>
+          <t>2026/05/15 10:55:11</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -2498,7 +3570,7 @@
         </is>
       </c>
       <c r="D3">
-        <v>79</v>
+        <v>74</v>
       </c>
       <c r="E3" t="inlineStr">
         <is>
@@ -2612,7 +3684,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>10.07</v>
+        <v>10.29</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -2652,7 +3724,7 @@
         </is>
       </c>
       <c r="E3">
-        <v>9.94</v>
+        <v>10.51</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
@@ -2692,7 +3764,7 @@
         </is>
       </c>
       <c r="E4">
-        <v>17.84</v>
+        <v>17.26</v>
       </c>
       <c r="F4" t="inlineStr">
         <is>
@@ -2732,7 +3804,7 @@
         </is>
       </c>
       <c r="E5">
-        <v>4.481</v>
+        <v>4.461</v>
       </c>
       <c r="F5" t="inlineStr">
         <is>
@@ -3136,7 +4208,7 @@
         </is>
       </c>
       <c r="F2">
-        <v>80</v>
+        <v>84</v>
       </c>
       <c r="G2" t="inlineStr">
         <is>
@@ -3181,7 +4253,7 @@
         </is>
       </c>
       <c r="F3">
-        <v>79</v>
+        <v>74</v>
       </c>
       <c r="G3" t="inlineStr">
         <is>
@@ -5082,6 +6154,774 @@
       <c r="F57" t="inlineStr">
         <is>
           <t>終値5542 / 20日騰落19.13% / 出来高倍率1.21 / PER44.27 / PBR6.89 / EPS125.2</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>2026/05/15 10:53:45</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>8035.T</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>60</t>
+        </is>
+      </c>
+      <c r="D58" t="inlineStr">
+        <is>
+          <t>様子見</t>
+        </is>
+      </c>
+      <c r="E58" t="inlineStr">
+        <is>
+          <t>価格・市場・一部財務で計算</t>
+        </is>
+      </c>
+      <c r="F58" t="inlineStr">
+        <is>
+          <t>終値51010 / 20日騰落20.14% / 出来高倍率0.3 / PER未取得 / PBR11.17 / EPS未取得</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>2026/05/15 10:53:45</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>6857.T</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>60</t>
+        </is>
+      </c>
+      <c r="D59" t="inlineStr">
+        <is>
+          <t>様子見</t>
+        </is>
+      </c>
+      <c r="E59" t="inlineStr">
+        <is>
+          <t>価格・市場・一部財務で計算</t>
+        </is>
+      </c>
+      <c r="F59" t="inlineStr">
+        <is>
+          <t>終値27550 / 20日騰落10.73% / 出来高倍率0.31 / PER42.32 / PBR24.74 / EPS641.61</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>2026/05/15 10:53:45</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>4519.T</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>33</t>
+        </is>
+      </c>
+      <c r="D60" t="inlineStr">
+        <is>
+          <t>除外/待機</t>
+        </is>
+      </c>
+      <c r="E60" t="inlineStr">
+        <is>
+          <t>価格・市場・一部財務で計算</t>
+        </is>
+      </c>
+      <c r="F60" t="inlineStr">
+        <is>
+          <t>終値8024 / 20日騰落-6.53% / 出来高倍率0.15 / PER未取得 / PBR6.94 / EPS未取得</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>2026/05/15 10:53:45</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>8306.T</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>65</t>
+        </is>
+      </c>
+      <c r="D61" t="inlineStr">
+        <is>
+          <t>様子見</t>
+        </is>
+      </c>
+      <c r="E61" t="inlineStr">
+        <is>
+          <t>価格・市場・一部財務で計算</t>
+        </is>
+      </c>
+      <c r="F61" t="inlineStr">
+        <is>
+          <t>終値2926.5 / 20日騰落2.33% / 出来高倍率0.58 / PER未取得 / PBR1.55 / EPS未取得</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>2026/05/15 10:53:45</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>8058.T</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>84</t>
+        </is>
+      </c>
+      <c r="D62" t="inlineStr">
+        <is>
+          <t>買い候補（決算要確認）</t>
+        </is>
+      </c>
+      <c r="E62" t="inlineStr">
+        <is>
+          <t>価格・市場・一部財務で計算</t>
+        </is>
+      </c>
+      <c r="F62" t="inlineStr">
+        <is>
+          <t>終値5858 / 20日騰落11.05% / 出来高倍率0.29 / PER19.44 / PBR2.26 / EPS300.42</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>2026/05/15 10:53:45</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>7974.T</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>39</t>
+        </is>
+      </c>
+      <c r="D63" t="inlineStr">
+        <is>
+          <t>除外/待機</t>
+        </is>
+      </c>
+      <c r="E63" t="inlineStr">
+        <is>
+          <t>価格・市場・一部財務で計算</t>
+        </is>
+      </c>
+      <c r="F63" t="inlineStr">
+        <is>
+          <t>終値6997 / 20日騰落-15.67% / 出来高倍率0.36 / PER26.11 / PBR2.74 / EPS268.9</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>2026/05/15 10:53:45</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>9433.T</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>58</t>
+        </is>
+      </c>
+      <c r="D64" t="inlineStr">
+        <is>
+          <t>様子見</t>
+        </is>
+      </c>
+      <c r="E64" t="inlineStr">
+        <is>
+          <t>価格・市場・一部財務で計算</t>
+        </is>
+      </c>
+      <c r="F64" t="inlineStr">
+        <is>
+          <t>終値2646 / 20日騰落0.99% / 出来高倍率0.3 / PER未取得 / PBR1.99 / EPS未取得</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>2026/05/15 10:53:45</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>2802.T</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>74</t>
+        </is>
+      </c>
+      <c r="D65" t="inlineStr">
+        <is>
+          <t>少額候補（決算要確認）</t>
+        </is>
+      </c>
+      <c r="E65" t="inlineStr">
+        <is>
+          <t>価格・市場・一部財務で計算</t>
+        </is>
+      </c>
+      <c r="F65" t="inlineStr">
+        <is>
+          <t>終値5426 / 20日騰落17.78% / 出来高倍率0.23 / PER43.09 / PBR6.71 / EPS125.2</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>2026/05/15 10:54:26</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>8035.T</t>
+        </is>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>60</t>
+        </is>
+      </c>
+      <c r="D66" t="inlineStr">
+        <is>
+          <t>様子見</t>
+        </is>
+      </c>
+      <c r="E66" t="inlineStr">
+        <is>
+          <t>価格・市場・一部財務で計算</t>
+        </is>
+      </c>
+      <c r="F66" t="inlineStr">
+        <is>
+          <t>終値50940 / 20日騰落19.97% / 出来高倍率0.3 / PER未取得 / PBR11.18 / EPS未取得</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>2026/05/15 10:54:26</t>
+        </is>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>6857.T</t>
+        </is>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>60</t>
+        </is>
+      </c>
+      <c r="D67" t="inlineStr">
+        <is>
+          <t>様子見</t>
+        </is>
+      </c>
+      <c r="E67" t="inlineStr">
+        <is>
+          <t>価格・市場・一部財務で計算</t>
+        </is>
+      </c>
+      <c r="F67" t="inlineStr">
+        <is>
+          <t>終値27535 / 20日騰落10.67% / 出来高倍率0.31 / PER42.39 / PBR24.78 / EPS641.61</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>2026/05/15 10:54:26</t>
+        </is>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>4519.T</t>
+        </is>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>33</t>
+        </is>
+      </c>
+      <c r="D68" t="inlineStr">
+        <is>
+          <t>除外/待機</t>
+        </is>
+      </c>
+      <c r="E68" t="inlineStr">
+        <is>
+          <t>価格・市場・一部財務で計算</t>
+        </is>
+      </c>
+      <c r="F68" t="inlineStr">
+        <is>
+          <t>終値8025 / 20日騰落-6.52% / 出来高倍率0.15 / PER未取得 / PBR6.93 / EPS未取得</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>2026/05/15 10:54:26</t>
+        </is>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>8306.T</t>
+        </is>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>65</t>
+        </is>
+      </c>
+      <c r="D69" t="inlineStr">
+        <is>
+          <t>様子見</t>
+        </is>
+      </c>
+      <c r="E69" t="inlineStr">
+        <is>
+          <t>価格・市場・一部財務で計算</t>
+        </is>
+      </c>
+      <c r="F69" t="inlineStr">
+        <is>
+          <t>終値2925 / 20日騰落2.27% / 出来高倍率0.58 / PER未取得 / PBR1.55 / EPS未取得</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>2026/05/15 10:54:26</t>
+        </is>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>8058.T</t>
+        </is>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>84</t>
+        </is>
+      </c>
+      <c r="D70" t="inlineStr">
+        <is>
+          <t>買い候補（決算要確認）</t>
+        </is>
+      </c>
+      <c r="E70" t="inlineStr">
+        <is>
+          <t>価格・市場・一部財務で計算</t>
+        </is>
+      </c>
+      <c r="F70" t="inlineStr">
+        <is>
+          <t>終値5857 / 20日騰落11.03% / 出来高倍率0.29 / PER19.44 / PBR2.27 / EPS300.42</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>2026/05/15 10:54:26</t>
+        </is>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>7974.T</t>
+        </is>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>39</t>
+        </is>
+      </c>
+      <c r="D71" t="inlineStr">
+        <is>
+          <t>除外/待機</t>
+        </is>
+      </c>
+      <c r="E71" t="inlineStr">
+        <is>
+          <t>価格・市場・一部財務で計算</t>
+        </is>
+      </c>
+      <c r="F71" t="inlineStr">
+        <is>
+          <t>終値6993 / 20日騰落-15.72% / 出来高倍率0.36 / PER26.09 / PBR2.74 / EPS268.9</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>2026/05/15 10:54:26</t>
+        </is>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>9433.T</t>
+        </is>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>65</t>
+        </is>
+      </c>
+      <c r="D72" t="inlineStr">
+        <is>
+          <t>様子見</t>
+        </is>
+      </c>
+      <c r="E72" t="inlineStr">
+        <is>
+          <t>価格・市場・一部財務で計算</t>
+        </is>
+      </c>
+      <c r="F72" t="inlineStr">
+        <is>
+          <t>終値2652 / 20日騰落1.22% / 出来高倍率0.3 / PER未取得 / PBR1.99 / EPS未取得</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>2026/05/15 10:54:26</t>
+        </is>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>2802.T</t>
+        </is>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>74</t>
+        </is>
+      </c>
+      <c r="D73" t="inlineStr">
+        <is>
+          <t>少額候補（決算要確認）</t>
+        </is>
+      </c>
+      <c r="E73" t="inlineStr">
+        <is>
+          <t>価格・市場・一部財務で計算</t>
+        </is>
+      </c>
+      <c r="F73" t="inlineStr">
+        <is>
+          <t>終値5427 / 20日騰落17.8% / 出来高倍率0.23 / PER43.08 / PBR6.71 / EPS125.2</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>2026/05/15 10:55:11</t>
+        </is>
+      </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>8035.T</t>
+        </is>
+      </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>60</t>
+        </is>
+      </c>
+      <c r="D74" t="inlineStr">
+        <is>
+          <t>様子見</t>
+        </is>
+      </c>
+      <c r="E74" t="inlineStr">
+        <is>
+          <t>価格・市場・一部財務で計算</t>
+        </is>
+      </c>
+      <c r="F74" t="inlineStr">
+        <is>
+          <t>終値51030 / 20日騰落20.18% / 出来高倍率0.31 / PER未取得 / PBR11.18 / EPS未取得</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>2026/05/15 10:55:11</t>
+        </is>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>6857.T</t>
+        </is>
+      </c>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>60</t>
+        </is>
+      </c>
+      <c r="D75" t="inlineStr">
+        <is>
+          <t>様子見</t>
+        </is>
+      </c>
+      <c r="E75" t="inlineStr">
+        <is>
+          <t>価格・市場・一部財務で計算</t>
+        </is>
+      </c>
+      <c r="F75" t="inlineStr">
+        <is>
+          <t>終値27535 / 20日騰落10.67% / 出来高倍率0.31 / PER42.39 / PBR24.78 / EPS641.61</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>2026/05/15 10:55:11</t>
+        </is>
+      </c>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>4519.T</t>
+        </is>
+      </c>
+      <c r="C76" t="inlineStr">
+        <is>
+          <t>33</t>
+        </is>
+      </c>
+      <c r="D76" t="inlineStr">
+        <is>
+          <t>除外/待機</t>
+        </is>
+      </c>
+      <c r="E76" t="inlineStr">
+        <is>
+          <t>価格・市場・一部財務で計算</t>
+        </is>
+      </c>
+      <c r="F76" t="inlineStr">
+        <is>
+          <t>終値8014 / 20日騰落-6.65% / 出来高倍率0.15 / PER未取得 / PBR6.93 / EPS未取得</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>2026/05/15 10:55:11</t>
+        </is>
+      </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>8306.T</t>
+        </is>
+      </c>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>65</t>
+        </is>
+      </c>
+      <c r="D77" t="inlineStr">
+        <is>
+          <t>様子見</t>
+        </is>
+      </c>
+      <c r="E77" t="inlineStr">
+        <is>
+          <t>価格・市場・一部財務で計算</t>
+        </is>
+      </c>
+      <c r="F77" t="inlineStr">
+        <is>
+          <t>終値2927.5 / 20日騰落2.36% / 出来高倍率0.58 / PER未取得 / PBR1.55 / EPS未取得</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t>2026/05/15 10:55:11</t>
+        </is>
+      </c>
+      <c r="B78" t="inlineStr">
+        <is>
+          <t>8058.T</t>
+        </is>
+      </c>
+      <c r="C78" t="inlineStr">
+        <is>
+          <t>84</t>
+        </is>
+      </c>
+      <c r="D78" t="inlineStr">
+        <is>
+          <t>買い候補（決算要確認）</t>
+        </is>
+      </c>
+      <c r="E78" t="inlineStr">
+        <is>
+          <t>価格・市場・一部財務で計算</t>
+        </is>
+      </c>
+      <c r="F78" t="inlineStr">
+        <is>
+          <t>終値5859 / 20日騰落11.07% / 出来高倍率0.29 / PER19.44 / PBR2.27 / EPS300.42</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="inlineStr">
+        <is>
+          <t>2026/05/15 10:55:11</t>
+        </is>
+      </c>
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>7974.T</t>
+        </is>
+      </c>
+      <c r="C79" t="inlineStr">
+        <is>
+          <t>39</t>
+        </is>
+      </c>
+      <c r="D79" t="inlineStr">
+        <is>
+          <t>除外/待機</t>
+        </is>
+      </c>
+      <c r="E79" t="inlineStr">
+        <is>
+          <t>価格・市場・一部財務で計算</t>
+        </is>
+      </c>
+      <c r="F79" t="inlineStr">
+        <is>
+          <t>終値6992 / 20日騰落-15.73% / 出来高倍率0.36 / PER26.11 / PBR2.74 / EPS268.9</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="inlineStr">
+        <is>
+          <t>2026/05/15 10:55:11</t>
+        </is>
+      </c>
+      <c r="B80" t="inlineStr">
+        <is>
+          <t>9433.T</t>
+        </is>
+      </c>
+      <c r="C80" t="inlineStr">
+        <is>
+          <t>65</t>
+        </is>
+      </c>
+      <c r="D80" t="inlineStr">
+        <is>
+          <t>様子見</t>
+        </is>
+      </c>
+      <c r="E80" t="inlineStr">
+        <is>
+          <t>価格・市場・一部財務で計算</t>
+        </is>
+      </c>
+      <c r="F80" t="inlineStr">
+        <is>
+          <t>終値2653 / 20日騰落1.26% / 出来高倍率0.31 / PER未取得 / PBR1.99 / EPS未取得</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="inlineStr">
+        <is>
+          <t>2026/05/15 10:55:11</t>
+        </is>
+      </c>
+      <c r="B81" t="inlineStr">
+        <is>
+          <t>2802.T</t>
+        </is>
+      </c>
+      <c r="C81" t="inlineStr">
+        <is>
+          <t>74</t>
+        </is>
+      </c>
+      <c r="D81" t="inlineStr">
+        <is>
+          <t>少額候補（決算要確認）</t>
+        </is>
+      </c>
+      <c r="E81" t="inlineStr">
+        <is>
+          <t>価格・市場・一部財務で計算</t>
+        </is>
+      </c>
+      <c r="F81" t="inlineStr">
+        <is>
+          <t>終値5426 / 20日騰落17.78% / 出来高倍率0.24 / PER43.07 / PBR6.7 / EPS125.2</t>
         </is>
       </c>
     </row>
@@ -5165,7 +7005,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026/05/14 21:24:24</t>
+          <t>2026/05/15 10:55:11</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -5179,7 +7019,7 @@
         </is>
       </c>
       <c r="D2">
-        <v>80</v>
+        <v>84</v>
       </c>
       <c r="E2">
         <v>7</v>
@@ -5188,7 +7028,7 @@
         <v>-11</v>
       </c>
       <c r="G2">
-        <v>76</v>
+        <v>80</v>
       </c>
       <c r="H2" t="inlineStr">
         <is>
@@ -5214,7 +7054,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026/05/14 21:24:24</t>
+          <t>2026/05/15 10:55:11</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -5228,7 +7068,7 @@
         </is>
       </c>
       <c r="D3">
-        <v>79</v>
+        <v>74</v>
       </c>
       <c r="E3">
         <v>8</v>
@@ -5237,7 +7077,7 @@
         <v>-15</v>
       </c>
       <c r="G3">
-        <v>72</v>
+        <v>67</v>
       </c>
       <c r="H3" t="inlineStr">
         <is>
@@ -5647,28 +7487,28 @@
         </is>
       </c>
       <c r="B2">
-        <v>51200</v>
+        <v>51030</v>
       </c>
       <c r="C2">
-        <v>45873.6</v>
+        <v>46380</v>
       </c>
       <c r="D2">
-        <v>42674</v>
+        <v>42804.93</v>
       </c>
       <c r="E2">
-        <v>34139.57</v>
+        <v>34257.68</v>
       </c>
       <c r="F2">
-        <v>-1.01</v>
+        <v>-2.71</v>
       </c>
       <c r="G2">
-        <v>16.26</v>
+        <v>20.18</v>
       </c>
       <c r="H2">
-        <v>23.37</v>
+        <v>23.56</v>
       </c>
       <c r="I2">
-        <v>0.61</v>
+        <v>0.31</v>
       </c>
       <c r="J2" t="inlineStr">
         <is>
@@ -5676,7 +7516,7 @@
         </is>
       </c>
       <c r="K2">
-        <v>11.38</v>
+        <v>11.18</v>
       </c>
       <c r="L2" t="inlineStr">
         <is>
@@ -5687,7 +7527,7 @@
         <v>-5.75</v>
       </c>
       <c r="N2">
-        <v>3.3</v>
+        <v>3.28</v>
       </c>
       <c r="O2">
         <f>IF(B2&gt;=C2,6,0)+IF(B2&gt;=D2,7,0)+IF(B2&gt;=E2,7,0)</f>
@@ -5718,43 +7558,43 @@
         </is>
       </c>
       <c r="B3">
-        <v>28615</v>
+        <v>27535</v>
       </c>
       <c r="C3">
-        <v>27438.2</v>
+        <v>27662.4</v>
       </c>
       <c r="D3">
-        <v>25608.73</v>
+        <v>25685.6</v>
       </c>
       <c r="E3">
-        <v>19856.25</v>
+        <v>19935.33</v>
       </c>
       <c r="F3">
-        <v>-3.7</v>
+        <v>-7.86</v>
       </c>
       <c r="G3">
-        <v>14.51</v>
+        <v>10.67</v>
       </c>
       <c r="H3">
-        <v>3.4</v>
+        <v>2.7</v>
       </c>
       <c r="I3">
-        <v>0.9</v>
+        <v>0.31</v>
       </c>
       <c r="J3">
-        <v>44.6</v>
+        <v>42.39</v>
       </c>
       <c r="K3">
-        <v>26.07</v>
+        <v>24.78</v>
       </c>
       <c r="L3">
         <v>641.61</v>
       </c>
       <c r="M3">
-        <v>-11.7</v>
+        <v>-12.59</v>
       </c>
       <c r="N3">
-        <v>3.99</v>
+        <v>3.67</v>
       </c>
       <c r="O3">
         <f>IF(B3&gt;=C3,6,0)+IF(B3&gt;=D3,7,0)+IF(B3&gt;=E3,7,0)</f>
@@ -5785,28 +7625,28 @@
         </is>
       </c>
       <c r="B4">
-        <v>8096</v>
+        <v>8014</v>
       </c>
       <c r="C4">
-        <v>8403.88</v>
+        <v>8369.84</v>
       </c>
       <c r="D4">
-        <v>8880.21</v>
+        <v>8876.2</v>
       </c>
       <c r="E4">
-        <v>7934.89</v>
+        <v>7940.72</v>
       </c>
       <c r="F4">
-        <v>0.01</v>
+        <v>1.44</v>
       </c>
       <c r="G4">
-        <v>-6.67</v>
+        <v>-6.65</v>
       </c>
       <c r="H4">
-        <v>-10.26</v>
+        <v>-12.89</v>
       </c>
       <c r="I4">
-        <v>0.75</v>
+        <v>0.15</v>
       </c>
       <c r="J4" t="inlineStr">
         <is>
@@ -5814,7 +7654,7 @@
         </is>
       </c>
       <c r="K4">
-        <v>6.98</v>
+        <v>6.93</v>
       </c>
       <c r="L4" t="inlineStr">
         <is>
@@ -5825,7 +7665,7 @@
         <v>-16.59</v>
       </c>
       <c r="N4">
-        <v>4.49</v>
+        <v>4.5</v>
       </c>
       <c r="O4">
         <f>IF(B4&gt;=C4,6,0)+IF(B4&gt;=D4,7,0)+IF(B4&gt;=E4,7,0)</f>
@@ -5856,28 +7696,28 @@
         </is>
       </c>
       <c r="B5">
-        <v>2877</v>
+        <v>2927.5</v>
       </c>
       <c r="C5">
-        <v>2844.34</v>
+        <v>2849.76</v>
       </c>
       <c r="D5">
-        <v>2812.37</v>
+        <v>2813.65</v>
       </c>
       <c r="E5">
-        <v>2522.66</v>
+        <v>2527.3</v>
       </c>
       <c r="F5">
-        <v>0.49</v>
+        <v>4.31</v>
       </c>
       <c r="G5">
-        <v>1.23</v>
+        <v>2.36</v>
       </c>
       <c r="H5">
-        <v>-5.17</v>
+        <v>-5.11</v>
       </c>
       <c r="I5">
-        <v>0.96</v>
+        <v>0.58</v>
       </c>
       <c r="J5" t="inlineStr">
         <is>
@@ -5885,7 +7725,7 @@
         </is>
       </c>
       <c r="K5">
-        <v>1.53</v>
+        <v>1.55</v>
       </c>
       <c r="L5" t="inlineStr">
         <is>
@@ -5896,7 +7736,7 @@
         <v>-6.6</v>
       </c>
       <c r="N5">
-        <v>1.67</v>
+        <v>1.71</v>
       </c>
       <c r="O5">
         <f>IF(B5&gt;=C5,6,0)+IF(B5&gt;=D5,7,0)+IF(B5&gt;=E5,7,0)</f>
@@ -5927,43 +7767,43 @@
         </is>
       </c>
       <c r="B6">
-        <v>5882</v>
+        <v>5859</v>
       </c>
       <c r="C6">
-        <v>5192</v>
+        <v>5210.16</v>
       </c>
       <c r="D6">
-        <v>5037.77</v>
+        <v>5061.95</v>
       </c>
       <c r="E6">
-        <v>4075.95</v>
+        <v>4090.93</v>
       </c>
       <c r="F6">
-        <v>8.97</v>
+        <v>11.62</v>
       </c>
       <c r="G6">
-        <v>10.83</v>
+        <v>11.07</v>
       </c>
       <c r="H6">
-        <v>14.5</v>
+        <v>13.46</v>
       </c>
       <c r="I6">
-        <v>0.71</v>
+        <v>0.29</v>
       </c>
       <c r="J6">
-        <v>19.58</v>
+        <v>19.44</v>
       </c>
       <c r="K6">
-        <v>2.28</v>
+        <v>2.27</v>
       </c>
       <c r="L6">
         <v>300.42</v>
       </c>
       <c r="M6">
-        <v>-10.03</v>
+        <v>-8.61</v>
       </c>
       <c r="N6">
-        <v>2.92</v>
+        <v>2.88</v>
       </c>
       <c r="O6">
         <f>IF(B6&gt;=C6,6,0)+IF(B6&gt;=D6,7,0)+IF(B6&gt;=E6,7,0)</f>
@@ -5994,34 +7834,34 @@
         </is>
       </c>
       <c r="B7">
-        <v>6864</v>
+        <v>6992</v>
       </c>
       <c r="C7">
-        <v>8030.04</v>
+        <v>7955.76</v>
       </c>
       <c r="D7">
-        <v>8814.31</v>
+        <v>8771.8</v>
       </c>
       <c r="E7">
-        <v>11235.42</v>
+        <v>11207.75</v>
       </c>
       <c r="F7">
-        <v>-7.29</v>
+        <v>-8.8</v>
       </c>
       <c r="G7">
-        <v>-17.3</v>
+        <v>-15.73</v>
       </c>
       <c r="H7">
-        <v>-23.14</v>
+        <v>-19.07</v>
       </c>
       <c r="I7">
-        <v>1.36</v>
+        <v>0.36</v>
       </c>
       <c r="J7">
-        <v>25.53</v>
+        <v>26.11</v>
       </c>
       <c r="K7">
-        <v>2.68</v>
+        <v>2.74</v>
       </c>
       <c r="L7">
         <v>268.9</v>
@@ -6030,7 +7870,7 @@
         <v>-20.33</v>
       </c>
       <c r="N7">
-        <v>2.7</v>
+        <v>2.77</v>
       </c>
       <c r="O7">
         <f>IF(B7&gt;=C7,6,0)+IF(B7&gt;=D7,7,0)+IF(B7&gt;=E7,7,0)</f>
@@ -6061,28 +7901,28 @@
         </is>
       </c>
       <c r="B8">
-        <v>2645.5</v>
+        <v>2653</v>
       </c>
       <c r="C8">
-        <v>2604.04</v>
+        <v>2599.62</v>
       </c>
       <c r="D8">
-        <v>2647.67</v>
+        <v>2647.45</v>
       </c>
       <c r="E8">
-        <v>2593.13</v>
+        <v>2594.29</v>
       </c>
       <c r="F8">
-        <v>4.77</v>
+        <v>4.92</v>
       </c>
       <c r="G8">
-        <v>2.46</v>
+        <v>1.26</v>
       </c>
       <c r="H8">
-        <v>2.54</v>
+        <v>-0.32</v>
       </c>
       <c r="I8">
-        <v>1.2</v>
+        <v>0.31</v>
       </c>
       <c r="J8" t="inlineStr">
         <is>
@@ -6090,7 +7930,7 @@
         </is>
       </c>
       <c r="K8">
-        <v>1.98</v>
+        <v>1.99</v>
       </c>
       <c r="L8" t="inlineStr">
         <is>
@@ -6132,34 +7972,34 @@
         </is>
       </c>
       <c r="B9">
-        <v>5542</v>
+        <v>5426</v>
       </c>
       <c r="C9">
-        <v>4854.44</v>
+        <v>4885.2</v>
       </c>
       <c r="D9">
-        <v>4477.05</v>
+        <v>4500.57</v>
       </c>
       <c r="E9">
-        <v>4107.9</v>
+        <v>4115.51</v>
       </c>
       <c r="F9">
-        <v>11.78</v>
+        <v>7.87</v>
       </c>
       <c r="G9">
-        <v>19.13</v>
+        <v>17.78</v>
       </c>
       <c r="H9">
-        <v>28.73</v>
+        <v>24.56</v>
       </c>
       <c r="I9">
-        <v>1.21</v>
+        <v>0.24</v>
       </c>
       <c r="J9">
-        <v>44.27</v>
+        <v>43.07</v>
       </c>
       <c r="K9">
-        <v>6.89</v>
+        <v>6.7</v>
       </c>
       <c r="L9">
         <v>125.2</v>
@@ -6168,7 +8008,7 @@
         <v>-4.09</v>
       </c>
       <c r="N9">
-        <v>2.99</v>
+        <v>3.06</v>
       </c>
       <c r="O9">
         <f>IF(B9&gt;=C9,6,0)+IF(B9&gt;=D9,7,0)+IF(B9&gt;=E9,7,0)</f>
@@ -6621,10 +8461,10 @@
         </is>
       </c>
       <c r="B3">
-        <v>69</v>
+        <v>60</v>
       </c>
       <c r="C3">
-        <v>69</v>
+        <v>60</v>
       </c>
       <c r="D3">
         <v>0</v>
@@ -6636,7 +8476,7 @@
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>trend:20/20, momentum:11/11, volume:6/6, valuation:2/2, macro:15/15, fundamental:12/12, risk:3/3</t>
+          <t>trend:14/14, momentum:11/11, volume:3/3, valuation:2/2, macro:15/15, fundamental:12/12, risk:3/3</t>
         </is>
       </c>
     </row>
@@ -6673,10 +8513,10 @@
         </is>
       </c>
       <c r="B5">
-        <v>68</v>
+        <v>65</v>
       </c>
       <c r="C5">
-        <v>68</v>
+        <v>65</v>
       </c>
       <c r="D5">
         <v>0</v>
@@ -6688,7 +8528,7 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>trend:20/20, momentum:9/9, volume:6/6, valuation:5/5, macro:15/15, fundamental:3/3, risk:10/10</t>
+          <t>trend:20/20, momentum:9/9, volume:3/3, valuation:5/5, macro:15/15, fundamental:3/3, risk:10/10</t>
         </is>
       </c>
     </row>
@@ -6699,10 +8539,10 @@
         </is>
       </c>
       <c r="B6">
-        <v>80</v>
+        <v>84</v>
       </c>
       <c r="C6">
-        <v>80</v>
+        <v>84</v>
       </c>
       <c r="D6">
         <v>0</v>
@@ -6714,7 +8554,7 @@
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>trend:20/20, momentum:15/15, volume:3/3, valuation:9/9, macro:15/15, fundamental:12/12, risk:6/6</t>
+          <t>trend:20/20, momentum:15/15, volume:3/3, valuation:9/9, macro:15/15, fundamental:12/12, risk:10/10</t>
         </is>
       </c>
     </row>
@@ -6725,10 +8565,10 @@
         </is>
       </c>
       <c r="B7">
-        <v>44</v>
+        <v>39</v>
       </c>
       <c r="C7">
-        <v>44</v>
+        <v>39</v>
       </c>
       <c r="D7">
         <v>0</v>
@@ -6740,7 +8580,7 @@
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>trend:0/0, momentum:0/0, volume:8/8, valuation:6/6, macro:15/15, fundamental:12/12, risk:3/3</t>
+          <t>trend:0/0, momentum:0/0, volume:3/3, valuation:6/6, macro:15/15, fundamental:12/12, risk:3/3</t>
         </is>
       </c>
     </row>
@@ -6751,10 +8591,10 @@
         </is>
       </c>
       <c r="B8">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="C8">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="D8">
         <v>0</v>
@@ -6766,7 +8606,7 @@
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>trend:13/13, momentum:15/15, volume:6/6, valuation:5/5, macro:15/15, fundamental:3/3, risk:10/10</t>
+          <t>trend:20/20, momentum:9/9, volume:3/3, valuation:5/5, macro:15/15, fundamental:3/3, risk:10/10</t>
         </is>
       </c>
     </row>
@@ -6777,10 +8617,10 @@
         </is>
       </c>
       <c r="B9">
-        <v>79</v>
+        <v>74</v>
       </c>
       <c r="C9">
-        <v>79</v>
+        <v>74</v>
       </c>
       <c r="D9">
         <v>0</v>
@@ -6792,7 +8632,7 @@
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>trend:20/20, momentum:12/12, volume:8/8, valuation:2/2, macro:15/15, fundamental:12/12, risk:10/10</t>
+          <t>trend:20/20, momentum:12/12, volume:3/3, valuation:2/2, macro:15/15, fundamental:12/12, risk:10/10</t>
         </is>
       </c>
     </row>
@@ -6870,7 +8710,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-05-14</t>
+          <t>2026-05-15</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -6879,19 +8719,19 @@
         </is>
       </c>
       <c r="C2">
-        <v>51590</v>
+        <v>52150</v>
       </c>
       <c r="D2">
-        <v>52730</v>
+        <v>52530</v>
       </c>
       <c r="E2">
-        <v>51200</v>
+        <v>50660</v>
       </c>
       <c r="F2">
-        <v>51200</v>
+        <v>51030</v>
       </c>
       <c r="G2">
-        <v>2051400</v>
+        <v>995000</v>
       </c>
       <c r="H2" t="inlineStr">
         <is>
@@ -6900,7 +8740,7 @@
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>2026/05/14 21:24:24</t>
+          <t>2026/05/15 10:55:11</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
@@ -6912,7 +8752,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-05-14</t>
+          <t>2026-05-15</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -6921,19 +8761,19 @@
         </is>
       </c>
       <c r="C3">
-        <v>28510</v>
+        <v>29015</v>
       </c>
       <c r="D3">
-        <v>29940</v>
+        <v>29020</v>
       </c>
       <c r="E3">
-        <v>28360</v>
+        <v>27310</v>
       </c>
       <c r="F3">
-        <v>28615</v>
+        <v>27535</v>
       </c>
       <c r="G3">
-        <v>9547900</v>
+        <v>3301600</v>
       </c>
       <c r="H3" t="inlineStr">
         <is>
@@ -6942,7 +8782,7 @@
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>2026/05/14 21:24:24</t>
+          <t>2026/05/15 10:55:11</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
@@ -6954,7 +8794,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2026-05-14</t>
+          <t>2026-05-15</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -6963,19 +8803,19 @@
         </is>
       </c>
       <c r="C4">
-        <v>7850</v>
+        <v>7946</v>
       </c>
       <c r="D4">
-        <v>8096</v>
+        <v>8063</v>
       </c>
       <c r="E4">
-        <v>7777</v>
+        <v>7925</v>
       </c>
       <c r="F4">
-        <v>8096</v>
+        <v>8014</v>
       </c>
       <c r="G4">
-        <v>2811500</v>
+        <v>572900</v>
       </c>
       <c r="H4" t="inlineStr">
         <is>
@@ -6984,7 +8824,7 @@
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>2026/05/14 21:24:24</t>
+          <t>2026/05/15 10:55:11</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
@@ -6996,7 +8836,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-05-14</t>
+          <t>2026-05-15</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -7005,19 +8845,19 @@
         </is>
       </c>
       <c r="C5">
-        <v>2920.5</v>
+        <v>2910.5</v>
       </c>
       <c r="D5">
-        <v>2923.5</v>
+        <v>2951.5</v>
       </c>
       <c r="E5">
-        <v>2875</v>
+        <v>2905</v>
       </c>
       <c r="F5">
-        <v>2877</v>
+        <v>2927.5</v>
       </c>
       <c r="G5">
-        <v>34334700</v>
+        <v>20658700</v>
       </c>
       <c r="H5" t="inlineStr">
         <is>
@@ -7026,7 +8866,7 @@
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>2026/05/14 21:24:24</t>
+          <t>2026/05/15 10:55:11</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
@@ -7038,7 +8878,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2026-05-14</t>
+          <t>2026-05-15</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -7047,19 +8887,19 @@
         </is>
       </c>
       <c r="C6">
-        <v>5935</v>
+        <v>5879</v>
       </c>
       <c r="D6">
-        <v>5939</v>
+        <v>6012</v>
       </c>
       <c r="E6">
-        <v>5774</v>
+        <v>5816</v>
       </c>
       <c r="F6">
-        <v>5882</v>
+        <v>5859</v>
       </c>
       <c r="G6">
-        <v>9361000</v>
+        <v>3840700</v>
       </c>
       <c r="H6" t="inlineStr">
         <is>
@@ -7068,7 +8908,7 @@
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>2026/05/14 21:24:24</t>
+          <t>2026/05/15 10:55:11</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
@@ -7080,7 +8920,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026-05-14</t>
+          <t>2026-05-15</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -7089,19 +8929,19 @@
         </is>
       </c>
       <c r="C7">
-        <v>7050</v>
+        <v>6863</v>
       </c>
       <c r="D7">
-        <v>7100</v>
+        <v>7030</v>
       </c>
       <c r="E7">
-        <v>6851</v>
+        <v>6849</v>
       </c>
       <c r="F7">
-        <v>6864</v>
+        <v>6992</v>
       </c>
       <c r="G7">
-        <v>16036100</v>
+        <v>4267600</v>
       </c>
       <c r="H7" t="inlineStr">
         <is>
@@ -7110,7 +8950,7 @@
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>2026/05/14 21:24:24</t>
+          <t>2026/05/15 10:55:11</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
@@ -7122,7 +8962,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>2026-05-14</t>
+          <t>2026-05-15</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -7131,19 +8971,19 @@
         </is>
       </c>
       <c r="C8">
-        <v>2590.5</v>
+        <v>2640</v>
       </c>
       <c r="D8">
-        <v>2645.5</v>
+        <v>2653.5</v>
       </c>
       <c r="E8">
-        <v>2562</v>
+        <v>2603</v>
       </c>
       <c r="F8">
-        <v>2645.5</v>
+        <v>2653</v>
       </c>
       <c r="G8">
-        <v>11355800</v>
+        <v>2798000</v>
       </c>
       <c r="H8" t="inlineStr">
         <is>
@@ -7152,7 +8992,7 @@
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>2026/05/14 21:24:24</t>
+          <t>2026/05/15 10:55:11</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
@@ -7164,7 +9004,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2026-05-14</t>
+          <t>2026-05-15</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -7173,19 +9013,19 @@
         </is>
       </c>
       <c r="C9">
-        <v>5587</v>
+        <v>5542</v>
       </c>
       <c r="D9">
-        <v>5716</v>
+        <v>5580</v>
       </c>
       <c r="E9">
-        <v>5521</v>
+        <v>5415</v>
       </c>
       <c r="F9">
-        <v>5542</v>
+        <v>5426</v>
       </c>
       <c r="G9">
-        <v>5720800</v>
+        <v>1145400</v>
       </c>
       <c r="H9" t="inlineStr">
         <is>
@@ -7194,7 +9034,7 @@
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>2026/05/14 21:24:24</t>
+          <t>2026/05/15 10:55:11</t>
         </is>
       </c>
       <c r="J9" t="inlineStr">
@@ -7275,17 +9115,17 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>2026-05-14</t>
+          <t>2026-05-15</t>
         </is>
       </c>
       <c r="D2">
-        <v>62654.05</v>
+        <v>62317.7</v>
       </c>
       <c r="E2">
-        <v>-0.29</v>
+        <v>-0.63</v>
       </c>
       <c r="F2">
-        <v>10.07</v>
+        <v>10.29</v>
       </c>
       <c r="G2" t="inlineStr">
         <is>
@@ -7294,7 +9134,7 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>2026/05/14 21:24:24</t>
+          <t>2026/05/15 10:55:11</t>
         </is>
       </c>
     </row>
@@ -7311,17 +9151,17 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>2026-05-14</t>
+          <t>2026-05-15</t>
         </is>
       </c>
       <c r="D3">
-        <v>411.2</v>
+        <v>412.5</v>
       </c>
       <c r="E3">
-        <v>0.98</v>
+        <v>1.63</v>
       </c>
       <c r="F3">
-        <v>3.71</v>
+        <v>4.48</v>
       </c>
       <c r="G3" t="inlineStr">
         <is>
@@ -7330,7 +9170,7 @@
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>2026/05/14 21:24:24</t>
+          <t>2026/05/15 10:55:11</t>
         </is>
       </c>
     </row>
@@ -7347,17 +9187,17 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>2026-05-13</t>
+          <t>2026-05-14</t>
         </is>
       </c>
       <c r="D4">
-        <v>7444.25</v>
+        <v>7501.24</v>
       </c>
       <c r="E4">
-        <v>1.07</v>
+        <v>2.24</v>
       </c>
       <c r="F4">
-        <v>6</v>
+        <v>6.53</v>
       </c>
       <c r="G4" t="inlineStr">
         <is>
@@ -7366,7 +9206,7 @@
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>2026/05/14 21:24:24</t>
+          <t>2026/05/15 10:55:11</t>
         </is>
       </c>
     </row>
@@ -7383,17 +9223,17 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>2026-05-13</t>
+          <t>2026-05-14</t>
         </is>
       </c>
       <c r="D5">
-        <v>26402.34</v>
+        <v>26635.22</v>
       </c>
       <c r="E5">
-        <v>2.18</v>
+        <v>3.21</v>
       </c>
       <c r="F5">
-        <v>9.94</v>
+        <v>10.51</v>
       </c>
       <c r="G5" t="inlineStr">
         <is>
@@ -7402,7 +9242,7 @@
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>2026/05/14 21:24:24</t>
+          <t>2026/05/15 10:55:11</t>
         </is>
       </c>
     </row>
@@ -7419,17 +9259,17 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>2026-05-14</t>
+          <t>2026-05-15</t>
         </is>
       </c>
       <c r="D6">
-        <v>157.9</v>
+        <v>158.49</v>
       </c>
       <c r="E6">
-        <v>0.89</v>
+        <v>1.06</v>
       </c>
       <c r="F6">
-        <v>-0.57</v>
+        <v>-0.45</v>
       </c>
       <c r="G6" t="inlineStr">
         <is>
@@ -7438,7 +9278,7 @@
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>2026/05/14 21:24:24</t>
+          <t>2026/05/15 10:55:11</t>
         </is>
       </c>
     </row>
@@ -7455,17 +9295,17 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>2026-05-13</t>
+          <t>2026-05-14</t>
         </is>
       </c>
       <c r="D7">
-        <v>4.481</v>
+        <v>4.461</v>
       </c>
       <c r="E7">
-        <v>2.87</v>
+        <v>1.57</v>
       </c>
       <c r="F7">
-        <v>4.65</v>
+        <v>3.53</v>
       </c>
       <c r="G7" t="inlineStr">
         <is>
@@ -7474,7 +9314,7 @@
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>2026/05/14 21:24:24</t>
+          <t>2026/05/15 10:55:11</t>
         </is>
       </c>
     </row>
@@ -7495,13 +9335,13 @@
         </is>
       </c>
       <c r="D8">
-        <v>17.84</v>
+        <v>17.26</v>
       </c>
       <c r="E8">
-        <v>4.45</v>
+        <v>1.05</v>
       </c>
       <c r="F8">
-        <v>-0.56</v>
+        <v>-3.79</v>
       </c>
       <c r="G8" t="inlineStr">
         <is>
@@ -7510,7 +9350,7 @@
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>2026/05/14 21:24:24</t>
+          <t>2026/05/15 10:55:11</t>
         </is>
       </c>
     </row>
@@ -7527,17 +9367,17 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>2026-05-14</t>
+          <t>2026-05-15</t>
         </is>
       </c>
       <c r="D9">
-        <v>98.55</v>
+        <v>99.04</v>
       </c>
       <c r="E9">
-        <v>0.3</v>
+        <v>1.23</v>
       </c>
       <c r="F9">
-        <v>0.33</v>
+        <v>0.96</v>
       </c>
       <c r="G9" t="inlineStr">
         <is>
@@ -7546,7 +9386,7 @@
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>2026/05/14 21:24:24</t>
+          <t>2026/05/15 10:55:11</t>
         </is>
       </c>
     </row>
@@ -7630,7 +9470,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026/05/14 21:24:24</t>
+          <t>2026/05/15 10:55:11</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -7644,7 +9484,7 @@
         </is>
       </c>
       <c r="D2">
-        <v>11.38</v>
+        <v>11.18</v>
       </c>
       <c r="E2" t="inlineStr">
         <is>
@@ -7685,7 +9525,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026/05/14 21:24:24</t>
+          <t>2026/05/15 10:55:11</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -7694,10 +9534,10 @@
         </is>
       </c>
       <c r="C3">
-        <v>44.6</v>
+        <v>42.39</v>
       </c>
       <c r="D3">
-        <v>26.07</v>
+        <v>24.78</v>
       </c>
       <c r="E3" t="inlineStr">
         <is>
@@ -7738,7 +9578,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2026/05/14 21:24:24</t>
+          <t>2026/05/15 10:55:11</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -7752,7 +9592,7 @@
         </is>
       </c>
       <c r="D4">
-        <v>6.98</v>
+        <v>6.93</v>
       </c>
       <c r="E4" t="inlineStr">
         <is>
@@ -7793,7 +9633,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026/05/14 21:24:24</t>
+          <t>2026/05/15 10:55:11</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -7807,7 +9647,7 @@
         </is>
       </c>
       <c r="D5">
-        <v>1.53</v>
+        <v>1.55</v>
       </c>
       <c r="E5" t="inlineStr">
         <is>
@@ -7848,7 +9688,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2026/05/14 21:24:24</t>
+          <t>2026/05/15 10:55:11</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -7857,10 +9697,10 @@
         </is>
       </c>
       <c r="C6">
-        <v>19.58</v>
+        <v>19.44</v>
       </c>
       <c r="D6">
-        <v>2.28</v>
+        <v>2.27</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
@@ -7901,7 +9741,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026/05/14 21:24:24</t>
+          <t>2026/05/15 10:55:11</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -7910,10 +9750,10 @@
         </is>
       </c>
       <c r="C7">
-        <v>25.53</v>
+        <v>26.11</v>
       </c>
       <c r="D7">
-        <v>2.68</v>
+        <v>2.74</v>
       </c>
       <c r="E7" t="inlineStr">
         <is>
@@ -7954,7 +9794,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>2026/05/14 21:24:24</t>
+          <t>2026/05/15 10:55:11</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -7968,7 +9808,7 @@
         </is>
       </c>
       <c r="D8">
-        <v>1.98</v>
+        <v>1.99</v>
       </c>
       <c r="E8" t="inlineStr">
         <is>
@@ -8009,7 +9849,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2026/05/14 21:24:24</t>
+          <t>2026/05/15 10:55:11</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -8018,10 +9858,10 @@
         </is>
       </c>
       <c r="C9">
-        <v>44.27</v>
+        <v>43.07</v>
       </c>
       <c r="D9">
-        <v>6.89</v>
+        <v>6.7</v>
       </c>
       <c r="E9" t="inlineStr">
         <is>
@@ -8395,7 +10235,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-05-14</t>
+          <t>2026-05-15</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -8404,37 +10244,37 @@
         </is>
       </c>
       <c r="C2">
-        <v>51200</v>
+        <v>51030</v>
       </c>
       <c r="D2">
-        <v>45873.6</v>
+        <v>46380</v>
       </c>
       <c r="E2">
-        <v>42674</v>
+        <v>42804.93</v>
       </c>
       <c r="F2">
-        <v>34139.57</v>
+        <v>34257.68</v>
       </c>
       <c r="G2">
-        <v>-1.01</v>
+        <v>-2.71</v>
       </c>
       <c r="H2">
-        <v>16.26</v>
+        <v>20.18</v>
       </c>
       <c r="I2">
-        <v>23.37</v>
+        <v>23.56</v>
       </c>
       <c r="J2">
-        <v>0.61</v>
+        <v>0.31</v>
       </c>
       <c r="K2">
-        <v>92.15</v>
+        <v>91.65</v>
       </c>
       <c r="L2">
         <v>-5.75</v>
       </c>
       <c r="M2">
-        <v>3.3</v>
+        <v>3.28</v>
       </c>
       <c r="N2" t="inlineStr">
         <is>
@@ -8445,7 +10285,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-05-14</t>
+          <t>2026-05-15</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -8454,37 +10294,37 @@
         </is>
       </c>
       <c r="C3">
-        <v>28615</v>
+        <v>27535</v>
       </c>
       <c r="D3">
-        <v>27438.2</v>
+        <v>27662.4</v>
       </c>
       <c r="E3">
-        <v>25608.73</v>
+        <v>25685.6</v>
       </c>
       <c r="F3">
-        <v>19856.25</v>
+        <v>19935.33</v>
       </c>
       <c r="G3">
-        <v>-3.7</v>
+        <v>-7.86</v>
       </c>
       <c r="H3">
-        <v>14.51</v>
+        <v>10.67</v>
       </c>
       <c r="I3">
-        <v>3.4</v>
+        <v>2.7</v>
       </c>
       <c r="J3">
-        <v>0.9</v>
+        <v>0.31</v>
       </c>
       <c r="K3">
-        <v>85.24</v>
+        <v>81.03</v>
       </c>
       <c r="L3">
-        <v>-11.7</v>
+        <v>-12.59</v>
       </c>
       <c r="M3">
-        <v>3.99</v>
+        <v>3.67</v>
       </c>
       <c r="N3" t="inlineStr">
         <is>
@@ -8495,7 +10335,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2026-05-14</t>
+          <t>2026-05-15</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -8504,37 +10344,37 @@
         </is>
       </c>
       <c r="C4">
-        <v>8096</v>
+        <v>8014</v>
       </c>
       <c r="D4">
-        <v>8403.88</v>
+        <v>8369.84</v>
       </c>
       <c r="E4">
-        <v>8880.21</v>
+        <v>8876.2</v>
       </c>
       <c r="F4">
-        <v>7934.89</v>
+        <v>7940.72</v>
       </c>
       <c r="G4">
-        <v>0.01</v>
+        <v>1.44</v>
       </c>
       <c r="H4">
-        <v>-6.67</v>
+        <v>-6.65</v>
       </c>
       <c r="I4">
-        <v>-10.26</v>
+        <v>-12.89</v>
       </c>
       <c r="J4">
-        <v>0.75</v>
+        <v>0.15</v>
       </c>
       <c r="K4">
-        <v>45.27</v>
+        <v>43.55</v>
       </c>
       <c r="L4">
         <v>-16.59</v>
       </c>
       <c r="M4">
-        <v>4.49</v>
+        <v>4.5</v>
       </c>
       <c r="N4" t="inlineStr">
         <is>
@@ -8545,7 +10385,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-05-14</t>
+          <t>2026-05-15</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -8554,37 +10394,37 @@
         </is>
       </c>
       <c r="C5">
-        <v>2877</v>
+        <v>2927.5</v>
       </c>
       <c r="D5">
-        <v>2844.34</v>
+        <v>2849.76</v>
       </c>
       <c r="E5">
-        <v>2812.37</v>
+        <v>2813.65</v>
       </c>
       <c r="F5">
-        <v>2522.66</v>
+        <v>2527.3</v>
       </c>
       <c r="G5">
-        <v>0.49</v>
+        <v>4.31</v>
       </c>
       <c r="H5">
-        <v>1.23</v>
+        <v>2.36</v>
       </c>
       <c r="I5">
-        <v>-5.17</v>
+        <v>-5.11</v>
       </c>
       <c r="J5">
-        <v>0.96</v>
+        <v>0.58</v>
       </c>
       <c r="K5">
-        <v>82.05</v>
+        <v>86.37</v>
       </c>
       <c r="L5">
         <v>-6.6</v>
       </c>
       <c r="M5">
-        <v>1.67</v>
+        <v>1.71</v>
       </c>
       <c r="N5" t="inlineStr">
         <is>
@@ -8595,7 +10435,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2026-05-14</t>
+          <t>2026-05-15</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -8604,37 +10444,37 @@
         </is>
       </c>
       <c r="C6">
-        <v>5882</v>
+        <v>5859</v>
       </c>
       <c r="D6">
-        <v>5192</v>
+        <v>5210.16</v>
       </c>
       <c r="E6">
-        <v>5037.77</v>
+        <v>5061.95</v>
       </c>
       <c r="F6">
-        <v>4075.95</v>
+        <v>4090.93</v>
       </c>
       <c r="G6">
-        <v>8.97</v>
+        <v>11.62</v>
       </c>
       <c r="H6">
-        <v>10.83</v>
+        <v>11.07</v>
       </c>
       <c r="I6">
-        <v>14.5</v>
+        <v>13.46</v>
       </c>
       <c r="J6">
-        <v>0.71</v>
+        <v>0.29</v>
       </c>
       <c r="K6">
-        <v>98.2</v>
+        <v>95.29</v>
       </c>
       <c r="L6">
-        <v>-10.03</v>
+        <v>-8.61</v>
       </c>
       <c r="M6">
-        <v>2.92</v>
+        <v>2.88</v>
       </c>
       <c r="N6" t="inlineStr">
         <is>
@@ -8645,7 +10485,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026-05-14</t>
+          <t>2026-05-15</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -8654,37 +10494,37 @@
         </is>
       </c>
       <c r="C7">
-        <v>6864</v>
+        <v>6992</v>
       </c>
       <c r="D7">
-        <v>8030.04</v>
+        <v>7955.76</v>
       </c>
       <c r="E7">
-        <v>8814.31</v>
+        <v>8771.8</v>
       </c>
       <c r="F7">
-        <v>11235.42</v>
+        <v>11207.75</v>
       </c>
       <c r="G7">
-        <v>-7.29</v>
+        <v>-8.8</v>
       </c>
       <c r="H7">
-        <v>-17.3</v>
+        <v>-15.73</v>
       </c>
       <c r="I7">
-        <v>-23.14</v>
+        <v>-19.07</v>
       </c>
       <c r="J7">
-        <v>1.36</v>
+        <v>0.36</v>
       </c>
       <c r="K7">
-        <v>0.16</v>
+        <v>1.8</v>
       </c>
       <c r="L7">
         <v>-20.33</v>
       </c>
       <c r="M7">
-        <v>2.7</v>
+        <v>2.77</v>
       </c>
       <c r="N7" t="inlineStr">
         <is>
@@ -8695,7 +10535,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>2026-05-14</t>
+          <t>2026-05-15</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -8704,31 +10544,31 @@
         </is>
       </c>
       <c r="C8">
-        <v>2645.5</v>
+        <v>2653</v>
       </c>
       <c r="D8">
-        <v>2604.04</v>
+        <v>2599.62</v>
       </c>
       <c r="E8">
-        <v>2647.67</v>
+        <v>2647.45</v>
       </c>
       <c r="F8">
-        <v>2593.13</v>
+        <v>2594.29</v>
       </c>
       <c r="G8">
-        <v>4.77</v>
+        <v>4.92</v>
       </c>
       <c r="H8">
-        <v>2.46</v>
+        <v>1.26</v>
       </c>
       <c r="I8">
-        <v>2.54</v>
+        <v>-0.32</v>
       </c>
       <c r="J8">
-        <v>1.2</v>
+        <v>0.31</v>
       </c>
       <c r="K8">
-        <v>65.06</v>
+        <v>66.51</v>
       </c>
       <c r="L8">
         <v>-4.4</v>
@@ -8745,7 +10585,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2026-05-14</t>
+          <t>2026-05-15</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -8754,37 +10594,37 @@
         </is>
       </c>
       <c r="C9">
-        <v>5542</v>
+        <v>5426</v>
       </c>
       <c r="D9">
-        <v>4854.44</v>
+        <v>4885.2</v>
       </c>
       <c r="E9">
-        <v>4477.05</v>
+        <v>4500.57</v>
       </c>
       <c r="F9">
-        <v>4107.9</v>
+        <v>4115.51</v>
       </c>
       <c r="G9">
-        <v>11.78</v>
+        <v>7.87</v>
       </c>
       <c r="H9">
-        <v>19.13</v>
+        <v>17.78</v>
       </c>
       <c r="I9">
-        <v>28.73</v>
+        <v>24.56</v>
       </c>
       <c r="J9">
-        <v>1.21</v>
+        <v>0.24</v>
       </c>
       <c r="K9">
-        <v>92.12</v>
+        <v>87.46</v>
       </c>
       <c r="L9">
         <v>-4.09</v>
       </c>
       <c r="M9">
-        <v>2.99</v>
+        <v>3.06</v>
       </c>
       <c r="N9" t="inlineStr">
         <is>
@@ -8884,7 +10724,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026/05/14 21:24:24</t>
+          <t>2026/05/15 10:55:11</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -8923,7 +10763,7 @@
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>終値51200 / 20日騰落16.26% / 出来高倍率0.61 / PER未取得 / PBR11.38 / EPS未取得</t>
+          <t>終値51030 / 20日騰落20.18% / 出来高倍率0.31 / PER未取得 / PBR11.18 / EPS未取得</t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
@@ -8935,7 +10775,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026/05/14 21:24:24</t>
+          <t>2026/05/15 10:55:11</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -8944,13 +10784,13 @@
         </is>
       </c>
       <c r="C3">
-        <v>20</v>
+        <v>14</v>
       </c>
       <c r="D3">
         <v>11</v>
       </c>
       <c r="E3">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="F3">
         <v>2</v>
@@ -8965,7 +10805,7 @@
         <v>3</v>
       </c>
       <c r="J3">
-        <v>69</v>
+        <v>60</v>
       </c>
       <c r="K3" t="inlineStr">
         <is>
@@ -8974,7 +10814,7 @@
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>終値28615 / 20日騰落14.51% / 出来高倍率0.9 / PER44.6 / PBR26.07 / EPS641.61</t>
+          <t>終値27535 / 20日騰落10.67% / 出来高倍率0.31 / PER42.39 / PBR24.78 / EPS641.61</t>
         </is>
       </c>
       <c r="M3" t="inlineStr">
@@ -8986,7 +10826,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2026/05/14 21:24:24</t>
+          <t>2026/05/15 10:55:11</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -9025,7 +10865,7 @@
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>終値8096 / 20日騰落-6.67% / 出来高倍率0.75 / PER未取得 / PBR6.98 / EPS未取得</t>
+          <t>終値8014 / 20日騰落-6.65% / 出来高倍率0.15 / PER未取得 / PBR6.93 / EPS未取得</t>
         </is>
       </c>
       <c r="M4" t="inlineStr">
@@ -9037,7 +10877,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026/05/14 21:24:24</t>
+          <t>2026/05/15 10:55:11</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -9052,7 +10892,7 @@
         <v>9</v>
       </c>
       <c r="E5">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="F5">
         <v>5</v>
@@ -9067,7 +10907,7 @@
         <v>10</v>
       </c>
       <c r="J5">
-        <v>68</v>
+        <v>65</v>
       </c>
       <c r="K5" t="inlineStr">
         <is>
@@ -9076,7 +10916,7 @@
       </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t>終値2877 / 20日騰落1.23% / 出来高倍率0.96 / PER未取得 / PBR1.53 / EPS未取得</t>
+          <t>終値2927.5 / 20日騰落2.36% / 出来高倍率0.58 / PER未取得 / PBR1.55 / EPS未取得</t>
         </is>
       </c>
       <c r="M5" t="inlineStr">
@@ -9088,7 +10928,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2026/05/14 21:24:24</t>
+          <t>2026/05/15 10:55:11</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -9115,10 +10955,10 @@
         <v>12</v>
       </c>
       <c r="I6">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="J6">
-        <v>80</v>
+        <v>84</v>
       </c>
       <c r="K6" t="inlineStr">
         <is>
@@ -9127,7 +10967,7 @@
       </c>
       <c r="L6" t="inlineStr">
         <is>
-          <t>終値5882 / 20日騰落10.83% / 出来高倍率0.71 / PER19.58 / PBR2.28 / EPS300.42</t>
+          <t>終値5859 / 20日騰落11.07% / 出来高倍率0.29 / PER19.44 / PBR2.27 / EPS300.42</t>
         </is>
       </c>
       <c r="M6" t="inlineStr">
@@ -9139,7 +10979,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026/05/14 21:24:24</t>
+          <t>2026/05/15 10:55:11</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -9154,7 +10994,7 @@
         <v>0</v>
       </c>
       <c r="E7">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="F7">
         <v>6</v>
@@ -9169,7 +11009,7 @@
         <v>3</v>
       </c>
       <c r="J7">
-        <v>44</v>
+        <v>39</v>
       </c>
       <c r="K7" t="inlineStr">
         <is>
@@ -9178,7 +11018,7 @@
       </c>
       <c r="L7" t="inlineStr">
         <is>
-          <t>終値6864 / 20日騰落-17.3% / 出来高倍率1.36 / PER25.53 / PBR2.68 / EPS268.9</t>
+          <t>終値6992 / 20日騰落-15.73% / 出来高倍率0.36 / PER26.11 / PBR2.74 / EPS268.9</t>
         </is>
       </c>
       <c r="M7" t="inlineStr">
@@ -9190,7 +11030,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>2026/05/14 21:24:24</t>
+          <t>2026/05/15 10:55:11</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -9199,13 +11039,13 @@
         </is>
       </c>
       <c r="C8">
-        <v>13</v>
+        <v>20</v>
       </c>
       <c r="D8">
-        <v>15</v>
+        <v>9</v>
       </c>
       <c r="E8">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="F8">
         <v>5</v>
@@ -9220,7 +11060,7 @@
         <v>10</v>
       </c>
       <c r="J8">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="K8" t="inlineStr">
         <is>
@@ -9229,7 +11069,7 @@
       </c>
       <c r="L8" t="inlineStr">
         <is>
-          <t>終値2645.5 / 20日騰落2.46% / 出来高倍率1.2 / PER未取得 / PBR1.98 / EPS未取得</t>
+          <t>終値2653 / 20日騰落1.26% / 出来高倍率0.31 / PER未取得 / PBR1.99 / EPS未取得</t>
         </is>
       </c>
       <c r="M8" t="inlineStr">
@@ -9241,7 +11081,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2026/05/14 21:24:24</t>
+          <t>2026/05/15 10:55:11</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -9256,7 +11096,7 @@
         <v>12</v>
       </c>
       <c r="E9">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="F9">
         <v>2</v>
@@ -9271,7 +11111,7 @@
         <v>10</v>
       </c>
       <c r="J9">
-        <v>79</v>
+        <v>74</v>
       </c>
       <c r="K9" t="inlineStr">
         <is>
@@ -9280,7 +11120,7 @@
       </c>
       <c r="L9" t="inlineStr">
         <is>
-          <t>終値5542 / 20日騰落19.13% / 出来高倍率1.21 / PER44.27 / PBR6.89 / EPS125.2</t>
+          <t>終値5426 / 20日騰落17.78% / 出来高倍率0.24 / PER43.07 / PBR6.7 / EPS125.2</t>
         </is>
       </c>
       <c r="M9" t="inlineStr">
@@ -9363,7 +11203,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026/05/14 21:24:24</t>
+          <t>2026/05/15 10:55:11</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">

</xml_diff>